<commit_message>
Actualizar resultados de Finalizacion 2026-II hasta el 20/09/2026
- Carga 24 partidos jugados entre el 10 y el 20 de septiembre
  (fechas 5, 7, 9, 10, 11 y 13 -- varios aplazados fuera de su
  jornada nominal) con actualizar_resultados.py.
- Tabla.csv/Partidos.csv/Historial_partidos.csv actualizados;
  historial pasa de 725 a 749 partidos. Tabla verificada contra
  Dimayor en vivo.
- model_params.csv: recalibrado el DrawBias (exacto, 221/749).
  HomeAdvantage/RatingScale/K_elo se dejan igual porque la busqueda
  en grilla dio un optimo en una zona plana, estadisticamente
  indistinguible del valor anterior.
- Corrige un error de sintaxis en model_params.csv (un ';' dentro
  del texto de Origen rompia el CSV de 3 columnas).
- Resultados.xlsx/Resultado.png regenerados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resultados.xlsx
+++ b/Resultados.xlsx
@@ -430,64 +430,64 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Millonarios</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Atlético Nacional</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Deportes Tolima</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>Independiente Medellín</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Atlético Nacional</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Millonarios</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Deportivo Cali</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>Llaneros</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Once Caldas</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>Águilas Doradas</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Atlético Bucaramanga</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Once Caldas</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Internacional de Bogotá</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
         <is>
           <t>Cúcuta Deportivo</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Deportivo Cali</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Internacional de Bogotá</t>
-        </is>
-      </c>
       <c r="O1" t="inlineStr">
         <is>
           <t>Fortaleza</t>
@@ -495,32 +495,32 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>Deportivo Pasto</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Alianza Valledupar</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Boyacá Chicó</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Jaguares</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>Deportivo Pereira</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Jaguares</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Boyacá Chicó</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Junior</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Deportivo Pasto</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Alianza Valledupar</t>
         </is>
       </c>
     </row>
@@ -529,64 +529,64 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>40.038</v>
+        <v>23.954</v>
       </c>
       <c r="C2" t="n">
-        <v>8.951000000000001</v>
+        <v>0.762</v>
       </c>
       <c r="D2" t="n">
-        <v>7.038</v>
+        <v>61.654</v>
       </c>
       <c r="E2" t="n">
-        <v>41.891</v>
+        <v>4.488</v>
       </c>
       <c r="F2" t="n">
-        <v>0.177</v>
+        <v>1.565</v>
       </c>
       <c r="G2" t="n">
-        <v>0.016</v>
+        <v>3.44</v>
       </c>
       <c r="H2" t="n">
-        <v>0.395</v>
+        <v>3.568000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>0.101</v>
+        <v>0.494</v>
       </c>
       <c r="J2" t="n">
-        <v>1.212</v>
+        <v>0.032</v>
       </c>
       <c r="K2" t="n">
-        <v>0.137</v>
+        <v>0.014</v>
       </c>
       <c r="L2" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
         <v>0.001</v>
       </c>
-      <c r="M2" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.011</v>
-      </c>
       <c r="T2" t="n">
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="3">
@@ -594,64 +594,64 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>32.811</v>
+        <v>36.69</v>
       </c>
       <c r="C3" t="n">
-        <v>16.114</v>
+        <v>3.398</v>
       </c>
       <c r="D3" t="n">
-        <v>13.319</v>
+        <v>22.111</v>
       </c>
       <c r="E3" t="n">
-        <v>30.001</v>
+        <v>10.869</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9520000000000001</v>
+        <v>5.353</v>
       </c>
       <c r="G3" t="n">
-        <v>0.067</v>
+        <v>9.533999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>1.821</v>
+        <v>9.071</v>
       </c>
       <c r="I3" t="n">
-        <v>0.467</v>
+        <v>2.406</v>
       </c>
       <c r="J3" t="n">
-        <v>3.46</v>
+        <v>0.237</v>
       </c>
       <c r="K3" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.096</v>
       </c>
       <c r="L3" t="n">
-        <v>0.015</v>
+        <v>0.163</v>
       </c>
       <c r="M3" t="n">
-        <v>0.191</v>
+        <v>0.003</v>
       </c>
       <c r="N3" t="n">
-        <v>0.02</v>
+        <v>0.001</v>
       </c>
       <c r="O3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
         <v>0.001</v>
       </c>
-      <c r="Q3" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
       <c r="S3" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.001</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
+        <v>0.066</v>
       </c>
     </row>
     <row r="4">
@@ -659,64 +659,64 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>15.486</v>
+        <v>17.856</v>
       </c>
       <c r="C4" t="n">
-        <v>24.882</v>
+        <v>7.82</v>
       </c>
       <c r="D4" t="n">
-        <v>22.029</v>
+        <v>8.433999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>14.675</v>
+        <v>16.27</v>
       </c>
       <c r="F4" t="n">
-        <v>3.213</v>
+        <v>11.187</v>
       </c>
       <c r="G4" t="n">
-        <v>0.364</v>
+        <v>16.777</v>
       </c>
       <c r="H4" t="n">
-        <v>5.592</v>
+        <v>14</v>
       </c>
       <c r="I4" t="n">
-        <v>1.659</v>
+        <v>5.597</v>
       </c>
       <c r="J4" t="n">
-        <v>8.039999999999999</v>
+        <v>0.701</v>
       </c>
       <c r="K4" t="n">
-        <v>2.505</v>
+        <v>0.479</v>
       </c>
       <c r="L4" t="n">
-        <v>0.112</v>
+        <v>0.522</v>
       </c>
       <c r="M4" t="n">
-        <v>0.774</v>
+        <v>0.023</v>
       </c>
       <c r="N4" t="n">
-        <v>0.161</v>
+        <v>0.002</v>
       </c>
       <c r="O4" t="n">
-        <v>0.011</v>
+        <v>0.001</v>
       </c>
       <c r="P4" t="n">
-        <v>0.014</v>
+        <v>0.002</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.016</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>0.008</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>0.458</v>
+        <v>0.01</v>
       </c>
       <c r="T4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="U4" t="n">
-        <v>0.001</v>
+        <v>0.318</v>
       </c>
     </row>
     <row r="5">
@@ -724,64 +724,64 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>7.207</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>20.844</v>
+        <v>11.294</v>
       </c>
       <c r="D5" t="n">
-        <v>21.08</v>
+        <v>4.043</v>
       </c>
       <c r="E5" t="n">
-        <v>7.487000000000001</v>
+        <v>16.336</v>
       </c>
       <c r="F5" t="n">
-        <v>6.5</v>
+        <v>14.433</v>
       </c>
       <c r="G5" t="n">
-        <v>1.098</v>
+        <v>16.321</v>
       </c>
       <c r="H5" t="n">
-        <v>9.890000000000001</v>
+        <v>14.895</v>
       </c>
       <c r="I5" t="n">
-        <v>3.41</v>
+        <v>8.266999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>12.726</v>
+        <v>1.612</v>
       </c>
       <c r="K5" t="n">
-        <v>5.435</v>
+        <v>1.2</v>
       </c>
       <c r="L5" t="n">
-        <v>0.402</v>
+        <v>1.168</v>
       </c>
       <c r="M5" t="n">
-        <v>1.881</v>
+        <v>0.103</v>
       </c>
       <c r="N5" t="n">
-        <v>0.555</v>
+        <v>0.011</v>
       </c>
       <c r="O5" t="n">
-        <v>0.045</v>
+        <v>0.001</v>
       </c>
       <c r="P5" t="n">
-        <v>0.033</v>
+        <v>0.005</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.077</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>0.023</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="S5" t="n">
-        <v>1.305</v>
+        <v>0.02</v>
       </c>
       <c r="T5" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="U5" t="n">
-        <v>0.002</v>
+        <v>0.741</v>
       </c>
     </row>
     <row r="6">
@@ -789,64 +789,64 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>2.754</v>
+        <v>5.647</v>
       </c>
       <c r="C6" t="n">
-        <v>12.249</v>
+        <v>14.11</v>
       </c>
       <c r="D6" t="n">
-        <v>13.628</v>
+        <v>1.99</v>
       </c>
       <c r="E6" t="n">
-        <v>3.159</v>
+        <v>14.783</v>
       </c>
       <c r="F6" t="n">
-        <v>10.815</v>
+        <v>15.177</v>
       </c>
       <c r="G6" t="n">
-        <v>2.627</v>
+        <v>14.729</v>
       </c>
       <c r="H6" t="n">
-        <v>13.914</v>
+        <v>14.151</v>
       </c>
       <c r="I6" t="n">
-        <v>6.191</v>
+        <v>10.491</v>
       </c>
       <c r="J6" t="n">
-        <v>15.86</v>
+        <v>2.775</v>
       </c>
       <c r="K6" t="n">
-        <v>9.1</v>
+        <v>2.27</v>
       </c>
       <c r="L6" t="n">
-        <v>1.127</v>
+        <v>1.987</v>
       </c>
       <c r="M6" t="n">
-        <v>4.004</v>
+        <v>0.261</v>
       </c>
       <c r="N6" t="n">
-        <v>1.312</v>
+        <v>0.057</v>
       </c>
       <c r="O6" t="n">
-        <v>0.119</v>
+        <v>0.014</v>
       </c>
       <c r="P6" t="n">
-        <v>0.145</v>
+        <v>0.029</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.189</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="R6" t="n">
-        <v>0.112</v>
+        <v>0.018</v>
       </c>
       <c r="S6" t="n">
-        <v>2.682</v>
+        <v>0.058</v>
       </c>
       <c r="T6" t="n">
-        <v>0.002</v>
+        <v>0.025</v>
       </c>
       <c r="U6" t="n">
-        <v>0.011</v>
+        <v>1.421</v>
       </c>
     </row>
     <row r="7">
@@ -854,64 +854,64 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>1.053</v>
+        <v>3.182</v>
       </c>
       <c r="C7" t="n">
-        <v>7.115</v>
+        <v>15.631</v>
       </c>
       <c r="D7" t="n">
-        <v>8.802999999999999</v>
+        <v>1.004</v>
       </c>
       <c r="E7" t="n">
-        <v>1.388</v>
+        <v>12.104</v>
       </c>
       <c r="F7" t="n">
-        <v>13.511</v>
+        <v>14.682</v>
       </c>
       <c r="G7" t="n">
-        <v>4.354</v>
+        <v>12.591</v>
       </c>
       <c r="H7" t="n">
-        <v>14.219</v>
+        <v>12.785</v>
       </c>
       <c r="I7" t="n">
-        <v>8.074</v>
+        <v>12.631</v>
       </c>
       <c r="J7" t="n">
-        <v>14.148</v>
+        <v>4.765</v>
       </c>
       <c r="K7" t="n">
-        <v>11.125</v>
+        <v>3.999</v>
       </c>
       <c r="L7" t="n">
-        <v>2.353</v>
+        <v>3.139</v>
       </c>
       <c r="M7" t="n">
-        <v>5.779999999999999</v>
+        <v>0.5640000000000001</v>
       </c>
       <c r="N7" t="n">
-        <v>2.464</v>
+        <v>0.136</v>
       </c>
       <c r="O7" t="n">
-        <v>0.333</v>
+        <v>0.023</v>
       </c>
       <c r="P7" t="n">
-        <v>0.269</v>
+        <v>0.057</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.436</v>
+        <v>0.015</v>
       </c>
       <c r="R7" t="n">
-        <v>0.267</v>
+        <v>0.05599999999999999</v>
       </c>
       <c r="S7" t="n">
-        <v>4.288</v>
+        <v>0.135</v>
       </c>
       <c r="T7" t="n">
-        <v>0.003</v>
+        <v>0.05599999999999999</v>
       </c>
       <c r="U7" t="n">
-        <v>0.017</v>
+        <v>2.445</v>
       </c>
     </row>
     <row r="8">
@@ -919,64 +919,64 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>0.398</v>
+        <v>1.726</v>
       </c>
       <c r="C8" t="n">
-        <v>4.288</v>
+        <v>15.348</v>
       </c>
       <c r="D8" t="n">
-        <v>5.546</v>
+        <v>0.469</v>
       </c>
       <c r="E8" t="n">
-        <v>0.705</v>
+        <v>9.727</v>
       </c>
       <c r="F8" t="n">
-        <v>13.718</v>
+        <v>12.828</v>
       </c>
       <c r="G8" t="n">
-        <v>6.039</v>
+        <v>10.001</v>
       </c>
       <c r="H8" t="n">
-        <v>13.087</v>
+        <v>10.789</v>
       </c>
       <c r="I8" t="n">
-        <v>9.92</v>
+        <v>13.888</v>
       </c>
       <c r="J8" t="n">
-        <v>11.529</v>
+        <v>7.298</v>
       </c>
       <c r="K8" t="n">
-        <v>11.872</v>
+        <v>6.521000000000001</v>
       </c>
       <c r="L8" t="n">
-        <v>3.414</v>
+        <v>4.804</v>
       </c>
       <c r="M8" t="n">
-        <v>7.288</v>
+        <v>1.316</v>
       </c>
       <c r="N8" t="n">
-        <v>3.638</v>
+        <v>0.363</v>
       </c>
       <c r="O8" t="n">
-        <v>0.604</v>
+        <v>0.065</v>
       </c>
       <c r="P8" t="n">
-        <v>0.59</v>
+        <v>0.141</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.791</v>
+        <v>0.06899999999999999</v>
       </c>
       <c r="R8" t="n">
-        <v>0.5599999999999999</v>
+        <v>0.131</v>
       </c>
       <c r="S8" t="n">
-        <v>5.965</v>
+        <v>0.307</v>
       </c>
       <c r="T8" t="n">
-        <v>0.011</v>
+        <v>0.154</v>
       </c>
       <c r="U8" t="n">
-        <v>0.037</v>
+        <v>4.055000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -984,64 +984,64 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.149</v>
+        <v>0.8880000000000001</v>
       </c>
       <c r="C9" t="n">
-        <v>2.54</v>
+        <v>13.087</v>
       </c>
       <c r="D9" t="n">
-        <v>3.514</v>
+        <v>0.176</v>
       </c>
       <c r="E9" t="n">
-        <v>0.347</v>
+        <v>6.577</v>
       </c>
       <c r="F9" t="n">
-        <v>12.611</v>
+        <v>10.385</v>
       </c>
       <c r="G9" t="n">
-        <v>7.817</v>
+        <v>7.239</v>
       </c>
       <c r="H9" t="n">
-        <v>11.018</v>
+        <v>8.332000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>10.663</v>
+        <v>14.081</v>
       </c>
       <c r="J9" t="n">
-        <v>9.364000000000001</v>
+        <v>10.221</v>
       </c>
       <c r="K9" t="n">
-        <v>11.817</v>
+        <v>9.811999999999999</v>
       </c>
       <c r="L9" t="n">
-        <v>4.873</v>
+        <v>7.385</v>
       </c>
       <c r="M9" t="n">
-        <v>8.656000000000001</v>
+        <v>2.573</v>
       </c>
       <c r="N9" t="n">
-        <v>4.977</v>
+        <v>0.859</v>
       </c>
       <c r="O9" t="n">
-        <v>1.057</v>
+        <v>0.177</v>
       </c>
       <c r="P9" t="n">
-        <v>0.988</v>
+        <v>0.333</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.326</v>
+        <v>0.173</v>
       </c>
       <c r="R9" t="n">
-        <v>0.877</v>
+        <v>0.312</v>
       </c>
       <c r="S9" t="n">
-        <v>7.303999999999999</v>
+        <v>0.599</v>
       </c>
       <c r="T9" t="n">
-        <v>0.019</v>
+        <v>0.38</v>
       </c>
       <c r="U9" t="n">
-        <v>0.083</v>
+        <v>6.411</v>
       </c>
     </row>
     <row r="10">
@@ -1049,64 +1049,64 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.06999999999999999</v>
+        <v>0.365</v>
       </c>
       <c r="C10" t="n">
-        <v>1.492</v>
+        <v>8.921999999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>2.255</v>
+        <v>0.091</v>
       </c>
       <c r="E10" t="n">
-        <v>0.181</v>
+        <v>4.273</v>
       </c>
       <c r="F10" t="n">
-        <v>10.708</v>
+        <v>6.682</v>
       </c>
       <c r="G10" t="n">
-        <v>9.401</v>
+        <v>4.43</v>
       </c>
       <c r="H10" t="n">
-        <v>8.755000000000001</v>
+        <v>5.462</v>
       </c>
       <c r="I10" t="n">
-        <v>10.822</v>
+        <v>11.674</v>
       </c>
       <c r="J10" t="n">
-        <v>7.282</v>
+        <v>13.626</v>
       </c>
       <c r="K10" t="n">
-        <v>10.923</v>
+        <v>13.512</v>
       </c>
       <c r="L10" t="n">
-        <v>6.500999999999999</v>
+        <v>10.351</v>
       </c>
       <c r="M10" t="n">
-        <v>9.649000000000001</v>
+        <v>4.821000000000001</v>
       </c>
       <c r="N10" t="n">
-        <v>6.511</v>
+        <v>1.868</v>
       </c>
       <c r="O10" t="n">
-        <v>1.756</v>
+        <v>0.439</v>
       </c>
       <c r="P10" t="n">
-        <v>1.527</v>
+        <v>0.8580000000000001</v>
       </c>
       <c r="Q10" t="n">
-        <v>2.006</v>
+        <v>0.455</v>
       </c>
       <c r="R10" t="n">
-        <v>1.435</v>
+        <v>0.784</v>
       </c>
       <c r="S10" t="n">
-        <v>8.494999999999999</v>
+        <v>1.166</v>
       </c>
       <c r="T10" t="n">
-        <v>0.061</v>
+        <v>0.7779999999999999</v>
       </c>
       <c r="U10" t="n">
-        <v>0.17</v>
+        <v>9.443</v>
       </c>
     </row>
     <row r="11">
@@ -1114,64 +1114,64 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.025</v>
+        <v>0.113</v>
       </c>
       <c r="C11" t="n">
-        <v>0.773</v>
+        <v>5.105</v>
       </c>
       <c r="D11" t="n">
-        <v>1.263</v>
+        <v>0.021</v>
       </c>
       <c r="E11" t="n">
-        <v>0.092</v>
+        <v>2.374</v>
       </c>
       <c r="F11" t="n">
-        <v>8.802999999999999</v>
+        <v>3.887</v>
       </c>
       <c r="G11" t="n">
-        <v>10.431</v>
+        <v>2.515</v>
       </c>
       <c r="H11" t="n">
-        <v>6.665999999999999</v>
+        <v>3.313</v>
       </c>
       <c r="I11" t="n">
-        <v>10.419</v>
+        <v>8.462</v>
       </c>
       <c r="J11" t="n">
-        <v>5.267</v>
+        <v>14.9</v>
       </c>
       <c r="K11" t="n">
-        <v>9.556000000000001</v>
+        <v>15.177</v>
       </c>
       <c r="L11" t="n">
-        <v>8.057</v>
+        <v>12.672</v>
       </c>
       <c r="M11" t="n">
-        <v>10.211</v>
+        <v>7.575</v>
       </c>
       <c r="N11" t="n">
-        <v>8.167</v>
+        <v>3.521</v>
       </c>
       <c r="O11" t="n">
-        <v>2.615</v>
+        <v>0.9039999999999999</v>
       </c>
       <c r="P11" t="n">
-        <v>2.431</v>
+        <v>1.782</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.027</v>
+        <v>0.9299999999999999</v>
       </c>
       <c r="R11" t="n">
-        <v>2.185</v>
+        <v>1.425</v>
       </c>
       <c r="S11" t="n">
-        <v>9.556000000000001</v>
+        <v>2.125</v>
       </c>
       <c r="T11" t="n">
-        <v>0.144</v>
+        <v>1.543</v>
       </c>
       <c r="U11" t="n">
-        <v>0.312</v>
+        <v>11.656</v>
       </c>
     </row>
     <row r="12">
@@ -1179,64 +1179,64 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>0.005</v>
+        <v>0.028</v>
       </c>
       <c r="C12" t="n">
-        <v>0.379</v>
+        <v>2.641</v>
       </c>
       <c r="D12" t="n">
-        <v>0.761</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>0.041</v>
+        <v>1.228</v>
       </c>
       <c r="F12" t="n">
-        <v>6.436999999999999</v>
+        <v>2.087</v>
       </c>
       <c r="G12" t="n">
-        <v>10.992</v>
+        <v>1.298</v>
       </c>
       <c r="H12" t="n">
-        <v>5.015</v>
+        <v>1.87</v>
       </c>
       <c r="I12" t="n">
-        <v>9.632</v>
+        <v>5.452</v>
       </c>
       <c r="J12" t="n">
-        <v>3.943</v>
+        <v>13.496</v>
       </c>
       <c r="K12" t="n">
-        <v>8.1</v>
+        <v>14.015</v>
       </c>
       <c r="L12" t="n">
-        <v>9.435</v>
+        <v>13.322</v>
       </c>
       <c r="M12" t="n">
-        <v>10.194</v>
+        <v>10.732</v>
       </c>
       <c r="N12" t="n">
-        <v>9.504999999999999</v>
+        <v>5.64</v>
       </c>
       <c r="O12" t="n">
-        <v>3.757</v>
+        <v>1.677</v>
       </c>
       <c r="P12" t="n">
-        <v>3.547</v>
+        <v>3.56</v>
       </c>
       <c r="Q12" t="n">
-        <v>4.257</v>
+        <v>1.791</v>
       </c>
       <c r="R12" t="n">
-        <v>3.14</v>
+        <v>2.493</v>
       </c>
       <c r="S12" t="n">
-        <v>9.997999999999999</v>
+        <v>3.422</v>
       </c>
       <c r="T12" t="n">
-        <v>0.296</v>
+        <v>2.686</v>
       </c>
       <c r="U12" t="n">
-        <v>0.5660000000000001</v>
+        <v>12.555</v>
       </c>
     </row>
     <row r="13">
@@ -1244,64 +1244,64 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>0.003</v>
+        <v>0.011</v>
       </c>
       <c r="C13" t="n">
-        <v>0.205</v>
+        <v>1.176</v>
       </c>
       <c r="D13" t="n">
-        <v>0.415</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0.016</v>
+        <v>0.5479999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>4.8</v>
+        <v>1.021</v>
       </c>
       <c r="G13" t="n">
-        <v>10.571</v>
+        <v>0.651</v>
       </c>
       <c r="H13" t="n">
-        <v>3.649</v>
+        <v>1.029</v>
       </c>
       <c r="I13" t="n">
-        <v>8.314</v>
+        <v>3.17</v>
       </c>
       <c r="J13" t="n">
-        <v>2.753</v>
+        <v>10.64</v>
       </c>
       <c r="K13" t="n">
-        <v>6.385000000000001</v>
+        <v>11.395</v>
       </c>
       <c r="L13" t="n">
-        <v>10.894</v>
+        <v>12.206</v>
       </c>
       <c r="M13" t="n">
-        <v>9.91</v>
+        <v>12.871</v>
       </c>
       <c r="N13" t="n">
-        <v>10.508</v>
+        <v>7.997999999999999</v>
       </c>
       <c r="O13" t="n">
-        <v>5.234</v>
+        <v>2.987</v>
       </c>
       <c r="P13" t="n">
-        <v>4.889</v>
+        <v>5.646</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.823</v>
+        <v>2.994</v>
       </c>
       <c r="R13" t="n">
-        <v>4.277</v>
+        <v>3.929</v>
       </c>
       <c r="S13" t="n">
-        <v>9.913</v>
+        <v>5.192</v>
       </c>
       <c r="T13" t="n">
-        <v>0.527</v>
+        <v>4.324999999999999</v>
       </c>
       <c r="U13" t="n">
-        <v>0.914</v>
+        <v>12.211</v>
       </c>
     </row>
     <row r="14">
@@ -1312,61 +1312,61 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0.101</v>
+        <v>0.47</v>
       </c>
       <c r="D14" t="n">
-        <v>0.195</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0.012</v>
+        <v>0.268</v>
       </c>
       <c r="F14" t="n">
-        <v>3.3</v>
+        <v>0.407</v>
       </c>
       <c r="G14" t="n">
-        <v>10.048</v>
+        <v>0.288</v>
       </c>
       <c r="H14" t="n">
-        <v>2.415</v>
+        <v>0.443</v>
       </c>
       <c r="I14" t="n">
-        <v>6.837</v>
+        <v>1.763</v>
       </c>
       <c r="J14" t="n">
-        <v>1.811</v>
+        <v>7.667</v>
       </c>
       <c r="K14" t="n">
-        <v>4.695</v>
+        <v>8.347999999999999</v>
       </c>
       <c r="L14" t="n">
-        <v>11.424</v>
+        <v>9.977</v>
       </c>
       <c r="M14" t="n">
-        <v>8.860999999999999</v>
+        <v>13.617</v>
       </c>
       <c r="N14" t="n">
-        <v>11.099</v>
+        <v>10.172</v>
       </c>
       <c r="O14" t="n">
-        <v>7.216</v>
+        <v>4.679</v>
       </c>
       <c r="P14" t="n">
-        <v>6.642</v>
+        <v>8.304</v>
       </c>
       <c r="Q14" t="n">
-        <v>7.622</v>
+        <v>4.464</v>
       </c>
       <c r="R14" t="n">
-        <v>5.759</v>
+        <v>5.622</v>
       </c>
       <c r="S14" t="n">
-        <v>9.353</v>
+        <v>7.231999999999999</v>
       </c>
       <c r="T14" t="n">
-        <v>1.054</v>
+        <v>6.088</v>
       </c>
       <c r="U14" t="n">
-        <v>1.556</v>
+        <v>10.191</v>
       </c>
     </row>
     <row r="15">
@@ -1374,64 +1374,64 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>0.044</v>
+        <v>0.171</v>
       </c>
       <c r="D15" t="n">
-        <v>0.104</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>0.004</v>
+        <v>0.106</v>
       </c>
       <c r="F15" t="n">
-        <v>2.041</v>
+        <v>0.164</v>
       </c>
       <c r="G15" t="n">
-        <v>8.794</v>
+        <v>0.112</v>
       </c>
       <c r="H15" t="n">
-        <v>1.621</v>
+        <v>0.167</v>
       </c>
       <c r="I15" t="n">
-        <v>5.165</v>
+        <v>0.868</v>
       </c>
       <c r="J15" t="n">
-        <v>1.129</v>
+        <v>5.082</v>
       </c>
       <c r="K15" t="n">
-        <v>3.247</v>
+        <v>5.443</v>
       </c>
       <c r="L15" t="n">
-        <v>11.039</v>
+        <v>7.693</v>
       </c>
       <c r="M15" t="n">
-        <v>7.396999999999999</v>
+        <v>12.372</v>
       </c>
       <c r="N15" t="n">
-        <v>10.932</v>
+        <v>11.796</v>
       </c>
       <c r="O15" t="n">
-        <v>9.556000000000001</v>
+        <v>6.666999999999999</v>
       </c>
       <c r="P15" t="n">
-        <v>8.530999999999999</v>
+        <v>10.435</v>
       </c>
       <c r="Q15" t="n">
-        <v>9.775</v>
+        <v>6.278</v>
       </c>
       <c r="R15" t="n">
-        <v>7.823</v>
+        <v>7.56</v>
       </c>
       <c r="S15" t="n">
-        <v>8.49</v>
+        <v>8.887</v>
       </c>
       <c r="T15" t="n">
-        <v>1.904</v>
+        <v>7.745</v>
       </c>
       <c r="U15" t="n">
-        <v>2.403</v>
+        <v>8.454000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -1442,61 +1442,61 @@
         <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>0.015</v>
+        <v>0.046</v>
       </c>
       <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
         <v>0.028</v>
       </c>
-      <c r="E16" t="n">
-        <v>0.001</v>
-      </c>
       <c r="F16" t="n">
-        <v>1.217</v>
+        <v>0.094</v>
       </c>
       <c r="G16" t="n">
-        <v>6.951000000000001</v>
+        <v>0.054</v>
       </c>
       <c r="H16" t="n">
-        <v>0.9769999999999999</v>
+        <v>0.08</v>
       </c>
       <c r="I16" t="n">
-        <v>3.601</v>
+        <v>0.421</v>
       </c>
       <c r="J16" t="n">
-        <v>0.746</v>
+        <v>3.224</v>
       </c>
       <c r="K16" t="n">
-        <v>2.13</v>
+        <v>3.528</v>
       </c>
       <c r="L16" t="n">
-        <v>9.98</v>
+        <v>5.448</v>
       </c>
       <c r="M16" t="n">
-        <v>5.774</v>
+        <v>10.106</v>
       </c>
       <c r="N16" t="n">
-        <v>9.536999999999999</v>
+        <v>12.22</v>
       </c>
       <c r="O16" t="n">
-        <v>11.801</v>
+        <v>8.803999999999998</v>
       </c>
       <c r="P16" t="n">
-        <v>10.991</v>
+        <v>12.18</v>
       </c>
       <c r="Q16" t="n">
-        <v>11.691</v>
+        <v>8.341999999999999</v>
       </c>
       <c r="R16" t="n">
-        <v>10.132</v>
+        <v>9.089</v>
       </c>
       <c r="S16" t="n">
-        <v>7.072000000000001</v>
+        <v>10.313</v>
       </c>
       <c r="T16" t="n">
-        <v>3.461</v>
+        <v>9.541</v>
       </c>
       <c r="U16" t="n">
-        <v>3.895</v>
+        <v>6.482</v>
       </c>
     </row>
     <row r="17">
@@ -1507,61 +1507,61 @@
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>0.003</v>
+        <v>0.015</v>
       </c>
       <c r="D17" t="n">
-        <v>0.016</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>0.014</v>
       </c>
       <c r="F17" t="n">
-        <v>0.721</v>
+        <v>0.032</v>
       </c>
       <c r="G17" t="n">
-        <v>4.918</v>
+        <v>0.014</v>
       </c>
       <c r="H17" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.032</v>
       </c>
       <c r="I17" t="n">
-        <v>2.403</v>
+        <v>0.216</v>
       </c>
       <c r="J17" t="n">
-        <v>0.397</v>
+        <v>1.937</v>
       </c>
       <c r="K17" t="n">
-        <v>1.241</v>
+        <v>2.101</v>
       </c>
       <c r="L17" t="n">
-        <v>8.074</v>
+        <v>3.817</v>
       </c>
       <c r="M17" t="n">
-        <v>4.141999999999999</v>
+        <v>8.079000000000001</v>
       </c>
       <c r="N17" t="n">
-        <v>7.869</v>
+        <v>11.689</v>
       </c>
       <c r="O17" t="n">
-        <v>13.755</v>
+        <v>10.962</v>
       </c>
       <c r="P17" t="n">
-        <v>12.971</v>
+        <v>12.678</v>
       </c>
       <c r="Q17" t="n">
-        <v>12.909</v>
+        <v>10.367</v>
       </c>
       <c r="R17" t="n">
-        <v>12.415</v>
+        <v>10.825</v>
       </c>
       <c r="S17" t="n">
-        <v>5.704</v>
+        <v>11.147</v>
       </c>
       <c r="T17" t="n">
-        <v>5.777</v>
+        <v>11.164</v>
       </c>
       <c r="U17" t="n">
-        <v>6.117999999999999</v>
+        <v>4.911</v>
       </c>
     </row>
     <row r="18">
@@ -1572,61 +1572,61 @@
         <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="D18" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="F18" t="n">
-        <v>0.325</v>
+        <v>0.008</v>
       </c>
       <c r="G18" t="n">
-        <v>3.089</v>
+        <v>0.003</v>
       </c>
       <c r="H18" t="n">
-        <v>0.265</v>
+        <v>0.008</v>
       </c>
       <c r="I18" t="n">
-        <v>1.342</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>0.226</v>
+        <v>1.032</v>
       </c>
       <c r="K18" t="n">
-        <v>0.655</v>
+        <v>1.195</v>
       </c>
       <c r="L18" t="n">
-        <v>6.007</v>
+        <v>2.547</v>
       </c>
       <c r="M18" t="n">
-        <v>2.772</v>
+        <v>6.104</v>
       </c>
       <c r="N18" t="n">
-        <v>5.959</v>
+        <v>10.863</v>
       </c>
       <c r="O18" t="n">
-        <v>14.568</v>
+        <v>13.079</v>
       </c>
       <c r="P18" t="n">
-        <v>14.514</v>
+        <v>12.42</v>
       </c>
       <c r="Q18" t="n">
-        <v>13.415</v>
+        <v>12.619</v>
       </c>
       <c r="R18" t="n">
-        <v>14.221</v>
+        <v>12.303</v>
       </c>
       <c r="S18" t="n">
-        <v>4.202999999999999</v>
+        <v>11.727</v>
       </c>
       <c r="T18" t="n">
-        <v>9.291</v>
+        <v>12.469</v>
       </c>
       <c r="U18" t="n">
-        <v>9.139999999999999</v>
+        <v>3.544</v>
       </c>
     </row>
     <row r="19">
@@ -1637,61 +1637,61 @@
         <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
         <v>0.002</v>
       </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
       <c r="F19" t="n">
-        <v>0.113</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>1.644</v>
+        <v>0.002</v>
       </c>
       <c r="H19" t="n">
-        <v>0.08800000000000001</v>
+        <v>0.005</v>
       </c>
       <c r="I19" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.037</v>
       </c>
       <c r="J19" t="n">
-        <v>0.08</v>
+        <v>0.503</v>
       </c>
       <c r="K19" t="n">
-        <v>0.298</v>
+        <v>0.5660000000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>3.954</v>
+        <v>1.536</v>
       </c>
       <c r="M19" t="n">
-        <v>1.611</v>
+        <v>4.465</v>
       </c>
       <c r="N19" t="n">
-        <v>3.984999999999999</v>
+        <v>9.585000000000001</v>
       </c>
       <c r="O19" t="n">
-        <v>13.479</v>
+        <v>15.06</v>
       </c>
       <c r="P19" t="n">
-        <v>14.737</v>
+        <v>11.647</v>
       </c>
       <c r="Q19" t="n">
-        <v>12.16</v>
+        <v>14.97</v>
       </c>
       <c r="R19" t="n">
-        <v>14.879</v>
+        <v>13.75</v>
       </c>
       <c r="S19" t="n">
-        <v>2.832</v>
+        <v>12.115</v>
       </c>
       <c r="T19" t="n">
-        <v>14.951</v>
+        <v>13.208</v>
       </c>
       <c r="U19" t="n">
-        <v>14.498</v>
+        <v>2.54</v>
       </c>
     </row>
     <row r="20">
@@ -1711,52 +1711,52 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0.034</v>
+        <v>0.001</v>
       </c>
       <c r="G20" t="n">
-        <v>0.643</v>
+        <v>0.001</v>
       </c>
       <c r="H20" t="n">
-        <v>0.037</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>0.238</v>
+        <v>0.008</v>
       </c>
       <c r="J20" t="n">
-        <v>0.026</v>
+        <v>0.207</v>
       </c>
       <c r="K20" t="n">
-        <v>0.076</v>
+        <v>0.27</v>
       </c>
       <c r="L20" t="n">
-        <v>1.868</v>
+        <v>0.876</v>
       </c>
       <c r="M20" t="n">
-        <v>0.705</v>
+        <v>2.855</v>
       </c>
       <c r="N20" t="n">
-        <v>2.182</v>
+        <v>7.704999999999999</v>
       </c>
       <c r="O20" t="n">
-        <v>9.587</v>
+        <v>16.721</v>
       </c>
       <c r="P20" t="n">
-        <v>11.508</v>
+        <v>10.803</v>
       </c>
       <c r="Q20" t="n">
-        <v>9.352</v>
+        <v>17.291</v>
       </c>
       <c r="R20" t="n">
-        <v>13.171</v>
+        <v>15.041</v>
       </c>
       <c r="S20" t="n">
-        <v>1.659</v>
+        <v>12.432</v>
       </c>
       <c r="T20" t="n">
-        <v>25.268</v>
+        <v>14.099</v>
       </c>
       <c r="U20" t="n">
-        <v>23.646</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="21">
@@ -1776,52 +1776,52 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>0.136</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0.009000000000000001</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0.054</v>
+        <v>0.002</v>
       </c>
       <c r="J21" t="n">
-        <v>0.001</v>
+        <v>0.045</v>
       </c>
       <c r="K21" t="n">
-        <v>0.02</v>
+        <v>0.059</v>
       </c>
       <c r="L21" t="n">
-        <v>0.47</v>
+        <v>0.364</v>
       </c>
       <c r="M21" t="n">
-        <v>0.169</v>
+        <v>1.56</v>
       </c>
       <c r="N21" t="n">
-        <v>0.618</v>
+        <v>5.514</v>
       </c>
       <c r="O21" t="n">
-        <v>4.505</v>
+        <v>17.74</v>
       </c>
       <c r="P21" t="n">
-        <v>5.672</v>
+        <v>9.120000000000001</v>
       </c>
       <c r="Q21" t="n">
-        <v>5.124</v>
+        <v>19.235</v>
       </c>
       <c r="R21" t="n">
-        <v>8.715999999999999</v>
+        <v>16.654</v>
       </c>
       <c r="S21" t="n">
-        <v>0.64</v>
+        <v>13.111</v>
       </c>
       <c r="T21" t="n">
-        <v>37.23099999999999</v>
+        <v>15.735</v>
       </c>
       <c r="U21" t="n">
-        <v>36.631</v>
+        <v>0.861</v>
       </c>
     </row>
   </sheetData>
@@ -1853,61 +1853,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>América de Cali</t>
+          <t>Atlético Nacional</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99.896</v>
+        <v>99.881</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Atlético Nacional</t>
+          <t>América de Cali</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.65300000000001</v>
+        <v>99.48299999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Atlético Bucaramanga</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>96.983</v>
+        <v>91.154</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Independiente Medellín</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>94.95699999999999</v>
+        <v>90.63200000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Atlético Bucaramanga</t>
+          <t>Independiente Medellín</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>76.339</v>
+        <v>87.59100000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Deportes Tolima</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>69.93600000000001</v>
+        <v>85.61000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -1917,47 +1917,47 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>61.497</v>
+        <v>81.45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Once Caldas</t>
+          <t>Deportivo Cali</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>52.674</v>
+        <v>67.855</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Águilas Doradas</t>
+          <t>Llaneros</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>40.485</v>
+        <v>27.641</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Deportivo Cali</t>
+          <t>Once Caldas</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>28.605</v>
+        <v>24.391</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Llaneros</t>
+          <t>Águilas Doradas</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>22.382</v>
+        <v>19.191</v>
       </c>
     </row>
     <row r="13">
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>22.085</v>
+        <v>15.462</v>
       </c>
     </row>
     <row r="14">
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>13.128</v>
+        <v>4.843</v>
       </c>
     </row>
     <row r="15">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12.297</v>
+        <v>1.429</v>
       </c>
     </row>
     <row r="16">
@@ -1997,27 +1997,27 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.839</v>
+        <v>1.131</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Deportivo Pereira</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2.171</v>
+        <v>0.619</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Deportivo Pereira</t>
+          <t>Deportivo Pasto</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2.04</v>
+        <v>0.5670000000000001</v>
       </c>
     </row>
     <row r="19">
@@ -2027,27 +2027,27 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1.847</v>
+        <v>0.525</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Alianza Valledupar</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.151</v>
+        <v>0.281</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Deportivo Pasto</t>
+          <t>Alianza Valledupar</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.035</v>
+        <v>0.264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar resultados de Finalizacion 2026-II hasta el 23/09/2026
- Carga 3 partidos jugados el 22 y 23 de septiembre (Independiente
  Medellin 2-1 Jaguares, Santa Fe 0-1 Deportivo Cali, America de
  Cali 1-0 Aguilas Doradas) con actualizar_resultados.py.
- Tabla.csv/Partidos.csv/Historial_partidos.csv actualizados;
  historial pasa de 749 a 752 partidos. Tabla verificada contra
  Dimayor en vivo.
- model_params.csv: DrawBias recalibrado exacto (221/752).
- Resultados.xlsx/Resultado.png regenerados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resultados.xlsx
+++ b/Resultados.xlsx
@@ -435,34 +435,34 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Independiente Medellín</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Atlético Nacional</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Deportivo Cali</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
         <is>
           <t>Atlético Bucaramanga</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Deportes Tolima</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Santa Fe</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Independiente Medellín</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Deportivo Cali</t>
-        </is>
-      </c>
       <c r="J1" t="inlineStr">
         <is>
           <t>Llaneros</t>
@@ -510,12 +510,12 @@
       </c>
       <c r="S1" t="inlineStr">
         <is>
+          <t>Deportivo Pereira</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>Jaguares</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Deportivo Pereira</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
@@ -529,37 +529,37 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>23.954</v>
+        <v>30.125</v>
       </c>
       <c r="C2" t="n">
-        <v>0.762</v>
+        <v>0.597</v>
       </c>
       <c r="D2" t="n">
-        <v>61.654</v>
+        <v>4.723</v>
       </c>
       <c r="E2" t="n">
-        <v>4.488</v>
+        <v>57.126</v>
       </c>
       <c r="F2" t="n">
-        <v>1.565</v>
+        <v>1.736</v>
       </c>
       <c r="G2" t="n">
-        <v>3.44</v>
+        <v>3.851</v>
       </c>
       <c r="H2" t="n">
-        <v>3.568000000000001</v>
+        <v>1.231</v>
       </c>
       <c r="I2" t="n">
-        <v>0.494</v>
+        <v>0.5740000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>0.032</v>
+        <v>0.017</v>
       </c>
       <c r="K2" t="n">
-        <v>0.014</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="L2" t="n">
-        <v>0.023</v>
+        <v>0.003</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -580,13 +580,13 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>0.005</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="3">
@@ -594,40 +594,40 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>36.69</v>
+        <v>38.68</v>
       </c>
       <c r="C3" t="n">
-        <v>3.398</v>
+        <v>2.52</v>
       </c>
       <c r="D3" t="n">
-        <v>22.111</v>
+        <v>10.741</v>
       </c>
       <c r="E3" t="n">
-        <v>10.869</v>
+        <v>25.4</v>
       </c>
       <c r="F3" t="n">
-        <v>5.353</v>
+        <v>6.265</v>
       </c>
       <c r="G3" t="n">
-        <v>9.533999999999999</v>
+        <v>9.218999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>9.071</v>
+        <v>4.378</v>
       </c>
       <c r="I3" t="n">
-        <v>2.406</v>
+        <v>2.478</v>
       </c>
       <c r="J3" t="n">
-        <v>0.237</v>
+        <v>0.145</v>
       </c>
       <c r="K3" t="n">
-        <v>0.096</v>
+        <v>0.075</v>
       </c>
       <c r="L3" t="n">
-        <v>0.163</v>
+        <v>0.045</v>
       </c>
       <c r="M3" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
         <v>0.001</v>
@@ -642,16 +642,16 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0.066</v>
+        <v>0.053</v>
       </c>
     </row>
     <row r="4">
@@ -659,64 +659,64 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>17.856</v>
+        <v>15.686</v>
       </c>
       <c r="C4" t="n">
-        <v>7.82</v>
+        <v>7.274999999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>8.433999999999999</v>
+        <v>18.112</v>
       </c>
       <c r="E4" t="n">
-        <v>16.27</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>11.187</v>
+        <v>13.647</v>
       </c>
       <c r="G4" t="n">
-        <v>16.777</v>
+        <v>16.696</v>
       </c>
       <c r="H4" t="n">
-        <v>14</v>
+        <v>10.925</v>
       </c>
       <c r="I4" t="n">
-        <v>5.597</v>
+        <v>7.044</v>
       </c>
       <c r="J4" t="n">
-        <v>0.701</v>
+        <v>0.65</v>
       </c>
       <c r="K4" t="n">
-        <v>0.479</v>
+        <v>0.412</v>
       </c>
       <c r="L4" t="n">
-        <v>0.522</v>
+        <v>0.229</v>
       </c>
       <c r="M4" t="n">
-        <v>0.023</v>
+        <v>0.022</v>
       </c>
       <c r="N4" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
         <v>0.001</v>
       </c>
-      <c r="P4" t="n">
-        <v>0.002</v>
-      </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="S4" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="T4" t="n">
         <v>0.001</v>
       </c>
       <c r="U4" t="n">
-        <v>0.318</v>
+        <v>0.253</v>
       </c>
     </row>
     <row r="5">
@@ -724,64 +724,64 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>9.539999999999999</v>
+        <v>7.922</v>
       </c>
       <c r="C5" t="n">
-        <v>11.294</v>
+        <v>10.7</v>
       </c>
       <c r="D5" t="n">
-        <v>4.043</v>
+        <v>16.931</v>
       </c>
       <c r="E5" t="n">
-        <v>16.336</v>
+        <v>4.225000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>14.433</v>
+        <v>15.958</v>
       </c>
       <c r="G5" t="n">
-        <v>16.321</v>
+        <v>16.553</v>
       </c>
       <c r="H5" t="n">
-        <v>14.895</v>
+        <v>13.785</v>
       </c>
       <c r="I5" t="n">
-        <v>8.266999999999999</v>
+        <v>10.005</v>
       </c>
       <c r="J5" t="n">
-        <v>1.612</v>
+        <v>1.476</v>
       </c>
       <c r="K5" t="n">
-        <v>1.2</v>
+        <v>1.133</v>
       </c>
       <c r="L5" t="n">
-        <v>1.168</v>
+        <v>0.542</v>
       </c>
       <c r="M5" t="n">
-        <v>0.103</v>
+        <v>0.09</v>
       </c>
       <c r="N5" t="n">
         <v>0.011</v>
       </c>
       <c r="O5" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
         <v>0.001</v>
       </c>
-      <c r="P5" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="T5" t="n">
         <v>0.006999999999999999</v>
       </c>
-      <c r="S5" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0.003</v>
-      </c>
       <c r="U5" t="n">
-        <v>0.741</v>
+        <v>0.649</v>
       </c>
     </row>
     <row r="6">
@@ -789,64 +789,64 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>5.647</v>
+        <v>4.112</v>
       </c>
       <c r="C6" t="n">
-        <v>14.11</v>
+        <v>13.711</v>
       </c>
       <c r="D6" t="n">
-        <v>1.99</v>
+        <v>14.42</v>
       </c>
       <c r="E6" t="n">
-        <v>14.783</v>
+        <v>2.2</v>
       </c>
       <c r="F6" t="n">
-        <v>15.177</v>
+        <v>15.822</v>
       </c>
       <c r="G6" t="n">
-        <v>14.729</v>
+        <v>15.021</v>
       </c>
       <c r="H6" t="n">
-        <v>14.151</v>
+        <v>14.968</v>
       </c>
       <c r="I6" t="n">
-        <v>10.491</v>
+        <v>12.349</v>
       </c>
       <c r="J6" t="n">
-        <v>2.775</v>
+        <v>2.638</v>
       </c>
       <c r="K6" t="n">
-        <v>2.27</v>
+        <v>2.12</v>
       </c>
       <c r="L6" t="n">
-        <v>1.987</v>
+        <v>1.053</v>
       </c>
       <c r="M6" t="n">
-        <v>0.261</v>
+        <v>0.23</v>
       </c>
       <c r="N6" t="n">
         <v>0.057</v>
       </c>
       <c r="O6" t="n">
-        <v>0.014</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="P6" t="n">
-        <v>0.029</v>
+        <v>0.02</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.004</v>
       </c>
       <c r="R6" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="S6" t="n">
         <v>0.018</v>
       </c>
-      <c r="S6" t="n">
-        <v>0.058</v>
-      </c>
       <c r="T6" t="n">
-        <v>0.025</v>
+        <v>0.019</v>
       </c>
       <c r="U6" t="n">
-        <v>1.421</v>
+        <v>1.212</v>
       </c>
     </row>
     <row r="7">
@@ -854,64 +854,64 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>3.182</v>
+        <v>2.075</v>
       </c>
       <c r="C7" t="n">
-        <v>15.631</v>
+        <v>15.872</v>
       </c>
       <c r="D7" t="n">
-        <v>1.004</v>
+        <v>11.712</v>
       </c>
       <c r="E7" t="n">
-        <v>12.104</v>
+        <v>1.069</v>
       </c>
       <c r="F7" t="n">
-        <v>14.682</v>
+        <v>14.349</v>
       </c>
       <c r="G7" t="n">
-        <v>12.591</v>
+        <v>12.548</v>
       </c>
       <c r="H7" t="n">
-        <v>12.785</v>
+        <v>14.836</v>
       </c>
       <c r="I7" t="n">
-        <v>12.631</v>
+        <v>14.527</v>
       </c>
       <c r="J7" t="n">
-        <v>4.765</v>
+        <v>4.409</v>
       </c>
       <c r="K7" t="n">
-        <v>3.999</v>
+        <v>3.689</v>
       </c>
       <c r="L7" t="n">
-        <v>3.139</v>
+        <v>1.821</v>
       </c>
       <c r="M7" t="n">
-        <v>0.5640000000000001</v>
+        <v>0.5760000000000001</v>
       </c>
       <c r="N7" t="n">
-        <v>0.136</v>
+        <v>0.128</v>
       </c>
       <c r="O7" t="n">
-        <v>0.023</v>
+        <v>0.022</v>
       </c>
       <c r="P7" t="n">
-        <v>0.057</v>
+        <v>0.044</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="R7" t="n">
-        <v>0.05599999999999999</v>
+        <v>0.036</v>
       </c>
       <c r="S7" t="n">
-        <v>0.135</v>
+        <v>0.049</v>
       </c>
       <c r="T7" t="n">
-        <v>0.05599999999999999</v>
+        <v>0.059</v>
       </c>
       <c r="U7" t="n">
-        <v>2.445</v>
+        <v>2.165</v>
       </c>
     </row>
     <row r="8">
@@ -919,64 +919,64 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>1.726</v>
+        <v>0.928</v>
       </c>
       <c r="C8" t="n">
-        <v>15.348</v>
+        <v>16.111</v>
       </c>
       <c r="D8" t="n">
-        <v>0.469</v>
+        <v>9.243</v>
       </c>
       <c r="E8" t="n">
-        <v>9.727</v>
+        <v>0.569</v>
       </c>
       <c r="F8" t="n">
-        <v>12.828</v>
+        <v>12.025</v>
       </c>
       <c r="G8" t="n">
-        <v>10.001</v>
+        <v>10.008</v>
       </c>
       <c r="H8" t="n">
-        <v>10.789</v>
+        <v>13.659</v>
       </c>
       <c r="I8" t="n">
-        <v>13.888</v>
+        <v>15.469</v>
       </c>
       <c r="J8" t="n">
-        <v>7.298</v>
+        <v>6.841</v>
       </c>
       <c r="K8" t="n">
-        <v>6.521000000000001</v>
+        <v>6.066</v>
       </c>
       <c r="L8" t="n">
-        <v>4.804</v>
+        <v>3.114</v>
       </c>
       <c r="M8" t="n">
-        <v>1.316</v>
+        <v>1.251</v>
       </c>
       <c r="N8" t="n">
-        <v>0.363</v>
+        <v>0.337</v>
       </c>
       <c r="O8" t="n">
-        <v>0.065</v>
+        <v>0.054</v>
       </c>
       <c r="P8" t="n">
-        <v>0.141</v>
+        <v>0.133</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.06899999999999999</v>
+        <v>0.053</v>
       </c>
       <c r="R8" t="n">
-        <v>0.131</v>
+        <v>0.112</v>
       </c>
       <c r="S8" t="n">
-        <v>0.307</v>
+        <v>0.14</v>
       </c>
       <c r="T8" t="n">
-        <v>0.154</v>
+        <v>0.124</v>
       </c>
       <c r="U8" t="n">
-        <v>4.055000000000001</v>
+        <v>3.763</v>
       </c>
     </row>
     <row r="9">
@@ -984,64 +984,64 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.8880000000000001</v>
+        <v>0.355</v>
       </c>
       <c r="C9" t="n">
-        <v>13.087</v>
+        <v>14.321</v>
       </c>
       <c r="D9" t="n">
-        <v>0.176</v>
+        <v>6.553000000000001</v>
       </c>
       <c r="E9" t="n">
-        <v>6.577</v>
+        <v>0.229</v>
       </c>
       <c r="F9" t="n">
-        <v>10.385</v>
+        <v>8.881</v>
       </c>
       <c r="G9" t="n">
-        <v>7.239</v>
+        <v>7.242999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>8.332000000000001</v>
+        <v>11.433</v>
       </c>
       <c r="I9" t="n">
-        <v>14.081</v>
+        <v>14.189</v>
       </c>
       <c r="J9" t="n">
-        <v>10.221</v>
+        <v>10.384</v>
       </c>
       <c r="K9" t="n">
-        <v>9.811999999999999</v>
+        <v>9.746</v>
       </c>
       <c r="L9" t="n">
-        <v>7.385</v>
+        <v>5.445</v>
       </c>
       <c r="M9" t="n">
-        <v>2.573</v>
+        <v>2.716</v>
       </c>
       <c r="N9" t="n">
-        <v>0.859</v>
+        <v>0.897</v>
       </c>
       <c r="O9" t="n">
-        <v>0.177</v>
+        <v>0.136</v>
       </c>
       <c r="P9" t="n">
-        <v>0.333</v>
+        <v>0.365</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.173</v>
+        <v>0.168</v>
       </c>
       <c r="R9" t="n">
-        <v>0.312</v>
+        <v>0.27</v>
       </c>
       <c r="S9" t="n">
-        <v>0.599</v>
+        <v>0.328</v>
       </c>
       <c r="T9" t="n">
-        <v>0.38</v>
+        <v>0.294</v>
       </c>
       <c r="U9" t="n">
-        <v>6.411</v>
+        <v>6.047000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -1049,64 +1049,64 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.365</v>
+        <v>0.1</v>
       </c>
       <c r="C10" t="n">
-        <v>8.921999999999999</v>
+        <v>9.371</v>
       </c>
       <c r="D10" t="n">
-        <v>0.091</v>
+        <v>3.953</v>
       </c>
       <c r="E10" t="n">
-        <v>4.273</v>
+        <v>0.105</v>
       </c>
       <c r="F10" t="n">
-        <v>6.682</v>
+        <v>5.611</v>
       </c>
       <c r="G10" t="n">
-        <v>4.43</v>
+        <v>4.359</v>
       </c>
       <c r="H10" t="n">
-        <v>5.462</v>
+        <v>7.255000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>11.674</v>
+        <v>10.021</v>
       </c>
       <c r="J10" t="n">
-        <v>13.626</v>
+        <v>14.811</v>
       </c>
       <c r="K10" t="n">
-        <v>13.512</v>
+        <v>14.364</v>
       </c>
       <c r="L10" t="n">
-        <v>10.351</v>
+        <v>8.859</v>
       </c>
       <c r="M10" t="n">
-        <v>4.821000000000001</v>
+        <v>5.177</v>
       </c>
       <c r="N10" t="n">
-        <v>1.868</v>
+        <v>2.147</v>
       </c>
       <c r="O10" t="n">
-        <v>0.439</v>
+        <v>0.422</v>
       </c>
       <c r="P10" t="n">
-        <v>0.8580000000000001</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.455</v>
+        <v>0.476</v>
       </c>
       <c r="R10" t="n">
-        <v>0.784</v>
+        <v>0.679</v>
       </c>
       <c r="S10" t="n">
-        <v>1.166</v>
+        <v>0.822</v>
       </c>
       <c r="T10" t="n">
-        <v>0.7779999999999999</v>
+        <v>0.718</v>
       </c>
       <c r="U10" t="n">
-        <v>9.443</v>
+        <v>9.814</v>
       </c>
     </row>
     <row r="11">
@@ -1114,64 +1114,64 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.113</v>
+        <v>0.017</v>
       </c>
       <c r="C11" t="n">
-        <v>5.105</v>
+        <v>5.235</v>
       </c>
       <c r="D11" t="n">
-        <v>0.021</v>
+        <v>2.02</v>
       </c>
       <c r="E11" t="n">
-        <v>2.374</v>
+        <v>0.031</v>
       </c>
       <c r="F11" t="n">
-        <v>3.887</v>
+        <v>3.101</v>
       </c>
       <c r="G11" t="n">
-        <v>2.515</v>
+        <v>2.425</v>
       </c>
       <c r="H11" t="n">
-        <v>3.313</v>
+        <v>3.928</v>
       </c>
       <c r="I11" t="n">
-        <v>8.462</v>
+        <v>6.263000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>14.9</v>
+        <v>15.599</v>
       </c>
       <c r="K11" t="n">
-        <v>15.177</v>
+        <v>16.274</v>
       </c>
       <c r="L11" t="n">
-        <v>12.672</v>
+        <v>12.076</v>
       </c>
       <c r="M11" t="n">
-        <v>7.575</v>
+        <v>8.154999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>3.521</v>
+        <v>3.999</v>
       </c>
       <c r="O11" t="n">
-        <v>0.9039999999999999</v>
+        <v>0.9129999999999999</v>
       </c>
       <c r="P11" t="n">
-        <v>1.782</v>
+        <v>2.008</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.9299999999999999</v>
+        <v>0.955</v>
       </c>
       <c r="R11" t="n">
-        <v>1.425</v>
+        <v>1.506</v>
       </c>
       <c r="S11" t="n">
-        <v>2.125</v>
+        <v>1.619</v>
       </c>
       <c r="T11" t="n">
-        <v>1.543</v>
+        <v>1.594</v>
       </c>
       <c r="U11" t="n">
-        <v>11.656</v>
+        <v>12.282</v>
       </c>
     </row>
     <row r="12">
@@ -1179,64 +1179,64 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>0.028</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>2.641</v>
+        <v>2.56</v>
       </c>
       <c r="D12" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.9950000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>1.228</v>
+        <v>0.005</v>
       </c>
       <c r="F12" t="n">
-        <v>2.087</v>
+        <v>1.495</v>
       </c>
       <c r="G12" t="n">
-        <v>1.298</v>
+        <v>1.208</v>
       </c>
       <c r="H12" t="n">
-        <v>1.87</v>
+        <v>2.019</v>
       </c>
       <c r="I12" t="n">
-        <v>5.452</v>
+        <v>3.492</v>
       </c>
       <c r="J12" t="n">
-        <v>13.496</v>
+        <v>13.891</v>
       </c>
       <c r="K12" t="n">
-        <v>14.015</v>
+        <v>14.237</v>
       </c>
       <c r="L12" t="n">
-        <v>13.322</v>
+        <v>13.806</v>
       </c>
       <c r="M12" t="n">
-        <v>10.732</v>
+        <v>11.39</v>
       </c>
       <c r="N12" t="n">
-        <v>5.64</v>
+        <v>6.248</v>
       </c>
       <c r="O12" t="n">
-        <v>1.677</v>
+        <v>1.808</v>
       </c>
       <c r="P12" t="n">
-        <v>3.56</v>
+        <v>3.786</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.791</v>
+        <v>1.879</v>
       </c>
       <c r="R12" t="n">
-        <v>2.493</v>
+        <v>2.635</v>
       </c>
       <c r="S12" t="n">
-        <v>3.422</v>
+        <v>2.865</v>
       </c>
       <c r="T12" t="n">
-        <v>2.686</v>
+        <v>2.7</v>
       </c>
       <c r="U12" t="n">
-        <v>12.555</v>
+        <v>12.981</v>
       </c>
     </row>
     <row r="13">
@@ -1244,64 +1244,64 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>0.011</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>1.176</v>
+        <v>1.155</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>0.398</v>
       </c>
       <c r="E13" t="n">
-        <v>0.5479999999999999</v>
+        <v>0.001</v>
       </c>
       <c r="F13" t="n">
-        <v>1.021</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>0.651</v>
+        <v>0.544</v>
       </c>
       <c r="H13" t="n">
-        <v>1.029</v>
+        <v>0.9199999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>3.17</v>
+        <v>1.856</v>
       </c>
       <c r="J13" t="n">
-        <v>10.64</v>
+        <v>10.481</v>
       </c>
       <c r="K13" t="n">
-        <v>11.395</v>
+        <v>11.252</v>
       </c>
       <c r="L13" t="n">
-        <v>12.206</v>
+        <v>13.37</v>
       </c>
       <c r="M13" t="n">
-        <v>12.871</v>
+        <v>13.148</v>
       </c>
       <c r="N13" t="n">
-        <v>7.997999999999999</v>
+        <v>8.540000000000001</v>
       </c>
       <c r="O13" t="n">
-        <v>2.987</v>
+        <v>3.094</v>
       </c>
       <c r="P13" t="n">
-        <v>5.646</v>
+        <v>6.101999999999999</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.994</v>
+        <v>3.18</v>
       </c>
       <c r="R13" t="n">
-        <v>3.929</v>
+        <v>4.215</v>
       </c>
       <c r="S13" t="n">
-        <v>5.192</v>
+        <v>4.514</v>
       </c>
       <c r="T13" t="n">
-        <v>4.324999999999999</v>
+        <v>4.288</v>
       </c>
       <c r="U13" t="n">
-        <v>12.211</v>
+        <v>12.25</v>
       </c>
     </row>
     <row r="14">
@@ -1312,61 +1312,61 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0.47</v>
+        <v>0.382</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>0.14</v>
       </c>
       <c r="E14" t="n">
-        <v>0.268</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.407</v>
+        <v>0.269</v>
       </c>
       <c r="G14" t="n">
-        <v>0.288</v>
+        <v>0.19</v>
       </c>
       <c r="H14" t="n">
-        <v>0.443</v>
+        <v>0.365</v>
       </c>
       <c r="I14" t="n">
-        <v>1.763</v>
+        <v>0.959</v>
       </c>
       <c r="J14" t="n">
-        <v>7.667</v>
+        <v>7.337000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>8.347999999999999</v>
+        <v>8.116</v>
       </c>
       <c r="L14" t="n">
-        <v>9.977</v>
+        <v>11.578</v>
       </c>
       <c r="M14" t="n">
-        <v>13.617</v>
+        <v>13.522</v>
       </c>
       <c r="N14" t="n">
-        <v>10.172</v>
+        <v>10.529</v>
       </c>
       <c r="O14" t="n">
-        <v>4.679</v>
+        <v>4.813</v>
       </c>
       <c r="P14" t="n">
-        <v>8.304</v>
+        <v>8.619</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.464</v>
+        <v>4.718</v>
       </c>
       <c r="R14" t="n">
-        <v>5.622</v>
+        <v>5.852</v>
       </c>
       <c r="S14" t="n">
-        <v>7.231999999999999</v>
+        <v>6.146</v>
       </c>
       <c r="T14" t="n">
-        <v>6.088</v>
+        <v>6.096</v>
       </c>
       <c r="U14" t="n">
-        <v>10.191</v>
+        <v>10.369</v>
       </c>
     </row>
     <row r="15">
@@ -1377,61 +1377,61 @@
         <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>0.171</v>
+        <v>0.135</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>0.044</v>
       </c>
       <c r="E15" t="n">
-        <v>0.106</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.164</v>
+        <v>0.107</v>
       </c>
       <c r="G15" t="n">
-        <v>0.112</v>
+        <v>0.095</v>
       </c>
       <c r="H15" t="n">
-        <v>0.167</v>
+        <v>0.193</v>
       </c>
       <c r="I15" t="n">
-        <v>0.868</v>
+        <v>0.451</v>
       </c>
       <c r="J15" t="n">
-        <v>5.082</v>
+        <v>4.923</v>
       </c>
       <c r="K15" t="n">
-        <v>5.443</v>
+        <v>5.278</v>
       </c>
       <c r="L15" t="n">
-        <v>7.693</v>
+        <v>9.120000000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>12.372</v>
+        <v>11.985</v>
       </c>
       <c r="N15" t="n">
-        <v>11.796</v>
+        <v>11.911</v>
       </c>
       <c r="O15" t="n">
-        <v>6.666999999999999</v>
+        <v>6.589</v>
       </c>
       <c r="P15" t="n">
-        <v>10.435</v>
+        <v>10.959</v>
       </c>
       <c r="Q15" t="n">
-        <v>6.278</v>
+        <v>6.497999999999999</v>
       </c>
       <c r="R15" t="n">
-        <v>7.56</v>
+        <v>7.542999999999999</v>
       </c>
       <c r="S15" t="n">
-        <v>8.887</v>
+        <v>8.015000000000001</v>
       </c>
       <c r="T15" t="n">
-        <v>7.745</v>
+        <v>7.988</v>
       </c>
       <c r="U15" t="n">
-        <v>8.454000000000001</v>
+        <v>8.166</v>
       </c>
     </row>
     <row r="16">
@@ -1442,61 +1442,61 @@
         <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>0.046</v>
+        <v>0.037</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>0.028</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0.094</v>
+        <v>0.026</v>
       </c>
       <c r="G16" t="n">
-        <v>0.054</v>
+        <v>0.031</v>
       </c>
       <c r="H16" t="n">
         <v>0.08</v>
       </c>
       <c r="I16" t="n">
-        <v>0.421</v>
+        <v>0.215</v>
       </c>
       <c r="J16" t="n">
-        <v>3.224</v>
+        <v>2.942</v>
       </c>
       <c r="K16" t="n">
-        <v>3.528</v>
+        <v>3.387</v>
       </c>
       <c r="L16" t="n">
-        <v>5.448</v>
+        <v>6.793</v>
       </c>
       <c r="M16" t="n">
-        <v>10.106</v>
+        <v>9.718999999999999</v>
       </c>
       <c r="N16" t="n">
-        <v>12.22</v>
+        <v>12.3</v>
       </c>
       <c r="O16" t="n">
-        <v>8.803999999999998</v>
+        <v>8.591999999999999</v>
       </c>
       <c r="P16" t="n">
-        <v>12.18</v>
+        <v>12.185</v>
       </c>
       <c r="Q16" t="n">
-        <v>8.341999999999999</v>
+        <v>8.486000000000001</v>
       </c>
       <c r="R16" t="n">
-        <v>9.089</v>
+        <v>9.216000000000001</v>
       </c>
       <c r="S16" t="n">
-        <v>10.313</v>
+        <v>9.854000000000001</v>
       </c>
       <c r="T16" t="n">
-        <v>9.541</v>
+        <v>9.415999999999999</v>
       </c>
       <c r="U16" t="n">
-        <v>6.482</v>
+        <v>6.714</v>
       </c>
     </row>
     <row r="17">
@@ -1507,61 +1507,61 @@
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="E17" t="n">
-        <v>0.014</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0.032</v>
+        <v>0.013</v>
       </c>
       <c r="G17" t="n">
-        <v>0.014</v>
+        <v>0.006</v>
       </c>
       <c r="H17" t="n">
-        <v>0.032</v>
+        <v>0.021</v>
       </c>
       <c r="I17" t="n">
-        <v>0.216</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>1.937</v>
+        <v>1.752</v>
       </c>
       <c r="K17" t="n">
-        <v>2.101</v>
+        <v>1.951</v>
       </c>
       <c r="L17" t="n">
-        <v>3.817</v>
+        <v>4.917</v>
       </c>
       <c r="M17" t="n">
-        <v>8.079000000000001</v>
+        <v>7.829999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>11.689</v>
+        <v>11.595</v>
       </c>
       <c r="O17" t="n">
-        <v>10.962</v>
+        <v>10.813</v>
       </c>
       <c r="P17" t="n">
-        <v>12.678</v>
+        <v>12.549</v>
       </c>
       <c r="Q17" t="n">
-        <v>10.367</v>
+        <v>10.707</v>
       </c>
       <c r="R17" t="n">
-        <v>10.825</v>
+        <v>10.903</v>
       </c>
       <c r="S17" t="n">
-        <v>11.147</v>
+        <v>11.109</v>
       </c>
       <c r="T17" t="n">
-        <v>11.164</v>
+        <v>10.956</v>
       </c>
       <c r="U17" t="n">
-        <v>4.911</v>
+        <v>4.784999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -1572,61 +1572,61 @@
         <v>0</v>
       </c>
       <c r="C18" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
         <v>0.002</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.008</v>
       </c>
       <c r="G18" t="n">
         <v>0.003</v>
       </c>
       <c r="H18" t="n">
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
       <c r="I18" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.024</v>
       </c>
       <c r="J18" t="n">
-        <v>1.032</v>
+        <v>0.984</v>
       </c>
       <c r="K18" t="n">
-        <v>1.195</v>
+        <v>1.063</v>
       </c>
       <c r="L18" t="n">
-        <v>2.547</v>
+        <v>3.293</v>
       </c>
       <c r="M18" t="n">
-        <v>6.104</v>
+        <v>5.776</v>
       </c>
       <c r="N18" t="n">
-        <v>10.863</v>
+        <v>10.344</v>
       </c>
       <c r="O18" t="n">
-        <v>13.079</v>
+        <v>13.154</v>
       </c>
       <c r="P18" t="n">
-        <v>12.42</v>
+        <v>12.286</v>
       </c>
       <c r="Q18" t="n">
-        <v>12.619</v>
+        <v>12.825</v>
       </c>
       <c r="R18" t="n">
-        <v>12.303</v>
+        <v>12.312</v>
       </c>
       <c r="S18" t="n">
-        <v>11.727</v>
+        <v>12.294</v>
       </c>
       <c r="T18" t="n">
-        <v>12.469</v>
+        <v>12.029</v>
       </c>
       <c r="U18" t="n">
-        <v>3.544</v>
+        <v>3.602</v>
       </c>
     </row>
     <row r="19">
@@ -1637,61 +1637,61 @@
         <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0.006999999999999999</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0.037</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>0.503</v>
+        <v>0.454</v>
       </c>
       <c r="K19" t="n">
-        <v>0.5660000000000001</v>
+        <v>0.553</v>
       </c>
       <c r="L19" t="n">
-        <v>1.536</v>
+        <v>2.172</v>
       </c>
       <c r="M19" t="n">
-        <v>4.465</v>
+        <v>4.233</v>
       </c>
       <c r="N19" t="n">
-        <v>9.585000000000001</v>
+        <v>8.853999999999999</v>
       </c>
       <c r="O19" t="n">
-        <v>15.06</v>
+        <v>15.113</v>
       </c>
       <c r="P19" t="n">
-        <v>11.647</v>
+        <v>11.192</v>
       </c>
       <c r="Q19" t="n">
-        <v>14.97</v>
+        <v>14.903</v>
       </c>
       <c r="R19" t="n">
-        <v>13.75</v>
+        <v>13.924</v>
       </c>
       <c r="S19" t="n">
-        <v>12.115</v>
+        <v>12.985</v>
       </c>
       <c r="T19" t="n">
-        <v>13.208</v>
+        <v>13.158</v>
       </c>
       <c r="U19" t="n">
-        <v>2.54</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="20">
@@ -1714,49 +1714,49 @@
         <v>0.001</v>
       </c>
       <c r="G20" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>0.008</v>
+        <v>0.003</v>
       </c>
       <c r="J20" t="n">
-        <v>0.207</v>
+        <v>0.214</v>
       </c>
       <c r="K20" t="n">
-        <v>0.27</v>
+        <v>0.216</v>
       </c>
       <c r="L20" t="n">
-        <v>0.876</v>
+        <v>1.238</v>
       </c>
       <c r="M20" t="n">
-        <v>2.855</v>
+        <v>2.821</v>
       </c>
       <c r="N20" t="n">
-        <v>7.704999999999999</v>
+        <v>7.037</v>
       </c>
       <c r="O20" t="n">
-        <v>16.721</v>
+        <v>16.9</v>
       </c>
       <c r="P20" t="n">
-        <v>10.803</v>
+        <v>10.303</v>
       </c>
       <c r="Q20" t="n">
-        <v>17.291</v>
+        <v>16.646</v>
       </c>
       <c r="R20" t="n">
-        <v>15.041</v>
+        <v>14.799</v>
       </c>
       <c r="S20" t="n">
-        <v>12.432</v>
+        <v>14.053</v>
       </c>
       <c r="T20" t="n">
-        <v>14.099</v>
+        <v>14.182</v>
       </c>
       <c r="U20" t="n">
-        <v>1.69</v>
+        <v>1.587</v>
       </c>
     </row>
     <row r="21">
@@ -1785,43 +1785,43 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0.045</v>
+        <v>0.052</v>
       </c>
       <c r="K21" t="n">
         <v>0.059</v>
       </c>
       <c r="L21" t="n">
-        <v>0.364</v>
+        <v>0.526</v>
       </c>
       <c r="M21" t="n">
-        <v>1.56</v>
+        <v>1.359</v>
       </c>
       <c r="N21" t="n">
-        <v>5.514</v>
+        <v>5.061</v>
       </c>
       <c r="O21" t="n">
-        <v>17.74</v>
+        <v>17.567</v>
       </c>
       <c r="P21" t="n">
-        <v>9.120000000000001</v>
+        <v>8.512</v>
       </c>
       <c r="Q21" t="n">
-        <v>19.235</v>
+        <v>18.487</v>
       </c>
       <c r="R21" t="n">
-        <v>16.654</v>
+        <v>15.977</v>
       </c>
       <c r="S21" t="n">
-        <v>13.111</v>
+        <v>15.179</v>
       </c>
       <c r="T21" t="n">
-        <v>15.735</v>
+        <v>16.371</v>
       </c>
       <c r="U21" t="n">
-        <v>0.861</v>
+        <v>0.8500000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1853,51 +1853,51 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Atlético Nacional</t>
+          <t>América de Cali</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99.881</v>
+        <v>99.88300000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>América de Cali</t>
+          <t>Atlético Nacional</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.48299999999999</v>
+        <v>99.85799999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Atlético Bucaramanga</t>
+          <t>Independiente Medellín</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>91.154</v>
+        <v>92.435</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Atlético Bucaramanga</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>90.63200000000001</v>
+        <v>91.13900000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Independiente Medellín</t>
+          <t>Deportivo Cali</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>87.59100000000001</v>
+        <v>88.68299999999999</v>
       </c>
     </row>
     <row r="7">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>85.61000000000001</v>
+        <v>85.215</v>
       </c>
     </row>
     <row r="8">
@@ -1917,17 +1917,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>81.45</v>
+        <v>81.107</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Deportivo Cali</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>67.855</v>
+        <v>76.63499999999999</v>
       </c>
     </row>
     <row r="10">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>27.641</v>
+        <v>26.56</v>
       </c>
     </row>
     <row r="11">
@@ -1947,27 +1947,27 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>24.391</v>
+        <v>23.25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Águilas Doradas</t>
+          <t>Junior</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>19.191</v>
+        <v>14.15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>Águilas Doradas</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15.462</v>
+        <v>12.252</v>
       </c>
     </row>
     <row r="14">
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4.843</v>
+        <v>4.885000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -1987,17 +1987,17 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.429</v>
+        <v>1.435</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jaguares</t>
+          <t>Deportivo Pasto</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.131</v>
+        <v>0.5630000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -2007,17 +2007,17 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.619</v>
+        <v>0.5449999999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Deportivo Pasto</t>
+          <t>Jaguares</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.5670000000000001</v>
+        <v>0.504</v>
       </c>
     </row>
     <row r="19">
@@ -2027,27 +2027,27 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.525</v>
+        <v>0.439</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Alianza Valledupar</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.281</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Alianza Valledupar</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.264</v>
+        <v>0.222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar resultados de Finalizacion 2026-II hasta el 25/09/2026
- Carga 3 partidos jugados el 24 y 25 de septiembre (Atletico
  Nacional 1-1 Millonarios, Boyaca Chico 3-0 Deportivo Pasto, Once
  Caldas 1-3 Atletico Bucaramanga) con actualizar_resultados.py.
- Tabla.csv/Partidos.csv/Historial_partidos.csv actualizados;
  historial pasa de 752 a 755 partidos. Tabla verificada contra
  Dimayor en vivo. Atletico Bucaramanga sube al 2 puesto.
- model_params.csv: DrawBias recalibrado exacto (222/755).
- Resultados.xlsx/Resultado.png regenerados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resultados.xlsx
+++ b/Resultados.xlsx
@@ -430,29 +430,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Atlético Bucaramanga</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Millonarios</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Atlético Nacional</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>Independiente Medellín</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Atlético Nacional</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Deportivo Cali</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Atlético Bucaramanga</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>Deportes Tolima</t>
@@ -485,27 +485,27 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>Boyacá Chicó</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>Cúcuta Deportivo</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Fortaleza</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Deportivo Pasto</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Alianza Valledupar</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Boyacá Chicó</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
@@ -529,37 +529,37 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>30.125</v>
+        <v>33.813</v>
       </c>
       <c r="C2" t="n">
-        <v>0.597</v>
+        <v>11.193</v>
       </c>
       <c r="D2" t="n">
-        <v>4.723</v>
+        <v>0.641</v>
       </c>
       <c r="E2" t="n">
-        <v>57.126</v>
+        <v>44.843</v>
       </c>
       <c r="F2" t="n">
-        <v>1.736</v>
+        <v>5.396999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>3.851</v>
+        <v>2.005</v>
       </c>
       <c r="H2" t="n">
-        <v>1.231</v>
+        <v>1.41</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5740000000000001</v>
+        <v>0.6629999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>0.017</v>
+        <v>0.021</v>
       </c>
       <c r="K2" t="n">
-        <v>0.009000000000000001</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>0.003</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -580,13 +580,13 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="3">
@@ -594,64 +594,64 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>38.68</v>
+        <v>31.403</v>
       </c>
       <c r="C3" t="n">
-        <v>2.52</v>
+        <v>16.958</v>
       </c>
       <c r="D3" t="n">
-        <v>10.741</v>
+        <v>2.578</v>
       </c>
       <c r="E3" t="n">
-        <v>25.4</v>
+        <v>27.261</v>
       </c>
       <c r="F3" t="n">
-        <v>6.265</v>
+        <v>9.653</v>
       </c>
       <c r="G3" t="n">
-        <v>9.218999999999999</v>
+        <v>5.503</v>
       </c>
       <c r="H3" t="n">
-        <v>4.378</v>
+        <v>4.059</v>
       </c>
       <c r="I3" t="n">
-        <v>2.478</v>
+        <v>2.369</v>
       </c>
       <c r="J3" t="n">
-        <v>0.145</v>
+        <v>0.137</v>
       </c>
       <c r="K3" t="n">
-        <v>0.075</v>
+        <v>0.003</v>
       </c>
       <c r="L3" t="n">
-        <v>0.045</v>
+        <v>0.028</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
         <v>0.001</v>
       </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0.053</v>
+        <v>0.046</v>
       </c>
     </row>
     <row r="4">
@@ -659,64 +659,64 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>15.686</v>
+        <v>16.397</v>
       </c>
       <c r="C4" t="n">
-        <v>7.274999999999999</v>
+        <v>22.234</v>
       </c>
       <c r="D4" t="n">
-        <v>18.112</v>
+        <v>7.041</v>
       </c>
       <c r="E4" t="n">
-        <v>9.039999999999999</v>
+        <v>13.16</v>
       </c>
       <c r="F4" t="n">
-        <v>13.647</v>
+        <v>15.068</v>
       </c>
       <c r="G4" t="n">
-        <v>16.696</v>
+        <v>11.022</v>
       </c>
       <c r="H4" t="n">
-        <v>10.925</v>
+        <v>8.584999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>7.044</v>
+        <v>5.606</v>
       </c>
       <c r="J4" t="n">
-        <v>0.65</v>
+        <v>0.453</v>
       </c>
       <c r="K4" t="n">
-        <v>0.412</v>
+        <v>0.039</v>
       </c>
       <c r="L4" t="n">
-        <v>0.229</v>
+        <v>0.178</v>
       </c>
       <c r="M4" t="n">
-        <v>0.022</v>
+        <v>0.016</v>
       </c>
       <c r="N4" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="P4" t="n">
         <v>0.001</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="T4" t="n">
         <v>0.001</v>
       </c>
       <c r="U4" t="n">
-        <v>0.253</v>
+        <v>0.193</v>
       </c>
     </row>
     <row r="5">
@@ -724,64 +724,64 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>7.922</v>
+        <v>9.098000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>10.7</v>
+        <v>17.427</v>
       </c>
       <c r="D5" t="n">
-        <v>16.931</v>
+        <v>11.538</v>
       </c>
       <c r="E5" t="n">
-        <v>4.225000000000001</v>
+        <v>7.238</v>
       </c>
       <c r="F5" t="n">
-        <v>15.958</v>
+        <v>16.697</v>
       </c>
       <c r="G5" t="n">
-        <v>16.553</v>
+        <v>14.668</v>
       </c>
       <c r="H5" t="n">
-        <v>13.785</v>
+        <v>12.513</v>
       </c>
       <c r="I5" t="n">
-        <v>10.005</v>
+        <v>8.554</v>
       </c>
       <c r="J5" t="n">
-        <v>1.476</v>
+        <v>1.164</v>
       </c>
       <c r="K5" t="n">
-        <v>1.133</v>
+        <v>0.132</v>
       </c>
       <c r="L5" t="n">
-        <v>0.542</v>
+        <v>0.399</v>
       </c>
       <c r="M5" t="n">
-        <v>0.09</v>
+        <v>0.055</v>
       </c>
       <c r="N5" t="n">
-        <v>0.011</v>
+        <v>0.01</v>
       </c>
       <c r="O5" t="n">
-        <v>0.003</v>
+        <v>0.008</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="Q5" t="n">
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.005</v>
       </c>
       <c r="T5" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.002</v>
       </c>
       <c r="U5" t="n">
-        <v>0.649</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="6">
@@ -789,64 +789,64 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>4.112</v>
+        <v>4.853</v>
       </c>
       <c r="C6" t="n">
-        <v>13.711</v>
+        <v>12.756</v>
       </c>
       <c r="D6" t="n">
-        <v>14.42</v>
+        <v>15.141</v>
       </c>
       <c r="E6" t="n">
-        <v>2.2</v>
+        <v>3.889</v>
       </c>
       <c r="F6" t="n">
-        <v>15.822</v>
+        <v>15.24</v>
       </c>
       <c r="G6" t="n">
-        <v>15.021</v>
+        <v>16.189</v>
       </c>
       <c r="H6" t="n">
-        <v>14.968</v>
+        <v>14.964</v>
       </c>
       <c r="I6" t="n">
-        <v>12.349</v>
+        <v>11.937</v>
       </c>
       <c r="J6" t="n">
-        <v>2.638</v>
+        <v>2.36</v>
       </c>
       <c r="K6" t="n">
-        <v>2.12</v>
+        <v>0.414</v>
       </c>
       <c r="L6" t="n">
-        <v>1.053</v>
+        <v>0.9209999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>0.23</v>
+        <v>0.177</v>
       </c>
       <c r="N6" t="n">
-        <v>0.057</v>
+        <v>0.038</v>
       </c>
       <c r="O6" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.02</v>
       </c>
       <c r="P6" t="n">
-        <v>0.02</v>
+        <v>0.004</v>
       </c>
       <c r="Q6" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="R6" t="n">
         <v>0.004</v>
       </c>
-      <c r="R6" t="n">
-        <v>0.019</v>
-      </c>
       <c r="S6" t="n">
-        <v>0.018</v>
+        <v>0.022</v>
       </c>
       <c r="T6" t="n">
-        <v>0.019</v>
+        <v>0.014</v>
       </c>
       <c r="U6" t="n">
-        <v>1.212</v>
+        <v>1.055</v>
       </c>
     </row>
     <row r="7">
@@ -854,64 +854,64 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>2.075</v>
+        <v>2.676</v>
       </c>
       <c r="C7" t="n">
-        <v>15.872</v>
+        <v>8.593</v>
       </c>
       <c r="D7" t="n">
-        <v>11.712</v>
+        <v>17.704</v>
       </c>
       <c r="E7" t="n">
-        <v>1.069</v>
+        <v>2.011</v>
       </c>
       <c r="F7" t="n">
-        <v>14.349</v>
+        <v>13.142</v>
       </c>
       <c r="G7" t="n">
-        <v>12.548</v>
+        <v>15.679</v>
       </c>
       <c r="H7" t="n">
-        <v>14.836</v>
+        <v>15.835</v>
       </c>
       <c r="I7" t="n">
-        <v>14.527</v>
+        <v>14.532</v>
       </c>
       <c r="J7" t="n">
-        <v>4.409</v>
+        <v>4.105</v>
       </c>
       <c r="K7" t="n">
-        <v>3.689</v>
+        <v>1.04</v>
       </c>
       <c r="L7" t="n">
-        <v>1.821</v>
+        <v>1.717</v>
       </c>
       <c r="M7" t="n">
-        <v>0.5760000000000001</v>
+        <v>0.483</v>
       </c>
       <c r="N7" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="O7" t="n">
         <v>0.128</v>
       </c>
-      <c r="O7" t="n">
-        <v>0.022</v>
-      </c>
       <c r="P7" t="n">
-        <v>0.044</v>
+        <v>0.013</v>
       </c>
       <c r="Q7" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="R7" t="n">
         <v>0.014</v>
       </c>
-      <c r="R7" t="n">
-        <v>0.036</v>
-      </c>
       <c r="S7" t="n">
-        <v>0.049</v>
+        <v>0.059</v>
       </c>
       <c r="T7" t="n">
-        <v>0.059</v>
+        <v>0.048</v>
       </c>
       <c r="U7" t="n">
-        <v>2.165</v>
+        <v>2.104</v>
       </c>
     </row>
     <row r="8">
@@ -919,64 +919,64 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>0.928</v>
+        <v>1.202</v>
       </c>
       <c r="C8" t="n">
-        <v>16.111</v>
+        <v>5.571000000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>9.243</v>
+        <v>17.714</v>
       </c>
       <c r="E8" t="n">
-        <v>0.569</v>
+        <v>0.9740000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>12.025</v>
+        <v>10.309</v>
       </c>
       <c r="G8" t="n">
-        <v>10.008</v>
+        <v>13.631</v>
       </c>
       <c r="H8" t="n">
-        <v>13.659</v>
+        <v>15.368</v>
       </c>
       <c r="I8" t="n">
-        <v>15.469</v>
+        <v>16.861</v>
       </c>
       <c r="J8" t="n">
-        <v>6.841</v>
+        <v>6.987</v>
       </c>
       <c r="K8" t="n">
-        <v>6.066</v>
+        <v>2.415</v>
       </c>
       <c r="L8" t="n">
-        <v>3.114</v>
+        <v>3.047</v>
       </c>
       <c r="M8" t="n">
-        <v>1.251</v>
+        <v>1.224</v>
       </c>
       <c r="N8" t="n">
-        <v>0.337</v>
+        <v>0.304</v>
       </c>
       <c r="O8" t="n">
-        <v>0.054</v>
+        <v>0.322</v>
       </c>
       <c r="P8" t="n">
-        <v>0.133</v>
+        <v>0.046</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.053</v>
+        <v>0.019</v>
       </c>
       <c r="R8" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="T8" t="n">
         <v>0.112</v>
       </c>
-      <c r="S8" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0.124</v>
-      </c>
       <c r="U8" t="n">
-        <v>3.763</v>
+        <v>3.695</v>
       </c>
     </row>
     <row r="9">
@@ -984,64 +984,64 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.355</v>
+        <v>0.427</v>
       </c>
       <c r="C9" t="n">
-        <v>14.321</v>
+        <v>3.183</v>
       </c>
       <c r="D9" t="n">
-        <v>6.553000000000001</v>
+        <v>14.343</v>
       </c>
       <c r="E9" t="n">
-        <v>0.229</v>
+        <v>0.439</v>
       </c>
       <c r="F9" t="n">
-        <v>8.881</v>
+        <v>7.524</v>
       </c>
       <c r="G9" t="n">
-        <v>7.242999999999999</v>
+        <v>10.178</v>
       </c>
       <c r="H9" t="n">
-        <v>11.433</v>
+        <v>13.115</v>
       </c>
       <c r="I9" t="n">
-        <v>14.189</v>
+        <v>16.305</v>
       </c>
       <c r="J9" t="n">
-        <v>10.384</v>
+        <v>11.372</v>
       </c>
       <c r="K9" t="n">
-        <v>9.746</v>
+        <v>5.165</v>
       </c>
       <c r="L9" t="n">
-        <v>5.445</v>
+        <v>5.627</v>
       </c>
       <c r="M9" t="n">
-        <v>2.716</v>
+        <v>2.675</v>
       </c>
       <c r="N9" t="n">
-        <v>0.897</v>
+        <v>0.828</v>
       </c>
       <c r="O9" t="n">
-        <v>0.136</v>
+        <v>1.017</v>
       </c>
       <c r="P9" t="n">
-        <v>0.365</v>
+        <v>0.178</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.168</v>
+        <v>0.059</v>
       </c>
       <c r="R9" t="n">
-        <v>0.27</v>
+        <v>0.161</v>
       </c>
       <c r="S9" t="n">
-        <v>0.328</v>
+        <v>0.385</v>
       </c>
       <c r="T9" t="n">
-        <v>0.294</v>
+        <v>0.347</v>
       </c>
       <c r="U9" t="n">
-        <v>6.047000000000001</v>
+        <v>6.672000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -1049,64 +1049,64 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="C10" t="n">
-        <v>9.371</v>
+        <v>1.353</v>
       </c>
       <c r="D10" t="n">
-        <v>3.953</v>
+        <v>7.76</v>
       </c>
       <c r="E10" t="n">
-        <v>0.105</v>
+        <v>0.133</v>
       </c>
       <c r="F10" t="n">
-        <v>5.611</v>
+        <v>3.967</v>
       </c>
       <c r="G10" t="n">
-        <v>4.359</v>
+        <v>5.847</v>
       </c>
       <c r="H10" t="n">
-        <v>7.255000000000001</v>
+        <v>7.317</v>
       </c>
       <c r="I10" t="n">
-        <v>10.021</v>
+        <v>10.822</v>
       </c>
       <c r="J10" t="n">
-        <v>14.811</v>
+        <v>17.358</v>
       </c>
       <c r="K10" t="n">
-        <v>14.364</v>
+        <v>10.375</v>
       </c>
       <c r="L10" t="n">
-        <v>8.859</v>
+        <v>10.274</v>
       </c>
       <c r="M10" t="n">
-        <v>5.177</v>
+        <v>5.93</v>
       </c>
       <c r="N10" t="n">
-        <v>2.147</v>
+        <v>1.924</v>
       </c>
       <c r="O10" t="n">
-        <v>0.422</v>
+        <v>2.469</v>
       </c>
       <c r="P10" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.4329999999999999</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.476</v>
+        <v>0.251</v>
       </c>
       <c r="R10" t="n">
-        <v>0.679</v>
+        <v>0.569</v>
       </c>
       <c r="S10" t="n">
-        <v>0.822</v>
+        <v>1.07</v>
       </c>
       <c r="T10" t="n">
-        <v>0.718</v>
+        <v>0.856</v>
       </c>
       <c r="U10" t="n">
-        <v>9.814</v>
+        <v>11.182</v>
       </c>
     </row>
     <row r="11">
@@ -1114,64 +1114,64 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.017</v>
+        <v>0.02</v>
       </c>
       <c r="C11" t="n">
-        <v>5.235</v>
+        <v>0.49</v>
       </c>
       <c r="D11" t="n">
-        <v>2.02</v>
+        <v>3.363</v>
       </c>
       <c r="E11" t="n">
-        <v>0.031</v>
+        <v>0.036</v>
       </c>
       <c r="F11" t="n">
-        <v>3.101</v>
+        <v>1.758</v>
       </c>
       <c r="G11" t="n">
-        <v>2.425</v>
+        <v>2.998</v>
       </c>
       <c r="H11" t="n">
-        <v>3.928</v>
+        <v>3.786</v>
       </c>
       <c r="I11" t="n">
-        <v>6.263000000000001</v>
+        <v>6.078</v>
       </c>
       <c r="J11" t="n">
-        <v>15.599</v>
+        <v>16.216</v>
       </c>
       <c r="K11" t="n">
-        <v>16.274</v>
+        <v>14.411</v>
       </c>
       <c r="L11" t="n">
-        <v>12.076</v>
+        <v>13.356</v>
       </c>
       <c r="M11" t="n">
-        <v>8.154999999999999</v>
+        <v>9.438000000000001</v>
       </c>
       <c r="N11" t="n">
-        <v>3.999</v>
+        <v>3.758</v>
       </c>
       <c r="O11" t="n">
-        <v>0.9129999999999999</v>
+        <v>4.464</v>
       </c>
       <c r="P11" t="n">
-        <v>2.008</v>
+        <v>1.009</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.955</v>
+        <v>0.657</v>
       </c>
       <c r="R11" t="n">
-        <v>1.506</v>
+        <v>1.224</v>
       </c>
       <c r="S11" t="n">
-        <v>1.619</v>
+        <v>1.963</v>
       </c>
       <c r="T11" t="n">
-        <v>1.594</v>
+        <v>1.778</v>
       </c>
       <c r="U11" t="n">
-        <v>12.282</v>
+        <v>13.197</v>
       </c>
     </row>
     <row r="12">
@@ -1179,64 +1179,64 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="C12" t="n">
-        <v>2.56</v>
+        <v>0.17</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9950000000000001</v>
+        <v>1.381</v>
       </c>
       <c r="E12" t="n">
-        <v>0.005</v>
+        <v>0.013</v>
       </c>
       <c r="F12" t="n">
-        <v>1.495</v>
+        <v>0.7979999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>1.208</v>
+        <v>1.313</v>
       </c>
       <c r="H12" t="n">
-        <v>2.019</v>
+        <v>1.706</v>
       </c>
       <c r="I12" t="n">
-        <v>3.492</v>
+        <v>3.223</v>
       </c>
       <c r="J12" t="n">
-        <v>13.891</v>
+        <v>12.672</v>
       </c>
       <c r="K12" t="n">
-        <v>14.237</v>
+        <v>15.6</v>
       </c>
       <c r="L12" t="n">
-        <v>13.806</v>
+        <v>14.07</v>
       </c>
       <c r="M12" t="n">
-        <v>11.39</v>
+        <v>12.015</v>
       </c>
       <c r="N12" t="n">
-        <v>6.248</v>
+        <v>5.865</v>
       </c>
       <c r="O12" t="n">
-        <v>1.808</v>
+        <v>6.504</v>
       </c>
       <c r="P12" t="n">
-        <v>3.786</v>
+        <v>1.944</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.879</v>
+        <v>1.518</v>
       </c>
       <c r="R12" t="n">
-        <v>2.635</v>
+        <v>2.141</v>
       </c>
       <c r="S12" t="n">
-        <v>2.865</v>
+        <v>3.266</v>
       </c>
       <c r="T12" t="n">
-        <v>2.7</v>
+        <v>2.935</v>
       </c>
       <c r="U12" t="n">
-        <v>12.981</v>
+        <v>12.865</v>
       </c>
     </row>
     <row r="13">
@@ -1247,61 +1247,61 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>1.155</v>
+        <v>0.055</v>
       </c>
       <c r="D13" t="n">
-        <v>0.398</v>
+        <v>0.5309999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="F13" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.286</v>
       </c>
       <c r="G13" t="n">
-        <v>0.544</v>
+        <v>0.582</v>
       </c>
       <c r="H13" t="n">
-        <v>0.9199999999999999</v>
+        <v>0.7779999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>1.856</v>
+        <v>1.664</v>
       </c>
       <c r="J13" t="n">
-        <v>10.481</v>
+        <v>9.494</v>
       </c>
       <c r="K13" t="n">
-        <v>11.252</v>
+        <v>14.202</v>
       </c>
       <c r="L13" t="n">
-        <v>13.37</v>
+        <v>12.735</v>
       </c>
       <c r="M13" t="n">
-        <v>13.148</v>
+        <v>13.086</v>
       </c>
       <c r="N13" t="n">
-        <v>8.540000000000001</v>
+        <v>7.85</v>
       </c>
       <c r="O13" t="n">
-        <v>3.094</v>
+        <v>8.612</v>
       </c>
       <c r="P13" t="n">
-        <v>6.101999999999999</v>
+        <v>3.263</v>
       </c>
       <c r="Q13" t="n">
-        <v>3.18</v>
+        <v>2.734</v>
       </c>
       <c r="R13" t="n">
-        <v>4.215</v>
+        <v>3.355</v>
       </c>
       <c r="S13" t="n">
-        <v>4.514</v>
+        <v>4.69</v>
       </c>
       <c r="T13" t="n">
-        <v>4.288</v>
+        <v>4.443</v>
       </c>
       <c r="U13" t="n">
-        <v>12.25</v>
+        <v>11.637</v>
       </c>
     </row>
     <row r="14">
@@ -1312,61 +1312,61 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0.382</v>
+        <v>0.013</v>
       </c>
       <c r="D14" t="n">
-        <v>0.14</v>
+        <v>0.196</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.269</v>
+        <v>0.117</v>
       </c>
       <c r="G14" t="n">
-        <v>0.19</v>
+        <v>0.233</v>
       </c>
       <c r="H14" t="n">
-        <v>0.365</v>
+        <v>0.348</v>
       </c>
       <c r="I14" t="n">
-        <v>0.959</v>
+        <v>0.752</v>
       </c>
       <c r="J14" t="n">
-        <v>7.337000000000001</v>
+        <v>6.79</v>
       </c>
       <c r="K14" t="n">
-        <v>8.116</v>
+        <v>11.869</v>
       </c>
       <c r="L14" t="n">
-        <v>11.578</v>
+        <v>10.652</v>
       </c>
       <c r="M14" t="n">
-        <v>13.522</v>
+        <v>12.828</v>
       </c>
       <c r="N14" t="n">
-        <v>10.529</v>
+        <v>9.763</v>
       </c>
       <c r="O14" t="n">
-        <v>4.813</v>
+        <v>10.403</v>
       </c>
       <c r="P14" t="n">
-        <v>8.619</v>
+        <v>4.673999999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.718</v>
+        <v>4.524</v>
       </c>
       <c r="R14" t="n">
-        <v>5.852</v>
+        <v>4.786</v>
       </c>
       <c r="S14" t="n">
-        <v>6.146</v>
+        <v>6.339</v>
       </c>
       <c r="T14" t="n">
-        <v>6.096</v>
+        <v>6.002</v>
       </c>
       <c r="U14" t="n">
-        <v>10.369</v>
+        <v>9.711</v>
       </c>
     </row>
     <row r="15">
@@ -1377,61 +1377,61 @@
         <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>0.135</v>
+        <v>0.003</v>
       </c>
       <c r="D15" t="n">
-        <v>0.044</v>
+        <v>0.055</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.107</v>
+        <v>0.037</v>
       </c>
       <c r="G15" t="n">
-        <v>0.095</v>
+        <v>0.101</v>
       </c>
       <c r="H15" t="n">
-        <v>0.193</v>
+        <v>0.123</v>
       </c>
       <c r="I15" t="n">
-        <v>0.451</v>
+        <v>0.35</v>
       </c>
       <c r="J15" t="n">
-        <v>4.923</v>
+        <v>4.434</v>
       </c>
       <c r="K15" t="n">
-        <v>5.278</v>
+        <v>8.782</v>
       </c>
       <c r="L15" t="n">
-        <v>9.120000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="M15" t="n">
-        <v>11.985</v>
+        <v>11.328</v>
       </c>
       <c r="N15" t="n">
-        <v>11.911</v>
+        <v>11.256</v>
       </c>
       <c r="O15" t="n">
-        <v>6.589</v>
+        <v>11.37</v>
       </c>
       <c r="P15" t="n">
-        <v>10.959</v>
+        <v>6.587999999999999</v>
       </c>
       <c r="Q15" t="n">
-        <v>6.497999999999999</v>
+        <v>6.786</v>
       </c>
       <c r="R15" t="n">
-        <v>7.542999999999999</v>
+        <v>6.457</v>
       </c>
       <c r="S15" t="n">
-        <v>8.015000000000001</v>
+        <v>8.028</v>
       </c>
       <c r="T15" t="n">
-        <v>7.988</v>
+        <v>7.836</v>
       </c>
       <c r="U15" t="n">
-        <v>8.166</v>
+        <v>7.965999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -1442,61 +1442,61 @@
         <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>0.037</v>
+        <v>0.001</v>
       </c>
       <c r="D16" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.011</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0.026</v>
+        <v>0.005</v>
       </c>
       <c r="G16" t="n">
-        <v>0.031</v>
+        <v>0.039</v>
       </c>
       <c r="H16" t="n">
-        <v>0.08</v>
+        <v>0.065</v>
       </c>
       <c r="I16" t="n">
-        <v>0.215</v>
+        <v>0.177</v>
       </c>
       <c r="J16" t="n">
-        <v>2.942</v>
+        <v>2.917</v>
       </c>
       <c r="K16" t="n">
-        <v>3.387</v>
+        <v>6.281000000000001</v>
       </c>
       <c r="L16" t="n">
-        <v>6.793</v>
+        <v>6.462</v>
       </c>
       <c r="M16" t="n">
-        <v>9.718999999999999</v>
+        <v>9.309000000000001</v>
       </c>
       <c r="N16" t="n">
-        <v>12.3</v>
+        <v>11.872</v>
       </c>
       <c r="O16" t="n">
-        <v>8.591999999999999</v>
+        <v>11.698</v>
       </c>
       <c r="P16" t="n">
-        <v>12.185</v>
+        <v>8.583</v>
       </c>
       <c r="Q16" t="n">
-        <v>8.486000000000001</v>
+        <v>9.284000000000001</v>
       </c>
       <c r="R16" t="n">
-        <v>9.216000000000001</v>
+        <v>8.513999999999999</v>
       </c>
       <c r="S16" t="n">
-        <v>9.854000000000001</v>
+        <v>9.276</v>
       </c>
       <c r="T16" t="n">
-        <v>9.415999999999999</v>
+        <v>9.347</v>
       </c>
       <c r="U16" t="n">
-        <v>6.714</v>
+        <v>6.159</v>
       </c>
     </row>
     <row r="17">
@@ -1507,61 +1507,61 @@
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>0.014</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.002</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0.013</v>
+        <v>0.001</v>
       </c>
       <c r="G17" t="n">
-        <v>0.006</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>0.021</v>
+        <v>0.019</v>
       </c>
       <c r="I17" t="n">
         <v>0.07200000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>1.752</v>
+        <v>1.781</v>
       </c>
       <c r="K17" t="n">
-        <v>1.951</v>
+        <v>4.181</v>
       </c>
       <c r="L17" t="n">
-        <v>4.917</v>
+        <v>4.682</v>
       </c>
       <c r="M17" t="n">
-        <v>7.829999999999999</v>
+        <v>7.500999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>11.595</v>
+        <v>12.1</v>
       </c>
       <c r="O17" t="n">
-        <v>10.813</v>
+        <v>11.091</v>
       </c>
       <c r="P17" t="n">
-        <v>12.549</v>
+        <v>10.601</v>
       </c>
       <c r="Q17" t="n">
-        <v>10.707</v>
+        <v>11.572</v>
       </c>
       <c r="R17" t="n">
-        <v>10.903</v>
+        <v>10.424</v>
       </c>
       <c r="S17" t="n">
-        <v>11.109</v>
+        <v>10.685</v>
       </c>
       <c r="T17" t="n">
-        <v>10.956</v>
+        <v>10.607</v>
       </c>
       <c r="U17" t="n">
-        <v>4.784999999999999</v>
+        <v>4.672</v>
       </c>
     </row>
     <row r="18">
@@ -1572,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0.001</v>
@@ -1581,52 +1581,52 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G18" t="n">
         <v>0.003</v>
       </c>
       <c r="H18" t="n">
-        <v>0.004</v>
+        <v>0.008</v>
       </c>
       <c r="I18" t="n">
-        <v>0.024</v>
+        <v>0.02</v>
       </c>
       <c r="J18" t="n">
-        <v>0.984</v>
+        <v>1.003</v>
       </c>
       <c r="K18" t="n">
-        <v>1.063</v>
+        <v>2.656</v>
       </c>
       <c r="L18" t="n">
-        <v>3.293</v>
+        <v>3.409</v>
       </c>
       <c r="M18" t="n">
-        <v>5.776</v>
+        <v>5.765</v>
       </c>
       <c r="N18" t="n">
-        <v>10.344</v>
+        <v>11.442</v>
       </c>
       <c r="O18" t="n">
-        <v>13.154</v>
+        <v>10.226</v>
       </c>
       <c r="P18" t="n">
-        <v>12.286</v>
+        <v>12.544</v>
       </c>
       <c r="Q18" t="n">
-        <v>12.825</v>
+        <v>13.631</v>
       </c>
       <c r="R18" t="n">
-        <v>12.312</v>
+        <v>12.378</v>
       </c>
       <c r="S18" t="n">
-        <v>12.294</v>
+        <v>11.88</v>
       </c>
       <c r="T18" t="n">
-        <v>12.029</v>
+        <v>11.598</v>
       </c>
       <c r="U18" t="n">
-        <v>3.602</v>
+        <v>3.435</v>
       </c>
     </row>
     <row r="19">
@@ -1652,46 +1652,46 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="I19" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="J19" t="n">
-        <v>0.454</v>
+        <v>0.4969999999999999</v>
       </c>
       <c r="K19" t="n">
-        <v>0.553</v>
+        <v>1.475</v>
       </c>
       <c r="L19" t="n">
-        <v>2.172</v>
+        <v>2.093</v>
       </c>
       <c r="M19" t="n">
-        <v>4.233</v>
+        <v>4.157</v>
       </c>
       <c r="N19" t="n">
-        <v>8.853999999999999</v>
+        <v>10.181</v>
       </c>
       <c r="O19" t="n">
-        <v>15.113</v>
+        <v>9.138</v>
       </c>
       <c r="P19" t="n">
-        <v>11.192</v>
+        <v>14.857</v>
       </c>
       <c r="Q19" t="n">
-        <v>14.903</v>
+        <v>15.101</v>
       </c>
       <c r="R19" t="n">
-        <v>13.924</v>
+        <v>14.313</v>
       </c>
       <c r="S19" t="n">
-        <v>12.985</v>
+        <v>12.87</v>
       </c>
       <c r="T19" t="n">
-        <v>13.158</v>
+        <v>12.848</v>
       </c>
       <c r="U19" t="n">
-        <v>2.45</v>
+        <v>2.459</v>
       </c>
     </row>
     <row r="20">
@@ -1711,7 +1711,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -1720,43 +1720,43 @@
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="J20" t="n">
-        <v>0.214</v>
+        <v>0.194</v>
       </c>
       <c r="K20" t="n">
-        <v>0.216</v>
+        <v>0.734</v>
       </c>
       <c r="L20" t="n">
-        <v>1.238</v>
+        <v>1.299</v>
       </c>
       <c r="M20" t="n">
-        <v>2.821</v>
+        <v>2.672</v>
       </c>
       <c r="N20" t="n">
-        <v>7.037</v>
+        <v>8.031000000000001</v>
       </c>
       <c r="O20" t="n">
-        <v>16.9</v>
+        <v>7.504</v>
       </c>
       <c r="P20" t="n">
-        <v>10.303</v>
+        <v>16.888</v>
       </c>
       <c r="Q20" t="n">
-        <v>16.646</v>
+        <v>16.304</v>
       </c>
       <c r="R20" t="n">
-        <v>14.799</v>
+        <v>16.439</v>
       </c>
       <c r="S20" t="n">
-        <v>14.053</v>
+        <v>14.251</v>
       </c>
       <c r="T20" t="n">
-        <v>14.182</v>
+        <v>14.101</v>
       </c>
       <c r="U20" t="n">
-        <v>1.587</v>
+        <v>1.578</v>
       </c>
     </row>
     <row r="21">
@@ -1788,40 +1788,40 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0.052</v>
+        <v>0.045</v>
       </c>
       <c r="K21" t="n">
-        <v>0.059</v>
+        <v>0.226</v>
       </c>
       <c r="L21" t="n">
-        <v>0.526</v>
+        <v>0.544</v>
       </c>
       <c r="M21" t="n">
-        <v>1.359</v>
+        <v>1.34</v>
       </c>
       <c r="N21" t="n">
-        <v>5.061</v>
+        <v>4.662</v>
       </c>
       <c r="O21" t="n">
-        <v>17.567</v>
+        <v>5.023</v>
       </c>
       <c r="P21" t="n">
-        <v>8.512</v>
+        <v>18.372</v>
       </c>
       <c r="Q21" t="n">
-        <v>18.487</v>
+        <v>17.554</v>
       </c>
       <c r="R21" t="n">
-        <v>15.977</v>
+        <v>19.157</v>
       </c>
       <c r="S21" t="n">
-        <v>15.179</v>
+        <v>15.074</v>
       </c>
       <c r="T21" t="n">
-        <v>16.371</v>
+        <v>17.125</v>
       </c>
       <c r="U21" t="n">
-        <v>0.8500000000000001</v>
+        <v>0.878</v>
       </c>
     </row>
   </sheetData>
@@ -1857,7 +1857,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99.88300000000001</v>
+        <v>99.869</v>
       </c>
     </row>
     <row r="3">
@@ -1867,27 +1867,27 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.85799999999999</v>
+        <v>99.815</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Independiente Medellín</t>
+          <t>Atlético Bucaramanga</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>92.435</v>
+        <v>97.91500000000002</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Atlético Bucaramanga</t>
+          <t>Independiente Medellín</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>91.13900000000001</v>
+        <v>93.03</v>
       </c>
     </row>
     <row r="6">
@@ -1897,27 +1897,27 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>88.68299999999999</v>
+        <v>88.875</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>85.215</v>
+        <v>86.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Millonarios</t>
+          <t>Deportes Tolima</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>81.107</v>
+        <v>85.84899999999999</v>
       </c>
     </row>
     <row r="9">
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>76.63499999999999</v>
+        <v>76.827</v>
       </c>
     </row>
     <row r="10">
@@ -1937,37 +1937,37 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>26.56</v>
+        <v>26.599</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Once Caldas</t>
+          <t>Junior</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>23.25</v>
+        <v>14.261</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>Águilas Doradas</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>14.15</v>
+        <v>11.924</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Águilas Doradas</t>
+          <t>Once Caldas</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>12.252</v>
+        <v>9.208</v>
       </c>
     </row>
     <row r="14">
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4.885000000000001</v>
+        <v>4.631</v>
       </c>
     </row>
     <row r="15">
@@ -1987,17 +1987,17 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.435</v>
+        <v>1.498</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Deportivo Pasto</t>
+          <t>Boyacá Chicó</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.5630000000000001</v>
+        <v>1.296</v>
       </c>
     </row>
     <row r="17">
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.5449999999999999</v>
+        <v>0.608</v>
       </c>
     </row>
     <row r="18">
@@ -2017,17 +2017,17 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.504</v>
+        <v>0.5239999999999999</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Boyacá Chicó</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.439</v>
+        <v>0.244</v>
       </c>
     </row>
     <row r="20">
@@ -2037,17 +2037,17 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.24</v>
+        <v>0.243</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Deportivo Pasto</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.222</v>
+        <v>0.08400000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar resultados de Finalizacion 2026-II hasta el 27/09/2026
- Carga 6 partidos jugados el 26 y 27 de septiembre (Deportivo
  Pereira 0-0 Internacional de Bogota, Cucuta Deportivo 2-1
  Llaneros, Junior 2-0 Independiente Medellin, Deportivo Cali 2-0
  Aguilas Doradas, Jaguares 1-2 Alianza Valledupar, Fortaleza 2-2
  Deportes Tolima) con actualizar_resultados.py.
- Tabla.csv/Partidos.csv/Historial_partidos.csv actualizados;
  historial pasa de 755 a 761 partidos. Tabla verificada contra
  Dimayor en vivo. Deportivo Cali sube al 2 puesto.
- model_params.csv: DrawBias recalibrado exacto (224/761).
- Resultados.xlsx/Resultado.png regenerados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resultados.xlsx
+++ b/Resultados.xlsx
@@ -430,29 +430,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Deportivo Cali</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Atlético Bucaramanga</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Millonarios</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Atlético Nacional</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Independiente Medellín</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Deportivo Cali</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>Deportes Tolima</t>
@@ -475,52 +475,52 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>Internacional de Bogotá</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Cúcuta Deportivo</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>Águilas Doradas</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Internacional de Bogotá</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Boyacá Chicó</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Cúcuta Deportivo</t>
-        </is>
-      </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>Alianza Valledupar</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>Fortaleza</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Deportivo Pereira</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
         <is>
           <t>Deportivo Pasto</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Alianza Valledupar</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Deportivo Pereira</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Jaguares</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Junior</t>
         </is>
       </c>
     </row>
@@ -529,43 +529,43 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>33.813</v>
+        <v>35.036</v>
       </c>
       <c r="C2" t="n">
-        <v>11.193</v>
+        <v>3.864</v>
       </c>
       <c r="D2" t="n">
-        <v>0.641</v>
+        <v>11.71</v>
       </c>
       <c r="E2" t="n">
-        <v>44.843</v>
+        <v>0.629</v>
       </c>
       <c r="F2" t="n">
-        <v>5.396999999999999</v>
+        <v>44.91</v>
       </c>
       <c r="G2" t="n">
-        <v>2.005</v>
+        <v>2.343</v>
       </c>
       <c r="H2" t="n">
-        <v>1.41</v>
+        <v>0.7230000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>0.6629999999999999</v>
+        <v>0.763</v>
       </c>
       <c r="J2" t="n">
-        <v>0.021</v>
+        <v>0.001</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>0.006999999999999999</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -574,19 +574,19 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>0.006</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -594,43 +594,43 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>31.403</v>
+        <v>31.784</v>
       </c>
       <c r="C3" t="n">
-        <v>16.958</v>
+        <v>9.596</v>
       </c>
       <c r="D3" t="n">
-        <v>2.578</v>
+        <v>17.202</v>
       </c>
       <c r="E3" t="n">
-        <v>27.261</v>
+        <v>2.813</v>
       </c>
       <c r="F3" t="n">
-        <v>9.653</v>
+        <v>27.695</v>
       </c>
       <c r="G3" t="n">
-        <v>5.503</v>
+        <v>5.595</v>
       </c>
       <c r="H3" t="n">
-        <v>4.059</v>
+        <v>2.759</v>
       </c>
       <c r="I3" t="n">
-        <v>2.369</v>
+        <v>2.427</v>
       </c>
       <c r="J3" t="n">
-        <v>0.137</v>
+        <v>0.021</v>
       </c>
       <c r="K3" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="L3" t="n">
-        <v>0.028</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -639,19 +639,19 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>0.096</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0.046</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -659,52 +659,52 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>16.397</v>
+        <v>16.05</v>
       </c>
       <c r="C4" t="n">
-        <v>22.234</v>
+        <v>17.234</v>
       </c>
       <c r="D4" t="n">
-        <v>7.041</v>
+        <v>22.579</v>
       </c>
       <c r="E4" t="n">
-        <v>13.16</v>
+        <v>6.914</v>
       </c>
       <c r="F4" t="n">
-        <v>15.068</v>
+        <v>13.151</v>
       </c>
       <c r="G4" t="n">
-        <v>11.022</v>
+        <v>10.405</v>
       </c>
       <c r="H4" t="n">
-        <v>8.584999999999999</v>
+        <v>6.977</v>
       </c>
       <c r="I4" t="n">
-        <v>5.606</v>
+        <v>6.066</v>
       </c>
       <c r="J4" t="n">
-        <v>0.453</v>
+        <v>0.116</v>
       </c>
       <c r="K4" t="n">
         <v>0.039</v>
       </c>
       <c r="L4" t="n">
-        <v>0.178</v>
+        <v>0.003</v>
       </c>
       <c r="M4" t="n">
-        <v>0.016</v>
+        <v>0.004</v>
       </c>
       <c r="N4" t="n">
-        <v>0.003</v>
+        <v>0.034</v>
       </c>
       <c r="O4" t="n">
-        <v>0.003</v>
+        <v>0.006</v>
       </c>
       <c r="P4" t="n">
         <v>0.001</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>0.421</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -713,10 +713,10 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>0.193</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -724,64 +724,64 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>9.098000000000001</v>
+        <v>8.598000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>17.427</v>
+        <v>19.037</v>
       </c>
       <c r="D5" t="n">
-        <v>11.538</v>
+        <v>17.363</v>
       </c>
       <c r="E5" t="n">
-        <v>7.238</v>
+        <v>11.929</v>
       </c>
       <c r="F5" t="n">
-        <v>16.697</v>
+        <v>6.815</v>
       </c>
       <c r="G5" t="n">
-        <v>14.668</v>
+        <v>14.197</v>
       </c>
       <c r="H5" t="n">
-        <v>12.513</v>
+        <v>11.066</v>
       </c>
       <c r="I5" t="n">
-        <v>8.554</v>
+        <v>9.198</v>
       </c>
       <c r="J5" t="n">
-        <v>1.164</v>
+        <v>0.382</v>
       </c>
       <c r="K5" t="n">
-        <v>0.132</v>
+        <v>0.155</v>
       </c>
       <c r="L5" t="n">
-        <v>0.399</v>
+        <v>0.018</v>
       </c>
       <c r="M5" t="n">
-        <v>0.055</v>
+        <v>0.033</v>
       </c>
       <c r="N5" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="O5" t="n">
         <v>0.01</v>
       </c>
-      <c r="O5" t="n">
-        <v>0.008</v>
-      </c>
       <c r="P5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>1.054</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>0.005</v>
+        <v>0.001</v>
       </c>
       <c r="T5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="U5" t="n">
-        <v>0.49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -789,64 +789,64 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>4.853</v>
+        <v>4.557</v>
       </c>
       <c r="C6" t="n">
-        <v>12.756</v>
+        <v>16.975</v>
       </c>
       <c r="D6" t="n">
-        <v>15.141</v>
+        <v>12.521</v>
       </c>
       <c r="E6" t="n">
-        <v>3.889</v>
+        <v>15.778</v>
       </c>
       <c r="F6" t="n">
-        <v>15.24</v>
+        <v>3.752</v>
       </c>
       <c r="G6" t="n">
-        <v>16.189</v>
+        <v>15.803</v>
       </c>
       <c r="H6" t="n">
-        <v>14.964</v>
+        <v>14.421</v>
       </c>
       <c r="I6" t="n">
-        <v>11.937</v>
+        <v>12.152</v>
       </c>
       <c r="J6" t="n">
-        <v>2.36</v>
+        <v>0.947</v>
       </c>
       <c r="K6" t="n">
-        <v>0.414</v>
+        <v>0.43</v>
       </c>
       <c r="L6" t="n">
-        <v>0.9209999999999999</v>
+        <v>0.08099999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>0.177</v>
+        <v>0.08099999999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>0.038</v>
+        <v>0.34</v>
       </c>
       <c r="O6" t="n">
-        <v>0.02</v>
+        <v>0.037</v>
       </c>
       <c r="P6" t="n">
-        <v>0.004</v>
+        <v>0.026</v>
       </c>
       <c r="Q6" t="n">
+        <v>2.085</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="U6" t="n">
         <v>0.002</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="U6" t="n">
-        <v>1.055</v>
       </c>
     </row>
     <row r="7">
@@ -854,64 +854,64 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>2.676</v>
+        <v>2.42</v>
       </c>
       <c r="C7" t="n">
-        <v>8.593</v>
+        <v>13.455</v>
       </c>
       <c r="D7" t="n">
-        <v>17.704</v>
+        <v>8.364000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>2.011</v>
+        <v>17.888</v>
       </c>
       <c r="F7" t="n">
-        <v>13.142</v>
+        <v>1.999</v>
       </c>
       <c r="G7" t="n">
-        <v>15.679</v>
+        <v>15.576</v>
       </c>
       <c r="H7" t="n">
-        <v>15.835</v>
+        <v>16.71</v>
       </c>
       <c r="I7" t="n">
-        <v>14.532</v>
+        <v>15.07</v>
       </c>
       <c r="J7" t="n">
-        <v>4.105</v>
+        <v>1.947</v>
       </c>
       <c r="K7" t="n">
-        <v>1.04</v>
+        <v>1.188</v>
       </c>
       <c r="L7" t="n">
-        <v>1.717</v>
+        <v>0.305</v>
       </c>
       <c r="M7" t="n">
-        <v>0.483</v>
+        <v>0.323</v>
       </c>
       <c r="N7" t="n">
-        <v>0.113</v>
+        <v>0.786</v>
       </c>
       <c r="O7" t="n">
-        <v>0.128</v>
+        <v>0.107</v>
       </c>
       <c r="P7" t="n">
-        <v>0.013</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="Q7" t="n">
+        <v>3.736</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="T7" t="n">
         <v>0.004</v>
       </c>
-      <c r="R7" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.059</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0.048</v>
-      </c>
       <c r="U7" t="n">
-        <v>2.104</v>
+        <v>0.006999999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -919,64 +919,64 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>1.202</v>
+        <v>1.047</v>
       </c>
       <c r="C8" t="n">
-        <v>5.571000000000001</v>
+        <v>9.395000000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>17.714</v>
+        <v>5.399</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9740000000000001</v>
+        <v>17.504</v>
       </c>
       <c r="F8" t="n">
-        <v>10.309</v>
+        <v>1.021</v>
       </c>
       <c r="G8" t="n">
-        <v>13.631</v>
+        <v>14.011</v>
       </c>
       <c r="H8" t="n">
-        <v>15.368</v>
+        <v>17.346</v>
       </c>
       <c r="I8" t="n">
-        <v>16.861</v>
+        <v>17.01</v>
       </c>
       <c r="J8" t="n">
-        <v>6.987</v>
+        <v>4.101</v>
       </c>
       <c r="K8" t="n">
-        <v>2.415</v>
+        <v>2.524</v>
       </c>
       <c r="L8" t="n">
-        <v>3.047</v>
+        <v>0.826</v>
       </c>
       <c r="M8" t="n">
-        <v>1.224</v>
+        <v>0.869</v>
       </c>
       <c r="N8" t="n">
-        <v>0.304</v>
+        <v>1.782</v>
       </c>
       <c r="O8" t="n">
-        <v>0.322</v>
+        <v>0.303</v>
       </c>
       <c r="P8" t="n">
-        <v>0.046</v>
+        <v>0.239</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.019</v>
+        <v>6.465</v>
       </c>
       <c r="R8" t="n">
-        <v>0.064</v>
+        <v>0.039</v>
       </c>
       <c r="S8" t="n">
-        <v>0.135</v>
+        <v>0.093</v>
       </c>
       <c r="T8" t="n">
-        <v>0.112</v>
+        <v>0.016</v>
       </c>
       <c r="U8" t="n">
-        <v>3.695</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="9">
@@ -984,64 +984,64 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.427</v>
+        <v>0.397</v>
       </c>
       <c r="C9" t="n">
-        <v>3.183</v>
+        <v>6.039</v>
       </c>
       <c r="D9" t="n">
-        <v>14.343</v>
+        <v>2.991</v>
       </c>
       <c r="E9" t="n">
-        <v>0.439</v>
+        <v>13.914</v>
       </c>
       <c r="F9" t="n">
-        <v>7.524</v>
+        <v>0.459</v>
       </c>
       <c r="G9" t="n">
-        <v>10.178</v>
+        <v>11.036</v>
       </c>
       <c r="H9" t="n">
-        <v>13.115</v>
+        <v>14.766</v>
       </c>
       <c r="I9" t="n">
-        <v>16.305</v>
+        <v>16.064</v>
       </c>
       <c r="J9" t="n">
-        <v>11.372</v>
+        <v>7.675999999999999</v>
       </c>
       <c r="K9" t="n">
-        <v>5.165</v>
+        <v>5.564</v>
       </c>
       <c r="L9" t="n">
-        <v>5.627</v>
+        <v>2.201</v>
       </c>
       <c r="M9" t="n">
-        <v>2.675</v>
+        <v>2.199</v>
       </c>
       <c r="N9" t="n">
-        <v>0.828</v>
+        <v>3.645</v>
       </c>
       <c r="O9" t="n">
-        <v>1.017</v>
+        <v>0.8880000000000001</v>
       </c>
       <c r="P9" t="n">
-        <v>0.178</v>
+        <v>0.6819999999999999</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.059</v>
+        <v>10.97</v>
       </c>
       <c r="R9" t="n">
-        <v>0.161</v>
+        <v>0.119</v>
       </c>
       <c r="S9" t="n">
-        <v>0.385</v>
+        <v>0.253</v>
       </c>
       <c r="T9" t="n">
-        <v>0.347</v>
+        <v>0.08</v>
       </c>
       <c r="U9" t="n">
-        <v>6.672000000000001</v>
+        <v>0.057</v>
       </c>
     </row>
     <row r="10">
@@ -1049,64 +1049,64 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.11</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="C10" t="n">
-        <v>1.353</v>
+        <v>2.877</v>
       </c>
       <c r="D10" t="n">
-        <v>7.76</v>
+        <v>1.218</v>
       </c>
       <c r="E10" t="n">
-        <v>0.133</v>
+        <v>7.309</v>
       </c>
       <c r="F10" t="n">
-        <v>3.967</v>
+        <v>0.148</v>
       </c>
       <c r="G10" t="n">
-        <v>5.847</v>
+        <v>5.970000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>7.317</v>
+        <v>8.347</v>
       </c>
       <c r="I10" t="n">
-        <v>10.822</v>
+        <v>10.166</v>
       </c>
       <c r="J10" t="n">
-        <v>17.358</v>
+        <v>13.298</v>
       </c>
       <c r="K10" t="n">
-        <v>10.375</v>
+        <v>10.934</v>
       </c>
       <c r="L10" t="n">
-        <v>10.274</v>
+        <v>4.913</v>
       </c>
       <c r="M10" t="n">
-        <v>5.93</v>
+        <v>5.101</v>
       </c>
       <c r="N10" t="n">
-        <v>1.924</v>
+        <v>7.339</v>
       </c>
       <c r="O10" t="n">
-        <v>2.469</v>
+        <v>2.176</v>
       </c>
       <c r="P10" t="n">
-        <v>0.4329999999999999</v>
+        <v>1.886</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.251</v>
+        <v>16.812</v>
       </c>
       <c r="R10" t="n">
-        <v>0.569</v>
+        <v>0.314</v>
       </c>
       <c r="S10" t="n">
-        <v>1.07</v>
+        <v>0.666</v>
       </c>
       <c r="T10" t="n">
-        <v>0.856</v>
+        <v>0.239</v>
       </c>
       <c r="U10" t="n">
-        <v>11.182</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11">
@@ -1114,64 +1114,64 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.02</v>
+        <v>0.024</v>
       </c>
       <c r="C11" t="n">
-        <v>0.49</v>
+        <v>1.016</v>
       </c>
       <c r="D11" t="n">
-        <v>3.363</v>
+        <v>0.4420000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>0.036</v>
+        <v>3.328</v>
       </c>
       <c r="F11" t="n">
-        <v>1.758</v>
+        <v>0.035</v>
       </c>
       <c r="G11" t="n">
-        <v>2.998</v>
+        <v>2.824</v>
       </c>
       <c r="H11" t="n">
-        <v>3.786</v>
+        <v>3.872</v>
       </c>
       <c r="I11" t="n">
-        <v>6.078</v>
+        <v>5.416</v>
       </c>
       <c r="J11" t="n">
-        <v>16.216</v>
+        <v>15.722</v>
       </c>
       <c r="K11" t="n">
-        <v>14.411</v>
+        <v>14.836</v>
       </c>
       <c r="L11" t="n">
-        <v>13.356</v>
+        <v>8.121</v>
       </c>
       <c r="M11" t="n">
-        <v>9.438000000000001</v>
+        <v>8.142000000000001</v>
       </c>
       <c r="N11" t="n">
-        <v>3.758</v>
+        <v>10.325</v>
       </c>
       <c r="O11" t="n">
-        <v>4.464</v>
+        <v>3.795</v>
       </c>
       <c r="P11" t="n">
-        <v>1.009</v>
+        <v>3.499</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.657</v>
+        <v>15.115</v>
       </c>
       <c r="R11" t="n">
-        <v>1.224</v>
+        <v>0.8580000000000001</v>
       </c>
       <c r="S11" t="n">
-        <v>1.963</v>
+        <v>1.458</v>
       </c>
       <c r="T11" t="n">
-        <v>1.778</v>
+        <v>0.698</v>
       </c>
       <c r="U11" t="n">
-        <v>13.197</v>
+        <v>0.474</v>
       </c>
     </row>
     <row r="12">
@@ -1179,64 +1179,64 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0.17</v>
+        <v>0.363</v>
       </c>
       <c r="D12" t="n">
-        <v>1.381</v>
+        <v>0.146</v>
       </c>
       <c r="E12" t="n">
-        <v>0.013</v>
+        <v>1.305</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7979999999999999</v>
+        <v>0.011</v>
       </c>
       <c r="G12" t="n">
-        <v>1.313</v>
+        <v>1.309</v>
       </c>
       <c r="H12" t="n">
+        <v>1.746</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2.826</v>
+      </c>
+      <c r="J12" t="n">
+        <v>14.754</v>
+      </c>
+      <c r="K12" t="n">
+        <v>14.865</v>
+      </c>
+      <c r="L12" t="n">
+        <v>10.727</v>
+      </c>
+      <c r="M12" t="n">
+        <v>10.537</v>
+      </c>
+      <c r="N12" t="n">
+        <v>11.954</v>
+      </c>
+      <c r="O12" t="n">
+        <v>5.587000000000001</v>
+      </c>
+      <c r="P12" t="n">
+        <v>5.437</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>12.002</v>
+      </c>
+      <c r="R12" t="n">
         <v>1.706</v>
       </c>
-      <c r="I12" t="n">
-        <v>3.223</v>
-      </c>
-      <c r="J12" t="n">
-        <v>12.672</v>
-      </c>
-      <c r="K12" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="L12" t="n">
-        <v>14.07</v>
-      </c>
-      <c r="M12" t="n">
-        <v>12.015</v>
-      </c>
-      <c r="N12" t="n">
-        <v>5.865</v>
-      </c>
-      <c r="O12" t="n">
-        <v>6.504</v>
-      </c>
-      <c r="P12" t="n">
-        <v>1.944</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>1.518</v>
-      </c>
-      <c r="R12" t="n">
-        <v>2.141</v>
-      </c>
       <c r="S12" t="n">
-        <v>3.266</v>
+        <v>2.442</v>
       </c>
       <c r="T12" t="n">
-        <v>2.935</v>
+        <v>1.403</v>
       </c>
       <c r="U12" t="n">
-        <v>12.865</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="13">
@@ -1247,61 +1247,61 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.055</v>
+        <v>0.105</v>
       </c>
       <c r="D13" t="n">
-        <v>0.5309999999999999</v>
+        <v>0.04</v>
       </c>
       <c r="E13" t="n">
+        <v>0.453</v>
+      </c>
+      <c r="F13" t="n">
         <v>0.003</v>
       </c>
-      <c r="F13" t="n">
-        <v>0.286</v>
-      </c>
       <c r="G13" t="n">
-        <v>0.582</v>
+        <v>0.584</v>
       </c>
       <c r="H13" t="n">
-        <v>0.7779999999999999</v>
+        <v>0.772</v>
       </c>
       <c r="I13" t="n">
-        <v>1.664</v>
+        <v>1.468</v>
       </c>
       <c r="J13" t="n">
-        <v>9.494</v>
+        <v>12.211</v>
       </c>
       <c r="K13" t="n">
-        <v>14.202</v>
+        <v>13.363</v>
       </c>
       <c r="L13" t="n">
-        <v>12.735</v>
+        <v>12.331</v>
       </c>
       <c r="M13" t="n">
-        <v>13.086</v>
+        <v>12.168</v>
       </c>
       <c r="N13" t="n">
-        <v>7.85</v>
+        <v>12.242</v>
       </c>
       <c r="O13" t="n">
-        <v>8.612</v>
+        <v>7.431</v>
       </c>
       <c r="P13" t="n">
-        <v>3.263</v>
+        <v>7.152</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.734</v>
+        <v>9.236000000000001</v>
       </c>
       <c r="R13" t="n">
-        <v>3.355</v>
+        <v>2.745</v>
       </c>
       <c r="S13" t="n">
-        <v>4.69</v>
+        <v>3.704</v>
       </c>
       <c r="T13" t="n">
-        <v>4.443</v>
+        <v>2.422</v>
       </c>
       <c r="U13" t="n">
-        <v>11.637</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="14">
@@ -1312,61 +1312,61 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0.013</v>
+        <v>0.033</v>
       </c>
       <c r="D14" t="n">
-        <v>0.196</v>
+        <v>0.015</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>0.167</v>
       </c>
       <c r="F14" t="n">
-        <v>0.117</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0.233</v>
+        <v>0.222</v>
       </c>
       <c r="H14" t="n">
-        <v>0.348</v>
+        <v>0.291</v>
       </c>
       <c r="I14" t="n">
-        <v>0.752</v>
+        <v>0.734</v>
       </c>
       <c r="J14" t="n">
-        <v>6.79</v>
+        <v>9.823</v>
       </c>
       <c r="K14" t="n">
-        <v>11.869</v>
+        <v>11.072</v>
       </c>
       <c r="L14" t="n">
-        <v>10.652</v>
+        <v>12.776</v>
       </c>
       <c r="M14" t="n">
-        <v>12.828</v>
+        <v>12.49</v>
       </c>
       <c r="N14" t="n">
-        <v>9.763</v>
+        <v>11.716</v>
       </c>
       <c r="O14" t="n">
-        <v>10.403</v>
+        <v>8.824</v>
       </c>
       <c r="P14" t="n">
-        <v>4.673999999999999</v>
+        <v>8.998000000000001</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.524</v>
+        <v>6.920999999999999</v>
       </c>
       <c r="R14" t="n">
-        <v>4.786</v>
+        <v>4.302</v>
       </c>
       <c r="S14" t="n">
-        <v>6.339</v>
+        <v>5.192</v>
       </c>
       <c r="T14" t="n">
-        <v>6.002</v>
+        <v>3.984999999999999</v>
       </c>
       <c r="U14" t="n">
-        <v>9.711</v>
+        <v>2.439</v>
       </c>
     </row>
     <row r="15">
@@ -1377,61 +1377,61 @@
         <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>0.003</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="D15" t="n">
-        <v>0.055</v>
+        <v>0.008</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>0.052</v>
       </c>
       <c r="F15" t="n">
-        <v>0.037</v>
+        <v>0.001</v>
       </c>
       <c r="G15" t="n">
-        <v>0.101</v>
+        <v>0.082</v>
       </c>
       <c r="H15" t="n">
-        <v>0.123</v>
+        <v>0.134</v>
       </c>
       <c r="I15" t="n">
-        <v>0.35</v>
+        <v>0.379</v>
       </c>
       <c r="J15" t="n">
-        <v>4.434</v>
+        <v>7.063</v>
       </c>
       <c r="K15" t="n">
-        <v>8.782</v>
+        <v>8.702999999999999</v>
       </c>
       <c r="L15" t="n">
-        <v>8.5</v>
+        <v>12.157</v>
       </c>
       <c r="M15" t="n">
-        <v>11.328</v>
+        <v>12.019</v>
       </c>
       <c r="N15" t="n">
-        <v>11.256</v>
+        <v>10.56</v>
       </c>
       <c r="O15" t="n">
-        <v>11.37</v>
+        <v>10.103</v>
       </c>
       <c r="P15" t="n">
-        <v>6.587999999999999</v>
+        <v>10.942</v>
       </c>
       <c r="Q15" t="n">
-        <v>6.786</v>
+        <v>5.325</v>
       </c>
       <c r="R15" t="n">
-        <v>6.457</v>
+        <v>6.005</v>
       </c>
       <c r="S15" t="n">
-        <v>8.028</v>
+        <v>6.827</v>
       </c>
       <c r="T15" t="n">
-        <v>7.836</v>
+        <v>5.96</v>
       </c>
       <c r="U15" t="n">
-        <v>7.965999999999999</v>
+        <v>3.671</v>
       </c>
     </row>
     <row r="16">
@@ -1445,58 +1445,58 @@
         <v>0.001</v>
       </c>
       <c r="D16" t="n">
-        <v>0.011</v>
+        <v>0.002</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>0.013</v>
       </c>
       <c r="F16" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>0.039</v>
+        <v>0.031</v>
       </c>
       <c r="H16" t="n">
-        <v>0.065</v>
+        <v>0.045</v>
       </c>
       <c r="I16" t="n">
-        <v>0.177</v>
+        <v>0.158</v>
       </c>
       <c r="J16" t="n">
-        <v>2.917</v>
+        <v>5.043</v>
       </c>
       <c r="K16" t="n">
-        <v>6.281000000000001</v>
+        <v>6.428000000000001</v>
       </c>
       <c r="L16" t="n">
-        <v>6.462</v>
+        <v>10.777</v>
       </c>
       <c r="M16" t="n">
-        <v>9.309000000000001</v>
+        <v>10.704</v>
       </c>
       <c r="N16" t="n">
-        <v>11.872</v>
+        <v>9.167999999999999</v>
       </c>
       <c r="O16" t="n">
-        <v>11.698</v>
+        <v>11.572</v>
       </c>
       <c r="P16" t="n">
-        <v>8.583</v>
+        <v>11.793</v>
       </c>
       <c r="Q16" t="n">
-        <v>9.284000000000001</v>
+        <v>3.717</v>
       </c>
       <c r="R16" t="n">
-        <v>8.513999999999999</v>
+        <v>8.075000000000001</v>
       </c>
       <c r="S16" t="n">
-        <v>9.276</v>
+        <v>8.757</v>
       </c>
       <c r="T16" t="n">
-        <v>9.347</v>
+        <v>8.465</v>
       </c>
       <c r="U16" t="n">
-        <v>6.159</v>
+        <v>5.251</v>
       </c>
     </row>
     <row r="17">
@@ -1507,61 +1507,61 @@
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
         <v>0.002</v>
       </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
       <c r="F17" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.005</v>
       </c>
       <c r="H17" t="n">
-        <v>0.019</v>
+        <v>0.02</v>
       </c>
       <c r="I17" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.06999999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>1.781</v>
+        <v>3.415</v>
       </c>
       <c r="K17" t="n">
-        <v>4.181</v>
+        <v>4.483000000000001</v>
       </c>
       <c r="L17" t="n">
-        <v>4.682</v>
+        <v>8.831</v>
       </c>
       <c r="M17" t="n">
-        <v>7.500999999999999</v>
+        <v>8.923</v>
       </c>
       <c r="N17" t="n">
-        <v>12.1</v>
+        <v>7.181999999999999</v>
       </c>
       <c r="O17" t="n">
-        <v>11.091</v>
+        <v>12.312</v>
       </c>
       <c r="P17" t="n">
-        <v>10.601</v>
+        <v>12.801</v>
       </c>
       <c r="Q17" t="n">
-        <v>11.572</v>
+        <v>2.488</v>
       </c>
       <c r="R17" t="n">
-        <v>10.424</v>
+        <v>10.466</v>
       </c>
       <c r="S17" t="n">
-        <v>10.685</v>
+        <v>10.876</v>
       </c>
       <c r="T17" t="n">
-        <v>10.607</v>
+        <v>10.917</v>
       </c>
       <c r="U17" t="n">
-        <v>4.672</v>
+        <v>7.208</v>
       </c>
     </row>
     <row r="18">
@@ -1575,58 +1575,58 @@
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="F18" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
         <v>0.003</v>
       </c>
       <c r="H18" t="n">
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
       <c r="I18" t="n">
-        <v>0.02</v>
+        <v>0.021</v>
       </c>
       <c r="J18" t="n">
-        <v>1.003</v>
+        <v>2.007</v>
       </c>
       <c r="K18" t="n">
-        <v>2.656</v>
+        <v>2.841</v>
       </c>
       <c r="L18" t="n">
-        <v>3.409</v>
+        <v>6.933</v>
       </c>
       <c r="M18" t="n">
-        <v>5.765</v>
+        <v>6.875000000000001</v>
       </c>
       <c r="N18" t="n">
-        <v>11.442</v>
+        <v>5.461</v>
       </c>
       <c r="O18" t="n">
-        <v>10.226</v>
+        <v>11.979</v>
       </c>
       <c r="P18" t="n">
-        <v>12.544</v>
+        <v>12.288</v>
       </c>
       <c r="Q18" t="n">
-        <v>13.631</v>
+        <v>1.753</v>
       </c>
       <c r="R18" t="n">
-        <v>12.378</v>
+        <v>13.497</v>
       </c>
       <c r="S18" t="n">
-        <v>11.88</v>
+        <v>12.806</v>
       </c>
       <c r="T18" t="n">
-        <v>11.598</v>
+        <v>13.594</v>
       </c>
       <c r="U18" t="n">
-        <v>3.435</v>
+        <v>9.936</v>
       </c>
     </row>
     <row r="19">
@@ -1649,49 +1649,49 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="H19" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0.01</v>
+        <v>0.008</v>
       </c>
       <c r="J19" t="n">
-        <v>0.4969999999999999</v>
+        <v>0.979</v>
       </c>
       <c r="K19" t="n">
-        <v>1.475</v>
+        <v>1.615</v>
       </c>
       <c r="L19" t="n">
-        <v>2.093</v>
+        <v>5.005</v>
       </c>
       <c r="M19" t="n">
-        <v>4.157</v>
+        <v>5.064</v>
       </c>
       <c r="N19" t="n">
-        <v>10.181</v>
+        <v>3.874</v>
       </c>
       <c r="O19" t="n">
-        <v>9.138</v>
+        <v>11.119</v>
       </c>
       <c r="P19" t="n">
-        <v>14.857</v>
+        <v>11.099</v>
       </c>
       <c r="Q19" t="n">
-        <v>15.101</v>
+        <v>1.037</v>
       </c>
       <c r="R19" t="n">
-        <v>14.313</v>
+        <v>16.12</v>
       </c>
       <c r="S19" t="n">
-        <v>12.87</v>
+        <v>14.755</v>
       </c>
       <c r="T19" t="n">
-        <v>12.848</v>
+        <v>15.832</v>
       </c>
       <c r="U19" t="n">
-        <v>2.459</v>
+        <v>13.489</v>
       </c>
     </row>
     <row r="20">
@@ -1717,46 +1717,46 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="I20" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
       <c r="J20" t="n">
-        <v>0.194</v>
+        <v>0.402</v>
       </c>
       <c r="K20" t="n">
-        <v>0.734</v>
+        <v>0.747</v>
       </c>
       <c r="L20" t="n">
-        <v>1.299</v>
+        <v>2.906</v>
       </c>
       <c r="M20" t="n">
-        <v>2.672</v>
+        <v>3.153</v>
       </c>
       <c r="N20" t="n">
-        <v>8.031000000000001</v>
+        <v>2.392</v>
       </c>
       <c r="O20" t="n">
-        <v>7.504</v>
+        <v>8.860999999999999</v>
       </c>
       <c r="P20" t="n">
-        <v>16.888</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="Q20" t="n">
-        <v>16.304</v>
+        <v>0.545</v>
       </c>
       <c r="R20" t="n">
-        <v>16.439</v>
+        <v>18.997</v>
       </c>
       <c r="S20" t="n">
-        <v>14.251</v>
+        <v>16.215</v>
       </c>
       <c r="T20" t="n">
-        <v>14.101</v>
+        <v>17.962</v>
       </c>
       <c r="U20" t="n">
-        <v>1.578</v>
+        <v>19.266</v>
       </c>
     </row>
     <row r="21">
@@ -1785,43 +1785,43 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="J21" t="n">
-        <v>0.045</v>
+        <v>0.092</v>
       </c>
       <c r="K21" t="n">
-        <v>0.226</v>
+        <v>0.212</v>
       </c>
       <c r="L21" t="n">
-        <v>0.544</v>
+        <v>1.089</v>
       </c>
       <c r="M21" t="n">
-        <v>1.34</v>
+        <v>1.313</v>
       </c>
       <c r="N21" t="n">
-        <v>4.662</v>
+        <v>1.05</v>
       </c>
       <c r="O21" t="n">
-        <v>5.023</v>
+        <v>4.89</v>
       </c>
       <c r="P21" t="n">
-        <v>18.372</v>
+        <v>4.518</v>
       </c>
       <c r="Q21" t="n">
-        <v>17.554</v>
+        <v>0.202</v>
       </c>
       <c r="R21" t="n">
-        <v>19.157</v>
+        <v>16.745</v>
       </c>
       <c r="S21" t="n">
-        <v>15.074</v>
+        <v>15.927</v>
       </c>
       <c r="T21" t="n">
-        <v>17.125</v>
+        <v>18.421</v>
       </c>
       <c r="U21" t="n">
-        <v>0.878</v>
+        <v>35.54</v>
       </c>
     </row>
   </sheetData>
@@ -1857,7 +1857,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99.869</v>
+        <v>99.88900000000001</v>
       </c>
     </row>
     <row r="3">
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.815</v>
+        <v>99.80199999999998</v>
       </c>
     </row>
     <row r="4">
@@ -1877,27 +1877,27 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>97.91500000000002</v>
+        <v>98.12899999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Independiente Medellín</t>
+          <t>Deportivo Cali</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>93.03</v>
+        <v>95.595</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Deportivo Cali</t>
+          <t>Independiente Medellín</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>88.875</v>
+        <v>88.96600000000001</v>
       </c>
     </row>
     <row r="7">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>86.7</v>
+        <v>87.369</v>
       </c>
     </row>
     <row r="8">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>85.84899999999999</v>
+        <v>84.768</v>
       </c>
     </row>
     <row r="9">
@@ -1927,67 +1927,67 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>76.827</v>
+        <v>78.75</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Llaneros</t>
+          <t>Junior</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>26.599</v>
+        <v>24.847</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>Llaneros</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>14.261</v>
+        <v>15.191</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Águilas Doradas</t>
+          <t>Once Caldas</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>11.924</v>
+        <v>9.901000000000002</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Once Caldas</t>
+          <t>Águilas Doradas</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9.208</v>
+        <v>6.737000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Internacional de Bogotá</t>
+          <t>Cúcuta Deportivo</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4.631</v>
+        <v>3.511</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cúcuta Deportivo</t>
+          <t>Internacional de Bogotá</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.498</v>
+        <v>3.434</v>
       </c>
     </row>
     <row r="16">
@@ -1997,27 +1997,27 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.296</v>
+        <v>1.351</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Deportivo Pereira</t>
+          <t>Alianza Valledupar</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.608</v>
+        <v>1.037</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Jaguares</t>
+          <t>Deportivo Pereira</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.5239999999999999</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="19">
@@ -2027,27 +2027,27 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.244</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Alianza Valledupar</t>
+          <t>Deportivo Pasto</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.243</v>
+        <v>0.102</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Deportivo Pasto</t>
+          <t>Jaguares</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.07599999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar resultados de Finalizacion 2026-II hasta el 04/10/2026
- Carga 7 partidos jugados entre el 29 de septiembre y el 4 de
  octubre (Deportivo Pereira 1-2 Santa Fe, Independiente Medellin
  2-2 Millonarios, Atletico Nacional 3-1 Junior, Deportivo Cali 3-1
  Alianza Valledupar, Aguilas Doradas 2-0 Jaguares, Deportes Tolima
  0-0 Boyaca Chico, Deportivo Pasto 0-0 Fortaleza) con
  actualizar_resultados.py.
- Tabla.csv/Partidos.csv/Historial_partidos.csv actualizados;
  historial pasa de 761 a 768 partidos. Tabla verificada contra
  Dimayor en vivo. America de Cali y Deportivo Cali quedan
  empatados en la punta (24 pts).
- model_params.csv: DrawBias recalibrado exacto (227/768).
- Resultados.xlsx/Resultado.png regenerados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resultados.xlsx
+++ b/Resultados.xlsx
@@ -435,19 +435,19 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Atlético Nacional</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Millonarios</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Atlético Bucaramanga</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Millonarios</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Atlético Nacional</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
           <t>Independiente Medellín</t>
@@ -455,14 +455,14 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Deportes Tolima</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
       <c r="J1" t="inlineStr">
         <is>
           <t>Llaneros</t>
@@ -470,24 +470,24 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>Águilas Doradas</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Once Caldas</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Internacional de Bogotá</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Cúcuta Deportivo</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Águilas Doradas</t>
-        </is>
-      </c>
       <c r="O1" t="inlineStr">
         <is>
           <t>Boyacá Chicó</t>
@@ -500,22 +500,22 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Fortaleza</t>
-        </is>
-      </c>
       <c r="S1" t="inlineStr">
         <is>
+          <t>Deportivo Pasto</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>Deportivo Pereira</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Deportivo Pasto</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
@@ -529,55 +529,55 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>35.036</v>
+        <v>29.139</v>
       </c>
       <c r="C2" t="n">
-        <v>3.864</v>
+        <v>4.843</v>
       </c>
       <c r="D2" t="n">
-        <v>11.71</v>
+        <v>54.72900000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>0.629</v>
+        <v>0.277</v>
       </c>
       <c r="F2" t="n">
-        <v>44.91</v>
+        <v>8.963000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>2.343</v>
+        <v>0.872</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7230000000000001</v>
+        <v>1.033</v>
       </c>
       <c r="I2" t="n">
-        <v>0.763</v>
+        <v>0.143</v>
       </c>
       <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
         <v>0.001</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
       </c>
       <c r="S2" t="n">
         <v>0</v>
@@ -594,55 +594,55 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>31.784</v>
+        <v>35.035</v>
       </c>
       <c r="C3" t="n">
-        <v>9.596</v>
+        <v>13.443</v>
       </c>
       <c r="D3" t="n">
-        <v>17.202</v>
+        <v>26.488</v>
       </c>
       <c r="E3" t="n">
-        <v>2.813</v>
+        <v>1.866</v>
       </c>
       <c r="F3" t="n">
-        <v>27.695</v>
+        <v>15.973</v>
       </c>
       <c r="G3" t="n">
-        <v>5.595</v>
+        <v>2.864</v>
       </c>
       <c r="H3" t="n">
-        <v>2.759</v>
+        <v>3.449</v>
       </c>
       <c r="I3" t="n">
-        <v>2.427</v>
+        <v>0.831</v>
       </c>
       <c r="J3" t="n">
-        <v>0.021</v>
+        <v>0.022</v>
       </c>
       <c r="K3" t="n">
-        <v>0.001</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
         <v>0.002</v>
       </c>
-      <c r="N3" t="n">
-        <v>0.009000000000000001</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.096</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>0</v>
+        <v>0.014</v>
       </c>
       <c r="S3" t="n">
         <v>0</v>
@@ -659,55 +659,55 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>16.05</v>
+        <v>17.471</v>
       </c>
       <c r="C4" t="n">
-        <v>17.234</v>
+        <v>23.522</v>
       </c>
       <c r="D4" t="n">
-        <v>22.579</v>
+        <v>10.576</v>
       </c>
       <c r="E4" t="n">
-        <v>6.914</v>
+        <v>6.457</v>
       </c>
       <c r="F4" t="n">
-        <v>13.151</v>
+        <v>23.058</v>
       </c>
       <c r="G4" t="n">
-        <v>10.405</v>
+        <v>6.793</v>
       </c>
       <c r="H4" t="n">
-        <v>6.977</v>
+        <v>8.895</v>
       </c>
       <c r="I4" t="n">
-        <v>6.066</v>
+        <v>2.897</v>
       </c>
       <c r="J4" t="n">
-        <v>0.116</v>
+        <v>0.115</v>
       </c>
       <c r="K4" t="n">
-        <v>0.039</v>
+        <v>0.05599999999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>0.003</v>
+        <v>0.023</v>
       </c>
       <c r="M4" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="N4" t="n">
         <v>0.004</v>
       </c>
-      <c r="N4" t="n">
-        <v>0.034</v>
-      </c>
       <c r="O4" t="n">
-        <v>0.006</v>
+        <v>0.002</v>
       </c>
       <c r="P4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.421</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>0.126</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
@@ -724,61 +724,61 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>8.598000000000001</v>
+        <v>9.578000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>19.037</v>
+        <v>22.686</v>
       </c>
       <c r="D5" t="n">
-        <v>17.363</v>
+        <v>4.606</v>
       </c>
       <c r="E5" t="n">
-        <v>11.929</v>
+        <v>12.015</v>
       </c>
       <c r="F5" t="n">
-        <v>6.815</v>
+        <v>19.052</v>
       </c>
       <c r="G5" t="n">
-        <v>14.197</v>
+        <v>11.131</v>
       </c>
       <c r="H5" t="n">
-        <v>11.066</v>
+        <v>13.535</v>
       </c>
       <c r="I5" t="n">
-        <v>9.198</v>
+        <v>6.212</v>
       </c>
       <c r="J5" t="n">
-        <v>0.382</v>
+        <v>0.351</v>
       </c>
       <c r="K5" t="n">
-        <v>0.155</v>
+        <v>0.215</v>
       </c>
       <c r="L5" t="n">
-        <v>0.018</v>
+        <v>0.11</v>
       </c>
       <c r="M5" t="n">
-        <v>0.033</v>
+        <v>0.015</v>
       </c>
       <c r="N5" t="n">
-        <v>0.14</v>
+        <v>0.026</v>
       </c>
       <c r="O5" t="n">
         <v>0.01</v>
       </c>
       <c r="P5" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.054</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>0.458</v>
       </c>
       <c r="S5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -789,64 +789,64 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>4.557</v>
+        <v>4.79</v>
       </c>
       <c r="C6" t="n">
-        <v>16.975</v>
+        <v>15.351</v>
       </c>
       <c r="D6" t="n">
-        <v>12.521</v>
+        <v>2.117</v>
       </c>
       <c r="E6" t="n">
-        <v>15.778</v>
+        <v>18.192</v>
       </c>
       <c r="F6" t="n">
-        <v>3.752</v>
+        <v>13.511</v>
       </c>
       <c r="G6" t="n">
-        <v>15.803</v>
+        <v>15.47</v>
       </c>
       <c r="H6" t="n">
-        <v>14.421</v>
+        <v>17.014</v>
       </c>
       <c r="I6" t="n">
-        <v>12.152</v>
+        <v>10.371</v>
       </c>
       <c r="J6" t="n">
-        <v>0.947</v>
+        <v>0.873</v>
       </c>
       <c r="K6" t="n">
-        <v>0.43</v>
+        <v>0.611</v>
       </c>
       <c r="L6" t="n">
-        <v>0.08099999999999999</v>
+        <v>0.4460000000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>0.08099999999999999</v>
+        <v>0.079</v>
       </c>
       <c r="N6" t="n">
-        <v>0.34</v>
+        <v>0.077</v>
       </c>
       <c r="O6" t="n">
-        <v>0.037</v>
+        <v>0.041</v>
       </c>
       <c r="P6" t="n">
-        <v>0.026</v>
+        <v>0.006</v>
       </c>
       <c r="Q6" t="n">
-        <v>2.085</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>0.005</v>
+        <v>1.051</v>
       </c>
       <c r="S6" t="n">
-        <v>0.006</v>
+        <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -854,64 +854,64 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>2.42</v>
+        <v>2.435</v>
       </c>
       <c r="C7" t="n">
-        <v>13.455</v>
+        <v>10.018</v>
       </c>
       <c r="D7" t="n">
-        <v>8.364000000000001</v>
+        <v>0.898</v>
       </c>
       <c r="E7" t="n">
-        <v>17.888</v>
+        <v>20.128</v>
       </c>
       <c r="F7" t="n">
-        <v>1.999</v>
+        <v>9.153</v>
       </c>
       <c r="G7" t="n">
-        <v>15.576</v>
+        <v>17.408</v>
       </c>
       <c r="H7" t="n">
-        <v>16.71</v>
+        <v>17.748</v>
       </c>
       <c r="I7" t="n">
-        <v>15.07</v>
+        <v>14.729</v>
       </c>
       <c r="J7" t="n">
-        <v>1.947</v>
+        <v>1.925</v>
       </c>
       <c r="K7" t="n">
-        <v>1.188</v>
+        <v>1.424</v>
       </c>
       <c r="L7" t="n">
-        <v>0.305</v>
+        <v>1.237</v>
       </c>
       <c r="M7" t="n">
-        <v>0.323</v>
+        <v>0.253</v>
       </c>
       <c r="N7" t="n">
-        <v>0.786</v>
+        <v>0.254</v>
       </c>
       <c r="O7" t="n">
-        <v>0.107</v>
+        <v>0.122</v>
       </c>
       <c r="P7" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.013</v>
       </c>
       <c r="Q7" t="n">
-        <v>3.736</v>
+        <v>0.005</v>
       </c>
       <c r="R7" t="n">
-        <v>0.006999999999999999</v>
+        <v>2.245</v>
       </c>
       <c r="S7" t="n">
-        <v>0.022</v>
+        <v>0.001</v>
       </c>
       <c r="T7" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="U7" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="8">
@@ -919,64 +919,64 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>1.047</v>
+        <v>1.081</v>
       </c>
       <c r="C8" t="n">
-        <v>9.395000000000001</v>
+        <v>5.855</v>
       </c>
       <c r="D8" t="n">
-        <v>5.399</v>
+        <v>0.411</v>
       </c>
       <c r="E8" t="n">
-        <v>17.504</v>
+        <v>18.005</v>
       </c>
       <c r="F8" t="n">
-        <v>1.021</v>
+        <v>5.527</v>
       </c>
       <c r="G8" t="n">
-        <v>14.011</v>
+        <v>17.649</v>
       </c>
       <c r="H8" t="n">
-        <v>17.346</v>
+        <v>16.247</v>
       </c>
       <c r="I8" t="n">
-        <v>17.01</v>
+        <v>18.969</v>
       </c>
       <c r="J8" t="n">
-        <v>4.101</v>
+        <v>4.008</v>
       </c>
       <c r="K8" t="n">
-        <v>2.524</v>
+        <v>3.201</v>
       </c>
       <c r="L8" t="n">
-        <v>0.826</v>
+        <v>2.686</v>
       </c>
       <c r="M8" t="n">
-        <v>0.869</v>
+        <v>0.741</v>
       </c>
       <c r="N8" t="n">
-        <v>1.782</v>
+        <v>0.741</v>
       </c>
       <c r="O8" t="n">
-        <v>0.303</v>
+        <v>0.336</v>
       </c>
       <c r="P8" t="n">
-        <v>0.239</v>
+        <v>0.064</v>
       </c>
       <c r="Q8" t="n">
-        <v>6.465</v>
+        <v>0.016</v>
       </c>
       <c r="R8" t="n">
-        <v>0.039</v>
+        <v>4.439</v>
       </c>
       <c r="S8" t="n">
-        <v>0.093</v>
+        <v>0.005</v>
       </c>
       <c r="T8" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="U8" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="9">
@@ -984,64 +984,64 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.397</v>
+        <v>0.378</v>
       </c>
       <c r="C9" t="n">
-        <v>6.039</v>
+        <v>2.929</v>
       </c>
       <c r="D9" t="n">
-        <v>2.991</v>
+        <v>0.143</v>
       </c>
       <c r="E9" t="n">
-        <v>13.914</v>
+        <v>13.281</v>
       </c>
       <c r="F9" t="n">
-        <v>0.459</v>
+        <v>2.954</v>
       </c>
       <c r="G9" t="n">
-        <v>11.036</v>
+        <v>13.847</v>
       </c>
       <c r="H9" t="n">
-        <v>14.766</v>
+        <v>11.752</v>
       </c>
       <c r="I9" t="n">
-        <v>16.064</v>
+        <v>20.989</v>
       </c>
       <c r="J9" t="n">
-        <v>7.675999999999999</v>
+        <v>7.593999999999999</v>
       </c>
       <c r="K9" t="n">
-        <v>5.564</v>
+        <v>6.262</v>
       </c>
       <c r="L9" t="n">
-        <v>2.201</v>
+        <v>5.709000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>2.199</v>
+        <v>2.138</v>
       </c>
       <c r="N9" t="n">
-        <v>3.645</v>
+        <v>1.968</v>
       </c>
       <c r="O9" t="n">
-        <v>0.8880000000000001</v>
+        <v>1.055</v>
       </c>
       <c r="P9" t="n">
-        <v>0.6819999999999999</v>
+        <v>0.283</v>
       </c>
       <c r="Q9" t="n">
-        <v>10.97</v>
+        <v>0.077</v>
       </c>
       <c r="R9" t="n">
-        <v>0.119</v>
+        <v>8.52</v>
       </c>
       <c r="S9" t="n">
-        <v>0.253</v>
+        <v>0.014</v>
       </c>
       <c r="T9" t="n">
-        <v>0.08</v>
+        <v>0.099</v>
       </c>
       <c r="U9" t="n">
-        <v>0.057</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="10">
@@ -1049,64 +1049,64 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.08099999999999999</v>
       </c>
       <c r="C10" t="n">
-        <v>2.877</v>
+        <v>0.9979999999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>1.218</v>
+        <v>0.027</v>
       </c>
       <c r="E10" t="n">
-        <v>7.309</v>
+        <v>6.081</v>
       </c>
       <c r="F10" t="n">
-        <v>0.148</v>
+        <v>1.199</v>
       </c>
       <c r="G10" t="n">
-        <v>5.970000000000001</v>
+        <v>7.571999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>8.347</v>
+        <v>5.766</v>
       </c>
       <c r="I10" t="n">
-        <v>10.166</v>
+        <v>12.62</v>
       </c>
       <c r="J10" t="n">
-        <v>13.298</v>
+        <v>14.057</v>
       </c>
       <c r="K10" t="n">
-        <v>10.934</v>
+        <v>11.396</v>
       </c>
       <c r="L10" t="n">
-        <v>4.913</v>
+        <v>11.141</v>
       </c>
       <c r="M10" t="n">
-        <v>5.101</v>
+        <v>4.889</v>
       </c>
       <c r="N10" t="n">
-        <v>7.339</v>
+        <v>4.956</v>
       </c>
       <c r="O10" t="n">
-        <v>2.176</v>
+        <v>2.889</v>
       </c>
       <c r="P10" t="n">
-        <v>1.886</v>
+        <v>0.9249999999999999</v>
       </c>
       <c r="Q10" t="n">
-        <v>16.812</v>
+        <v>0.245</v>
       </c>
       <c r="R10" t="n">
-        <v>0.314</v>
+        <v>14.747</v>
       </c>
       <c r="S10" t="n">
-        <v>0.666</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="T10" t="n">
-        <v>0.239</v>
+        <v>0.279</v>
       </c>
       <c r="U10" t="n">
-        <v>0.2</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="11">
@@ -1114,64 +1114,64 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.024</v>
+        <v>0.01</v>
       </c>
       <c r="C11" t="n">
-        <v>1.016</v>
+        <v>0.285</v>
       </c>
       <c r="D11" t="n">
-        <v>0.4420000000000001</v>
+        <v>0.005</v>
       </c>
       <c r="E11" t="n">
-        <v>3.328</v>
+        <v>2.472</v>
       </c>
       <c r="F11" t="n">
-        <v>0.035</v>
+        <v>0.427</v>
       </c>
       <c r="G11" t="n">
-        <v>2.824</v>
+        <v>3.532</v>
       </c>
       <c r="H11" t="n">
-        <v>3.872</v>
+        <v>2.67</v>
       </c>
       <c r="I11" t="n">
-        <v>5.416</v>
+        <v>6.600000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>15.722</v>
+        <v>15.606</v>
       </c>
       <c r="K11" t="n">
-        <v>14.836</v>
+        <v>14.361</v>
       </c>
       <c r="L11" t="n">
-        <v>8.121</v>
+        <v>14.535</v>
       </c>
       <c r="M11" t="n">
-        <v>8.142000000000001</v>
+        <v>8.131</v>
       </c>
       <c r="N11" t="n">
-        <v>10.325</v>
+        <v>7.933</v>
       </c>
       <c r="O11" t="n">
-        <v>3.795</v>
+        <v>4.987</v>
       </c>
       <c r="P11" t="n">
-        <v>3.499</v>
+        <v>1.988</v>
       </c>
       <c r="Q11" t="n">
-        <v>15.115</v>
+        <v>0.709</v>
       </c>
       <c r="R11" t="n">
-        <v>0.8580000000000001</v>
+        <v>14.741</v>
       </c>
       <c r="S11" t="n">
-        <v>1.458</v>
+        <v>0.248</v>
       </c>
       <c r="T11" t="n">
-        <v>0.698</v>
+        <v>0.596</v>
       </c>
       <c r="U11" t="n">
-        <v>0.474</v>
+        <v>0.164</v>
       </c>
     </row>
     <row r="12">
@@ -1179,64 +1179,64 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="C12" t="n">
-        <v>0.363</v>
+        <v>0.054</v>
       </c>
       <c r="D12" t="n">
-        <v>0.146</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>1.305</v>
+        <v>0.8420000000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>0.011</v>
+        <v>0.118</v>
       </c>
       <c r="G12" t="n">
-        <v>1.309</v>
+        <v>1.689</v>
       </c>
       <c r="H12" t="n">
-        <v>1.746</v>
+        <v>1.15</v>
       </c>
       <c r="I12" t="n">
-        <v>2.826</v>
+        <v>3.261</v>
       </c>
       <c r="J12" t="n">
-        <v>14.754</v>
+        <v>14.479</v>
       </c>
       <c r="K12" t="n">
-        <v>14.865</v>
+        <v>14.338</v>
       </c>
       <c r="L12" t="n">
-        <v>10.727</v>
+        <v>14.703</v>
       </c>
       <c r="M12" t="n">
-        <v>10.537</v>
+        <v>10.815</v>
       </c>
       <c r="N12" t="n">
-        <v>11.954</v>
+        <v>10.661</v>
       </c>
       <c r="O12" t="n">
-        <v>5.587000000000001</v>
+        <v>7.142999999999999</v>
       </c>
       <c r="P12" t="n">
-        <v>5.437</v>
+        <v>3.581</v>
       </c>
       <c r="Q12" t="n">
-        <v>12.002</v>
+        <v>1.448</v>
       </c>
       <c r="R12" t="n">
-        <v>1.706</v>
+        <v>13.448</v>
       </c>
       <c r="S12" t="n">
-        <v>2.442</v>
+        <v>0.65</v>
       </c>
       <c r="T12" t="n">
-        <v>1.403</v>
+        <v>1.216</v>
       </c>
       <c r="U12" t="n">
-        <v>0.88</v>
+        <v>0.402</v>
       </c>
     </row>
     <row r="13">
@@ -1247,61 +1247,61 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.105</v>
+        <v>0.014</v>
       </c>
       <c r="D13" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0.453</v>
+        <v>0.282</v>
       </c>
       <c r="F13" t="n">
-        <v>0.003</v>
+        <v>0.049</v>
       </c>
       <c r="G13" t="n">
-        <v>0.584</v>
+        <v>0.758</v>
       </c>
       <c r="H13" t="n">
-        <v>0.772</v>
+        <v>0.482</v>
       </c>
       <c r="I13" t="n">
-        <v>1.468</v>
+        <v>1.443</v>
       </c>
       <c r="J13" t="n">
-        <v>12.211</v>
+        <v>12.539</v>
       </c>
       <c r="K13" t="n">
-        <v>13.363</v>
+        <v>13.508</v>
       </c>
       <c r="L13" t="n">
-        <v>12.331</v>
+        <v>13.813</v>
       </c>
       <c r="M13" t="n">
-        <v>12.168</v>
+        <v>12.374</v>
       </c>
       <c r="N13" t="n">
-        <v>12.242</v>
+        <v>12.328</v>
       </c>
       <c r="O13" t="n">
-        <v>7.431</v>
+        <v>9.193</v>
       </c>
       <c r="P13" t="n">
-        <v>7.152</v>
+        <v>5.24</v>
       </c>
       <c r="Q13" t="n">
-        <v>9.236000000000001</v>
+        <v>2.511</v>
       </c>
       <c r="R13" t="n">
-        <v>2.745</v>
+        <v>11.228</v>
       </c>
       <c r="S13" t="n">
-        <v>3.704</v>
+        <v>1.302</v>
       </c>
       <c r="T13" t="n">
-        <v>2.422</v>
+        <v>2.171</v>
       </c>
       <c r="U13" t="n">
-        <v>1.57</v>
+        <v>0.765</v>
       </c>
     </row>
     <row r="14">
@@ -1312,61 +1312,61 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0.033</v>
+        <v>0.002</v>
       </c>
       <c r="D14" t="n">
-        <v>0.015</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0.167</v>
+        <v>0.08099999999999999</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="G14" t="n">
-        <v>0.222</v>
+        <v>0.278</v>
       </c>
       <c r="H14" t="n">
-        <v>0.291</v>
+        <v>0.181</v>
       </c>
       <c r="I14" t="n">
-        <v>0.734</v>
+        <v>0.617</v>
       </c>
       <c r="J14" t="n">
-        <v>9.823</v>
+        <v>9.98</v>
       </c>
       <c r="K14" t="n">
-        <v>11.072</v>
+        <v>11.348</v>
       </c>
       <c r="L14" t="n">
-        <v>12.776</v>
+        <v>11.644</v>
       </c>
       <c r="M14" t="n">
-        <v>12.49</v>
+        <v>13.443</v>
       </c>
       <c r="N14" t="n">
-        <v>11.716</v>
+        <v>13.391</v>
       </c>
       <c r="O14" t="n">
-        <v>8.824</v>
+        <v>11.037</v>
       </c>
       <c r="P14" t="n">
-        <v>8.998000000000001</v>
+        <v>7.292</v>
       </c>
       <c r="Q14" t="n">
-        <v>6.920999999999999</v>
+        <v>4.239</v>
       </c>
       <c r="R14" t="n">
-        <v>4.302</v>
+        <v>9.027000000000001</v>
       </c>
       <c r="S14" t="n">
-        <v>5.192</v>
+        <v>2.584</v>
       </c>
       <c r="T14" t="n">
-        <v>3.984999999999999</v>
+        <v>3.399</v>
       </c>
       <c r="U14" t="n">
-        <v>2.439</v>
+        <v>1.449</v>
       </c>
     </row>
     <row r="15">
@@ -1377,61 +1377,61 @@
         <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>0.009000000000000001</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>0.008</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>0.052</v>
+        <v>0.02</v>
       </c>
       <c r="F15" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="G15" t="n">
-        <v>0.082</v>
+        <v>0.107</v>
       </c>
       <c r="H15" t="n">
-        <v>0.134</v>
+        <v>0.06</v>
       </c>
       <c r="I15" t="n">
-        <v>0.379</v>
+        <v>0.214</v>
       </c>
       <c r="J15" t="n">
-        <v>7.063</v>
+        <v>7.441000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>8.702999999999999</v>
+        <v>8.789</v>
       </c>
       <c r="L15" t="n">
-        <v>12.157</v>
+        <v>9.052</v>
       </c>
       <c r="M15" t="n">
-        <v>12.019</v>
+        <v>12.921</v>
       </c>
       <c r="N15" t="n">
-        <v>10.56</v>
+        <v>13.175</v>
       </c>
       <c r="O15" t="n">
-        <v>10.103</v>
+        <v>12.463</v>
       </c>
       <c r="P15" t="n">
-        <v>10.942</v>
+        <v>9.997</v>
       </c>
       <c r="Q15" t="n">
-        <v>5.325</v>
+        <v>6.49</v>
       </c>
       <c r="R15" t="n">
-        <v>6.005</v>
+        <v>7.091</v>
       </c>
       <c r="S15" t="n">
-        <v>6.827</v>
+        <v>4.626</v>
       </c>
       <c r="T15" t="n">
-        <v>5.96</v>
+        <v>5.111000000000001</v>
       </c>
       <c r="U15" t="n">
-        <v>3.671</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="16">
@@ -1442,61 +1442,61 @@
         <v>0</v>
       </c>
       <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
         <v>0.001</v>
       </c>
-      <c r="D16" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0.013</v>
-      </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="G16" t="n">
-        <v>0.031</v>
+        <v>0.022</v>
       </c>
       <c r="H16" t="n">
-        <v>0.045</v>
+        <v>0.016</v>
       </c>
       <c r="I16" t="n">
-        <v>0.158</v>
+        <v>0.08499999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>5.043</v>
+        <v>4.945</v>
       </c>
       <c r="K16" t="n">
-        <v>6.428000000000001</v>
+        <v>6.145</v>
       </c>
       <c r="L16" t="n">
-        <v>10.777</v>
+        <v>6.324000000000001</v>
       </c>
       <c r="M16" t="n">
-        <v>10.704</v>
+        <v>11.325</v>
       </c>
       <c r="N16" t="n">
-        <v>9.167999999999999</v>
+        <v>11.431</v>
       </c>
       <c r="O16" t="n">
-        <v>11.572</v>
+        <v>13.36</v>
       </c>
       <c r="P16" t="n">
-        <v>11.793</v>
+        <v>12.539</v>
       </c>
       <c r="Q16" t="n">
-        <v>3.717</v>
+        <v>9.260999999999999</v>
       </c>
       <c r="R16" t="n">
-        <v>8.075000000000001</v>
+        <v>5.223</v>
       </c>
       <c r="S16" t="n">
-        <v>8.757</v>
+        <v>7.599</v>
       </c>
       <c r="T16" t="n">
-        <v>8.465</v>
+        <v>7.636</v>
       </c>
       <c r="U16" t="n">
-        <v>5.251</v>
+        <v>4.085</v>
       </c>
     </row>
     <row r="17">
@@ -1507,61 +1507,61 @@
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
       <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
         <v>0.002</v>
       </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
       <c r="G17" t="n">
-        <v>0.005</v>
+        <v>0.008</v>
       </c>
       <c r="H17" t="n">
-        <v>0.02</v>
+        <v>0.002</v>
       </c>
       <c r="I17" t="n">
-        <v>0.06999999999999999</v>
+        <v>0.016</v>
       </c>
       <c r="J17" t="n">
-        <v>3.415</v>
+        <v>3.076</v>
       </c>
       <c r="K17" t="n">
-        <v>4.483000000000001</v>
+        <v>4.164000000000001</v>
       </c>
       <c r="L17" t="n">
-        <v>8.831</v>
+        <v>4.145</v>
       </c>
       <c r="M17" t="n">
-        <v>8.923</v>
+        <v>8.727</v>
       </c>
       <c r="N17" t="n">
-        <v>7.181999999999999</v>
+        <v>9.007999999999999</v>
       </c>
       <c r="O17" t="n">
-        <v>12.312</v>
+        <v>12.395</v>
       </c>
       <c r="P17" t="n">
-        <v>12.801</v>
+        <v>14.688</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.488</v>
+        <v>12.698</v>
       </c>
       <c r="R17" t="n">
-        <v>10.466</v>
+        <v>3.468</v>
       </c>
       <c r="S17" t="n">
-        <v>10.876</v>
+        <v>11.259</v>
       </c>
       <c r="T17" t="n">
-        <v>10.917</v>
+        <v>10.225</v>
       </c>
       <c r="U17" t="n">
-        <v>7.208</v>
+        <v>6.119</v>
       </c>
     </row>
     <row r="18">
@@ -1578,55 +1578,55 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
         <v>0.003</v>
       </c>
-      <c r="H18" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0.021</v>
-      </c>
       <c r="J18" t="n">
-        <v>2.007</v>
+        <v>1.745</v>
       </c>
       <c r="K18" t="n">
-        <v>2.841</v>
+        <v>2.319</v>
       </c>
       <c r="L18" t="n">
-        <v>6.933</v>
+        <v>2.471</v>
       </c>
       <c r="M18" t="n">
-        <v>6.875000000000001</v>
+        <v>6.61</v>
       </c>
       <c r="N18" t="n">
-        <v>5.461</v>
+        <v>6.370000000000001</v>
       </c>
       <c r="O18" t="n">
-        <v>11.979</v>
+        <v>10.301</v>
       </c>
       <c r="P18" t="n">
-        <v>12.288</v>
+        <v>14.696</v>
       </c>
       <c r="Q18" t="n">
-        <v>1.753</v>
+        <v>16.149</v>
       </c>
       <c r="R18" t="n">
-        <v>13.497</v>
+        <v>2.111</v>
       </c>
       <c r="S18" t="n">
-        <v>12.806</v>
+        <v>14.659</v>
       </c>
       <c r="T18" t="n">
-        <v>13.594</v>
+        <v>13.177</v>
       </c>
       <c r="U18" t="n">
-        <v>9.936</v>
+        <v>9.388999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -1649,49 +1649,49 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0.008</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0.979</v>
+        <v>0.872</v>
       </c>
       <c r="K19" t="n">
-        <v>1.615</v>
+        <v>1.291</v>
       </c>
       <c r="L19" t="n">
-        <v>5.005</v>
+        <v>1.29</v>
       </c>
       <c r="M19" t="n">
-        <v>5.064</v>
+        <v>4.413</v>
       </c>
       <c r="N19" t="n">
-        <v>3.874</v>
+        <v>4.215</v>
       </c>
       <c r="O19" t="n">
-        <v>11.119</v>
+        <v>7.788</v>
       </c>
       <c r="P19" t="n">
-        <v>11.099</v>
+        <v>12.878</v>
       </c>
       <c r="Q19" t="n">
-        <v>1.037</v>
+        <v>18.149</v>
       </c>
       <c r="R19" t="n">
-        <v>16.12</v>
+        <v>1.223</v>
       </c>
       <c r="S19" t="n">
-        <v>14.755</v>
+        <v>18.203</v>
       </c>
       <c r="T19" t="n">
-        <v>15.832</v>
+        <v>16.454</v>
       </c>
       <c r="U19" t="n">
-        <v>13.489</v>
+        <v>13.224</v>
       </c>
     </row>
     <row r="20">
@@ -1717,46 +1717,46 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0.402</v>
+        <v>0.317</v>
       </c>
       <c r="K20" t="n">
-        <v>0.747</v>
+        <v>0.482</v>
       </c>
       <c r="L20" t="n">
-        <v>2.906</v>
+        <v>0.545</v>
       </c>
       <c r="M20" t="n">
-        <v>3.153</v>
+        <v>2.492</v>
       </c>
       <c r="N20" t="n">
-        <v>2.392</v>
+        <v>2.455</v>
       </c>
       <c r="O20" t="n">
-        <v>8.860999999999999</v>
+        <v>4.984</v>
       </c>
       <c r="P20" t="n">
-        <v>8.550000000000001</v>
+        <v>10.561</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.545</v>
+        <v>17.576</v>
       </c>
       <c r="R20" t="n">
-        <v>18.997</v>
+        <v>0.64</v>
       </c>
       <c r="S20" t="n">
-        <v>16.215</v>
+        <v>20.826</v>
       </c>
       <c r="T20" t="n">
-        <v>17.962</v>
+        <v>19.585</v>
       </c>
       <c r="U20" t="n">
-        <v>19.266</v>
+        <v>19.537</v>
       </c>
     </row>
     <row r="21">
@@ -1785,43 +1785,43 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0.092</v>
+        <v>0.055</v>
       </c>
       <c r="K21" t="n">
-        <v>0.212</v>
+        <v>0.08099999999999999</v>
       </c>
       <c r="L21" t="n">
-        <v>1.089</v>
+        <v>0.122</v>
       </c>
       <c r="M21" t="n">
-        <v>1.313</v>
+        <v>0.629</v>
       </c>
       <c r="N21" t="n">
-        <v>1.05</v>
+        <v>1.007</v>
       </c>
       <c r="O21" t="n">
-        <v>4.89</v>
+        <v>1.892</v>
       </c>
       <c r="P21" t="n">
-        <v>4.518</v>
+        <v>5.249000000000001</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.202</v>
+        <v>10.427</v>
       </c>
       <c r="R21" t="n">
-        <v>16.745</v>
+        <v>0.199</v>
       </c>
       <c r="S21" t="n">
-        <v>15.927</v>
+        <v>17.952</v>
       </c>
       <c r="T21" t="n">
-        <v>18.421</v>
+        <v>20.031</v>
       </c>
       <c r="U21" t="n">
-        <v>35.54</v>
+        <v>42.356</v>
       </c>
     </row>
   </sheetData>
@@ -1853,81 +1853,81 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>América de Cali</t>
+          <t>Atlético Nacional</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99.88900000000001</v>
+        <v>99.96800000000002</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Atlético Nacional</t>
+          <t>América de Cali</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.80199999999998</v>
+        <v>99.90699999999998</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Atlético Bucaramanga</t>
+          <t>Deportivo Cali</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>98.12899999999999</v>
+        <v>98.64699999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Deportivo Cali</t>
+          <t>Atlético Bucaramanga</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>95.595</v>
+        <v>98.191</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Independiente Medellín</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>88.96600000000001</v>
+        <v>90.221</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Millonarios</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>87.369</v>
+        <v>89.673</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Independiente Medellín</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>84.768</v>
+        <v>86.03399999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Deportes Tolima</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>78.75</v>
+        <v>75.14099999999999</v>
       </c>
     </row>
     <row r="10">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24.847</v>
+        <v>16.854</v>
       </c>
     </row>
     <row r="11">
@@ -1947,47 +1947,47 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15.191</v>
+        <v>14.888</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Once Caldas</t>
+          <t>Águilas Doradas</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9.901000000000002</v>
+        <v>11.778</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Águilas Doradas</t>
+          <t>Once Caldas</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6.737000000000001</v>
+        <v>10.215</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cúcuta Deportivo</t>
+          <t>Internacional de Bogotá</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3.511</v>
+        <v>3.231</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Internacional de Bogotá</t>
+          <t>Cúcuta Deportivo</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3.434</v>
+        <v>3.07</v>
       </c>
     </row>
     <row r="16">
@@ -1997,7 +1997,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.351</v>
+        <v>1.568</v>
       </c>
     </row>
     <row r="17">
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1.037</v>
+        <v>0.366</v>
       </c>
     </row>
     <row r="18">
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.375</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="19">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.17</v>
+        <v>0.098</v>
       </c>
     </row>
     <row r="20">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.102</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="21">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.07599999999999998</v>
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar resultados de Finalizacion 2026-II hasta el 08/10/2026
- Carga 7 partidos jugados entre el 4 y el 8 de octubre (Cucuta
  Deportivo 4-0 Deportivo Pereira, Atletico Bucaramanga 3-1 Junior,
  Llaneros 1-2 America de Cali, Internacional de Bogota 1-1 Once
  Caldas, Independiente Medellin 0-1 Santa Fe, Atletico Nacional 0-0
  Deportes Tolima, Fortaleza 1-1 Millonarios) con
  actualizar_resultados.py.
- Tabla.csv/Partidos.csv/Historial_partidos.csv actualizados;
  historial pasa de 768 a 775 partidos. Tabla verificada contra
  Dimayor en vivo. America de Cali se despega solo en la punta
  (27 pts, +17 DG).
- model_params.csv: DrawBias recalibrado exacto (230/775).
- Resultados.xlsx/Resultado.png regenerados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resultados.xlsx
+++ b/Resultados.xlsx
@@ -440,24 +440,24 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Atlético Bucaramanga</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Millonarios</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Atlético Bucaramanga</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Independiente Medellín</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
           <t>Deportes Tolima</t>
@@ -465,29 +465,29 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>Cúcuta Deportivo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>Llaneros</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Águilas Doradas</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Once Caldas</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Internacional de Bogotá</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Cúcuta Deportivo</t>
-        </is>
-      </c>
       <c r="O1" t="inlineStr">
         <is>
           <t>Boyacá Chicó</t>
@@ -495,12 +495,12 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>Alianza Valledupar</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Fortaleza</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
@@ -529,28 +529,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>29.139</v>
+        <v>46.212</v>
       </c>
       <c r="C2" t="n">
-        <v>4.843</v>
+        <v>4.383</v>
       </c>
       <c r="D2" t="n">
-        <v>54.72900000000001</v>
+        <v>33.591</v>
       </c>
       <c r="E2" t="n">
-        <v>0.277</v>
+        <v>13.462</v>
       </c>
       <c r="F2" t="n">
-        <v>8.963000000000001</v>
+        <v>0.039</v>
       </c>
       <c r="G2" t="n">
-        <v>0.872</v>
+        <v>2.196</v>
       </c>
       <c r="H2" t="n">
-        <v>1.033</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>0.143</v>
+        <v>0.031</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -577,7 +577,7 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
         <v>0</v>
@@ -594,37 +594,37 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>35.035</v>
+        <v>29.85</v>
       </c>
       <c r="C3" t="n">
-        <v>13.443</v>
+        <v>10.167</v>
       </c>
       <c r="D3" t="n">
-        <v>26.488</v>
+        <v>32.823</v>
       </c>
       <c r="E3" t="n">
-        <v>1.866</v>
+        <v>19.351</v>
       </c>
       <c r="F3" t="n">
-        <v>15.973</v>
+        <v>0.42</v>
       </c>
       <c r="G3" t="n">
-        <v>2.864</v>
+        <v>6.58</v>
       </c>
       <c r="H3" t="n">
-        <v>3.449</v>
+        <v>0.419</v>
       </c>
       <c r="I3" t="n">
-        <v>0.831</v>
+        <v>0.384</v>
       </c>
       <c r="J3" t="n">
-        <v>0.022</v>
+        <v>0.003</v>
       </c>
       <c r="K3" t="n">
-        <v>0.009000000000000001</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -633,7 +633,7 @@
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
@@ -642,7 +642,7 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>0.014</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
         <v>0</v>
@@ -659,55 +659,55 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>17.471</v>
+        <v>14.012</v>
       </c>
       <c r="C4" t="n">
-        <v>23.522</v>
+        <v>20.556</v>
       </c>
       <c r="D4" t="n">
-        <v>10.576</v>
+        <v>17.959</v>
       </c>
       <c r="E4" t="n">
-        <v>6.457</v>
+        <v>26.339</v>
       </c>
       <c r="F4" t="n">
-        <v>23.058</v>
+        <v>2.536</v>
       </c>
       <c r="G4" t="n">
-        <v>6.793</v>
+        <v>14.799</v>
       </c>
       <c r="H4" t="n">
-        <v>8.895</v>
+        <v>1.491</v>
       </c>
       <c r="I4" t="n">
-        <v>2.897</v>
+        <v>2.263</v>
       </c>
       <c r="J4" t="n">
-        <v>0.115</v>
+        <v>0.003</v>
       </c>
       <c r="K4" t="n">
-        <v>0.05599999999999999</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>0.023</v>
+        <v>0.025</v>
       </c>
       <c r="M4" t="n">
-        <v>0.005</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="N4" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="O4" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
         <v>0.002</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.126</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
@@ -724,46 +724,46 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>9.578000000000001</v>
+        <v>6.393</v>
       </c>
       <c r="C5" t="n">
-        <v>22.686</v>
+        <v>25.875</v>
       </c>
       <c r="D5" t="n">
-        <v>4.606</v>
+        <v>9.053000000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>12.015</v>
+        <v>18.993</v>
       </c>
       <c r="F5" t="n">
-        <v>19.052</v>
+        <v>7.842000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>11.131</v>
+        <v>21.273</v>
       </c>
       <c r="H5" t="n">
-        <v>13.535</v>
+        <v>3.984</v>
       </c>
       <c r="I5" t="n">
         <v>6.212</v>
       </c>
       <c r="J5" t="n">
-        <v>0.351</v>
+        <v>0.05</v>
       </c>
       <c r="K5" t="n">
-        <v>0.215</v>
+        <v>0.062</v>
       </c>
       <c r="L5" t="n">
-        <v>0.11</v>
+        <v>0.157</v>
       </c>
       <c r="M5" t="n">
-        <v>0.015</v>
+        <v>0.043</v>
       </c>
       <c r="N5" t="n">
-        <v>0.026</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
@@ -772,7 +772,7 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>0.458</v>
+        <v>0.057</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -789,55 +789,55 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>4.79</v>
+        <v>2.45</v>
       </c>
       <c r="C6" t="n">
-        <v>15.351</v>
+        <v>18.412</v>
       </c>
       <c r="D6" t="n">
-        <v>2.117</v>
+        <v>4.251</v>
       </c>
       <c r="E6" t="n">
-        <v>18.192</v>
+        <v>12.012</v>
       </c>
       <c r="F6" t="n">
-        <v>13.511</v>
+        <v>16.671</v>
       </c>
       <c r="G6" t="n">
-        <v>15.47</v>
+        <v>24.153</v>
       </c>
       <c r="H6" t="n">
-        <v>17.014</v>
+        <v>8.466999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>10.371</v>
+        <v>12.084</v>
       </c>
       <c r="J6" t="n">
-        <v>0.873</v>
+        <v>0.132</v>
       </c>
       <c r="K6" t="n">
-        <v>0.611</v>
+        <v>0.221</v>
       </c>
       <c r="L6" t="n">
-        <v>0.4460000000000001</v>
+        <v>0.5519999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>0.079</v>
+        <v>0.273</v>
       </c>
       <c r="N6" t="n">
-        <v>0.077</v>
+        <v>0.022</v>
       </c>
       <c r="O6" t="n">
-        <v>0.041</v>
+        <v>0.027</v>
       </c>
       <c r="P6" t="n">
-        <v>0.006</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="R6" t="n">
-        <v>1.051</v>
+        <v>0.27</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -854,64 +854,64 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>2.435</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>10.018</v>
+        <v>11.088</v>
       </c>
       <c r="D7" t="n">
-        <v>0.898</v>
+        <v>1.599</v>
       </c>
       <c r="E7" t="n">
-        <v>20.128</v>
+        <v>6.02</v>
       </c>
       <c r="F7" t="n">
-        <v>9.153</v>
+        <v>25.113</v>
       </c>
       <c r="G7" t="n">
-        <v>17.408</v>
+        <v>16.152</v>
       </c>
       <c r="H7" t="n">
-        <v>17.748</v>
+        <v>15.351</v>
       </c>
       <c r="I7" t="n">
-        <v>14.729</v>
+        <v>19.183</v>
       </c>
       <c r="J7" t="n">
-        <v>1.925</v>
+        <v>0.475</v>
       </c>
       <c r="K7" t="n">
-        <v>1.424</v>
+        <v>0.6839999999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>1.237</v>
+        <v>1.489</v>
       </c>
       <c r="M7" t="n">
-        <v>0.253</v>
+        <v>0.9079999999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>0.254</v>
+        <v>0.096</v>
       </c>
       <c r="O7" t="n">
-        <v>0.122</v>
+        <v>0.107</v>
       </c>
       <c r="P7" t="n">
-        <v>0.013</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.005</v>
+        <v>0.025</v>
       </c>
       <c r="R7" t="n">
-        <v>2.245</v>
+        <v>0.8999999999999999</v>
       </c>
       <c r="S7" t="n">
         <v>0.001</v>
       </c>
       <c r="T7" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="U7" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -919,64 +919,64 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>1.081</v>
+        <v>0.226</v>
       </c>
       <c r="C8" t="n">
-        <v>5.855</v>
+        <v>6.023</v>
       </c>
       <c r="D8" t="n">
-        <v>0.411</v>
+        <v>0.528</v>
       </c>
       <c r="E8" t="n">
-        <v>18.005</v>
+        <v>2.621</v>
       </c>
       <c r="F8" t="n">
-        <v>5.527</v>
+        <v>23.166</v>
       </c>
       <c r="G8" t="n">
-        <v>17.649</v>
+        <v>8.858000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>16.247</v>
+        <v>22.414</v>
       </c>
       <c r="I8" t="n">
-        <v>18.969</v>
+        <v>22.747</v>
       </c>
       <c r="J8" t="n">
-        <v>4.008</v>
+        <v>1.518</v>
       </c>
       <c r="K8" t="n">
-        <v>3.201</v>
+        <v>1.944</v>
       </c>
       <c r="L8" t="n">
-        <v>2.686</v>
+        <v>3.615</v>
       </c>
       <c r="M8" t="n">
-        <v>0.741</v>
+        <v>2.801</v>
       </c>
       <c r="N8" t="n">
-        <v>0.741</v>
+        <v>0.422</v>
       </c>
       <c r="O8" t="n">
-        <v>0.336</v>
+        <v>0.391</v>
       </c>
       <c r="P8" t="n">
-        <v>0.064</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.016</v>
+        <v>0.107</v>
       </c>
       <c r="R8" t="n">
-        <v>4.439</v>
+        <v>2.603</v>
       </c>
       <c r="S8" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
       <c r="T8" t="n">
-        <v>0.018</v>
+        <v>0.002</v>
       </c>
       <c r="U8" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="9">
@@ -984,64 +984,64 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.378</v>
+        <v>0.046</v>
       </c>
       <c r="C9" t="n">
-        <v>2.929</v>
+        <v>2.563</v>
       </c>
       <c r="D9" t="n">
-        <v>0.143</v>
+        <v>0.175</v>
       </c>
       <c r="E9" t="n">
-        <v>13.281</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>2.954</v>
+        <v>15.703</v>
       </c>
       <c r="G9" t="n">
-        <v>13.847</v>
+        <v>4.175</v>
       </c>
       <c r="H9" t="n">
-        <v>11.752</v>
+        <v>23.455</v>
       </c>
       <c r="I9" t="n">
-        <v>20.989</v>
+        <v>21.008</v>
       </c>
       <c r="J9" t="n">
-        <v>7.593999999999999</v>
+        <v>4.06</v>
       </c>
       <c r="K9" t="n">
-        <v>6.262</v>
+        <v>4.964</v>
       </c>
       <c r="L9" t="n">
-        <v>5.709000000000001</v>
+        <v>7.317</v>
       </c>
       <c r="M9" t="n">
-        <v>2.138</v>
+        <v>6.451999999999999</v>
       </c>
       <c r="N9" t="n">
-        <v>1.968</v>
+        <v>1.434</v>
       </c>
       <c r="O9" t="n">
-        <v>1.055</v>
+        <v>1.271</v>
       </c>
       <c r="P9" t="n">
-        <v>0.283</v>
+        <v>0.035</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.077</v>
+        <v>0.382</v>
       </c>
       <c r="R9" t="n">
-        <v>8.52</v>
+        <v>5.972</v>
       </c>
       <c r="S9" t="n">
         <v>0.014</v>
       </c>
       <c r="T9" t="n">
-        <v>0.099</v>
+        <v>0.021</v>
       </c>
       <c r="U9" t="n">
-        <v>0.008</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="10">
@@ -1049,64 +1049,64 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.08099999999999999</v>
+        <v>0.003</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9979999999999999</v>
+        <v>0.729</v>
       </c>
       <c r="D10" t="n">
-        <v>0.027</v>
+        <v>0.017</v>
       </c>
       <c r="E10" t="n">
-        <v>6.081</v>
+        <v>0.197</v>
       </c>
       <c r="F10" t="n">
-        <v>1.199</v>
+        <v>5.712</v>
       </c>
       <c r="G10" t="n">
-        <v>7.571999999999999</v>
+        <v>1.301</v>
       </c>
       <c r="H10" t="n">
-        <v>5.766</v>
+        <v>12.443</v>
       </c>
       <c r="I10" t="n">
-        <v>12.62</v>
+        <v>9.275</v>
       </c>
       <c r="J10" t="n">
-        <v>14.057</v>
+        <v>10.222</v>
       </c>
       <c r="K10" t="n">
-        <v>11.396</v>
+        <v>11.427</v>
       </c>
       <c r="L10" t="n">
-        <v>11.141</v>
+        <v>13.268</v>
       </c>
       <c r="M10" t="n">
-        <v>4.889</v>
+        <v>13.045</v>
       </c>
       <c r="N10" t="n">
-        <v>4.956</v>
+        <v>3.986</v>
       </c>
       <c r="O10" t="n">
-        <v>2.889</v>
+        <v>3.704</v>
       </c>
       <c r="P10" t="n">
-        <v>0.9249999999999999</v>
+        <v>0.156</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.245</v>
+        <v>1.289</v>
       </c>
       <c r="R10" t="n">
-        <v>14.747</v>
+        <v>12.964</v>
       </c>
       <c r="S10" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.104</v>
       </c>
       <c r="T10" t="n">
-        <v>0.279</v>
+        <v>0.08800000000000001</v>
       </c>
       <c r="U10" t="n">
-        <v>0.06</v>
+        <v>0.06999999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -1114,64 +1114,64 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>0.285</v>
+        <v>0.159</v>
       </c>
       <c r="D11" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
       <c r="E11" t="n">
-        <v>2.472</v>
+        <v>0.054</v>
       </c>
       <c r="F11" t="n">
-        <v>0.427</v>
+        <v>1.934</v>
       </c>
       <c r="G11" t="n">
-        <v>3.532</v>
+        <v>0.374</v>
       </c>
       <c r="H11" t="n">
-        <v>2.67</v>
+        <v>6.347</v>
       </c>
       <c r="I11" t="n">
-        <v>6.600000000000001</v>
+        <v>4.045</v>
       </c>
       <c r="J11" t="n">
-        <v>15.606</v>
+        <v>13.279</v>
       </c>
       <c r="K11" t="n">
-        <v>14.361</v>
+        <v>13.3</v>
       </c>
       <c r="L11" t="n">
-        <v>14.535</v>
+        <v>14.558</v>
       </c>
       <c r="M11" t="n">
-        <v>8.131</v>
+        <v>15.691</v>
       </c>
       <c r="N11" t="n">
-        <v>7.933</v>
+        <v>6.877</v>
       </c>
       <c r="O11" t="n">
-        <v>4.987</v>
+        <v>5.779999999999999</v>
       </c>
       <c r="P11" t="n">
-        <v>1.988</v>
+        <v>0.5309999999999999</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.709</v>
+        <v>2.521</v>
       </c>
       <c r="R11" t="n">
-        <v>14.741</v>
+        <v>13.86</v>
       </c>
       <c r="S11" t="n">
-        <v>0.248</v>
+        <v>0.322</v>
       </c>
       <c r="T11" t="n">
-        <v>0.596</v>
+        <v>0.191</v>
       </c>
       <c r="U11" t="n">
-        <v>0.164</v>
+        <v>0.173</v>
       </c>
     </row>
     <row r="12">
@@ -1179,64 +1179,64 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0.054</v>
+        <v>0.041</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>0.8420000000000001</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="F12" t="n">
-        <v>0.118</v>
+        <v>0.644</v>
       </c>
       <c r="G12" t="n">
-        <v>1.689</v>
+        <v>0.107</v>
       </c>
       <c r="H12" t="n">
-        <v>1.15</v>
+        <v>3.023</v>
       </c>
       <c r="I12" t="n">
-        <v>3.261</v>
+        <v>1.743</v>
       </c>
       <c r="J12" t="n">
-        <v>14.479</v>
+        <v>14.313</v>
       </c>
       <c r="K12" t="n">
-        <v>14.338</v>
+        <v>13.947</v>
       </c>
       <c r="L12" t="n">
-        <v>14.703</v>
+        <v>13.77</v>
       </c>
       <c r="M12" t="n">
-        <v>10.815</v>
+        <v>15.414</v>
       </c>
       <c r="N12" t="n">
-        <v>10.661</v>
+        <v>9.757</v>
       </c>
       <c r="O12" t="n">
-        <v>7.142999999999999</v>
+        <v>7.448</v>
       </c>
       <c r="P12" t="n">
-        <v>3.581</v>
+        <v>1.139</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.448</v>
+        <v>3.885</v>
       </c>
       <c r="R12" t="n">
-        <v>13.448</v>
+        <v>13.115</v>
       </c>
       <c r="S12" t="n">
-        <v>0.65</v>
+        <v>0.711</v>
       </c>
       <c r="T12" t="n">
-        <v>1.216</v>
+        <v>0.479</v>
       </c>
       <c r="U12" t="n">
-        <v>0.402</v>
+        <v>0.457</v>
       </c>
     </row>
     <row r="13">
@@ -1247,61 +1247,61 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.014</v>
+        <v>0.004</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0.282</v>
+        <v>0.001</v>
       </c>
       <c r="F13" t="n">
-        <v>0.049</v>
+        <v>0.175</v>
       </c>
       <c r="G13" t="n">
-        <v>0.758</v>
+        <v>0.02</v>
       </c>
       <c r="H13" t="n">
-        <v>0.482</v>
+        <v>1.537</v>
       </c>
       <c r="I13" t="n">
-        <v>1.443</v>
+        <v>0.6839999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>12.539</v>
+        <v>14.244</v>
       </c>
       <c r="K13" t="n">
-        <v>13.508</v>
+        <v>13.429</v>
       </c>
       <c r="L13" t="n">
-        <v>13.813</v>
+        <v>12.501</v>
       </c>
       <c r="M13" t="n">
-        <v>12.374</v>
+        <v>13.643</v>
       </c>
       <c r="N13" t="n">
-        <v>12.328</v>
+        <v>11.745</v>
       </c>
       <c r="O13" t="n">
-        <v>9.193</v>
+        <v>9.100999999999999</v>
       </c>
       <c r="P13" t="n">
-        <v>5.24</v>
+        <v>2.093</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.511</v>
+        <v>5.513</v>
       </c>
       <c r="R13" t="n">
-        <v>11.228</v>
+        <v>12.075</v>
       </c>
       <c r="S13" t="n">
-        <v>1.302</v>
+        <v>1.396</v>
       </c>
       <c r="T13" t="n">
-        <v>2.171</v>
+        <v>0.992</v>
       </c>
       <c r="U13" t="n">
-        <v>0.765</v>
+        <v>0.847</v>
       </c>
     </row>
     <row r="14">
@@ -1312,61 +1312,61 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0.08099999999999999</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.008</v>
+        <v>0.041</v>
       </c>
       <c r="G14" t="n">
-        <v>0.278</v>
+        <v>0.01</v>
       </c>
       <c r="H14" t="n">
-        <v>0.181</v>
+        <v>0.639</v>
       </c>
       <c r="I14" t="n">
-        <v>0.617</v>
+        <v>0.235</v>
       </c>
       <c r="J14" t="n">
-        <v>9.98</v>
+        <v>13.166</v>
       </c>
       <c r="K14" t="n">
-        <v>11.348</v>
+        <v>12.042</v>
       </c>
       <c r="L14" t="n">
-        <v>11.644</v>
+        <v>10.616</v>
       </c>
       <c r="M14" t="n">
-        <v>13.443</v>
+        <v>10.978</v>
       </c>
       <c r="N14" t="n">
-        <v>13.391</v>
+        <v>13.566</v>
       </c>
       <c r="O14" t="n">
-        <v>11.037</v>
+        <v>10.947</v>
       </c>
       <c r="P14" t="n">
-        <v>7.292</v>
+        <v>3.566</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.239</v>
+        <v>7.729</v>
       </c>
       <c r="R14" t="n">
-        <v>9.027000000000001</v>
+        <v>10.511</v>
       </c>
       <c r="S14" t="n">
-        <v>2.584</v>
+        <v>2.688</v>
       </c>
       <c r="T14" t="n">
-        <v>3.399</v>
+        <v>1.783</v>
       </c>
       <c r="U14" t="n">
-        <v>1.449</v>
+        <v>1.483</v>
       </c>
     </row>
     <row r="15">
@@ -1383,55 +1383,55 @@
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G15" t="n">
-        <v>0.107</v>
+        <v>0.002</v>
       </c>
       <c r="H15" t="n">
-        <v>0.06</v>
+        <v>0.241</v>
       </c>
       <c r="I15" t="n">
-        <v>0.214</v>
+        <v>0.082</v>
       </c>
       <c r="J15" t="n">
-        <v>7.441000000000001</v>
+        <v>10.943</v>
       </c>
       <c r="K15" t="n">
-        <v>8.789</v>
+        <v>10.143</v>
       </c>
       <c r="L15" t="n">
-        <v>9.052</v>
+        <v>8.626000000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>12.921</v>
+        <v>8.478</v>
       </c>
       <c r="N15" t="n">
-        <v>13.175</v>
+        <v>14.065</v>
       </c>
       <c r="O15" t="n">
-        <v>12.463</v>
+        <v>12.347</v>
       </c>
       <c r="P15" t="n">
-        <v>9.997</v>
+        <v>5.840999999999999</v>
       </c>
       <c r="Q15" t="n">
-        <v>6.49</v>
+        <v>10.025</v>
       </c>
       <c r="R15" t="n">
-        <v>7.091</v>
+        <v>8.972</v>
       </c>
       <c r="S15" t="n">
-        <v>4.626</v>
+        <v>4.764</v>
       </c>
       <c r="T15" t="n">
-        <v>5.111000000000001</v>
+        <v>2.963</v>
       </c>
       <c r="U15" t="n">
-        <v>2.44</v>
+        <v>2.504</v>
       </c>
     </row>
     <row r="16">
@@ -1448,55 +1448,55 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>0.022</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0.016</v>
+        <v>0.083</v>
       </c>
       <c r="I16" t="n">
-        <v>0.08499999999999999</v>
+        <v>0.02</v>
       </c>
       <c r="J16" t="n">
-        <v>4.945</v>
+        <v>7.927</v>
       </c>
       <c r="K16" t="n">
-        <v>6.145</v>
+        <v>7.609000000000001</v>
       </c>
       <c r="L16" t="n">
-        <v>6.324000000000001</v>
+        <v>5.999000000000001</v>
       </c>
       <c r="M16" t="n">
-        <v>11.325</v>
+        <v>5.806999999999999</v>
       </c>
       <c r="N16" t="n">
-        <v>11.431</v>
+        <v>12.736</v>
       </c>
       <c r="O16" t="n">
-        <v>13.36</v>
+        <v>13.356</v>
       </c>
       <c r="P16" t="n">
-        <v>12.539</v>
+        <v>9.379</v>
       </c>
       <c r="Q16" t="n">
-        <v>9.260999999999999</v>
+        <v>13.095</v>
       </c>
       <c r="R16" t="n">
-        <v>5.223</v>
+        <v>7.002</v>
       </c>
       <c r="S16" t="n">
-        <v>7.599</v>
+        <v>7.907999999999999</v>
       </c>
       <c r="T16" t="n">
-        <v>7.636</v>
+        <v>4.979</v>
       </c>
       <c r="U16" t="n">
-        <v>4.085</v>
+        <v>4.100000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -1516,52 +1516,52 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0.008</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0.002</v>
+        <v>0.017</v>
       </c>
       <c r="I17" t="n">
-        <v>0.016</v>
+        <v>0.004</v>
       </c>
       <c r="J17" t="n">
-        <v>3.076</v>
+        <v>4.997999999999999</v>
       </c>
       <c r="K17" t="n">
-        <v>4.164000000000001</v>
+        <v>5.231</v>
       </c>
       <c r="L17" t="n">
-        <v>4.145</v>
+        <v>3.8</v>
       </c>
       <c r="M17" t="n">
-        <v>8.727</v>
+        <v>3.461</v>
       </c>
       <c r="N17" t="n">
-        <v>9.007999999999999</v>
+        <v>10.346</v>
       </c>
       <c r="O17" t="n">
-        <v>12.395</v>
+        <v>12.453</v>
       </c>
       <c r="P17" t="n">
-        <v>14.688</v>
+        <v>13.643</v>
       </c>
       <c r="Q17" t="n">
-        <v>12.698</v>
+        <v>14.773</v>
       </c>
       <c r="R17" t="n">
-        <v>3.468</v>
+        <v>5.115</v>
       </c>
       <c r="S17" t="n">
-        <v>11.259</v>
+        <v>11.82</v>
       </c>
       <c r="T17" t="n">
-        <v>10.225</v>
+        <v>7.779</v>
       </c>
       <c r="U17" t="n">
-        <v>6.119</v>
+        <v>6.56</v>
       </c>
     </row>
     <row r="18">
@@ -1587,46 +1587,46 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="I18" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>1.745</v>
+        <v>2.811</v>
       </c>
       <c r="K18" t="n">
-        <v>2.319</v>
+        <v>2.98</v>
       </c>
       <c r="L18" t="n">
-        <v>2.471</v>
+        <v>2.225</v>
       </c>
       <c r="M18" t="n">
-        <v>6.61</v>
+        <v>1.839</v>
       </c>
       <c r="N18" t="n">
-        <v>6.370000000000001</v>
+        <v>7.413</v>
       </c>
       <c r="O18" t="n">
-        <v>10.301</v>
+        <v>9.869</v>
       </c>
       <c r="P18" t="n">
-        <v>14.696</v>
+        <v>17.975</v>
       </c>
       <c r="Q18" t="n">
-        <v>16.149</v>
+        <v>14.426</v>
       </c>
       <c r="R18" t="n">
-        <v>2.111</v>
+        <v>3.294</v>
       </c>
       <c r="S18" t="n">
-        <v>14.659</v>
+        <v>15.669</v>
       </c>
       <c r="T18" t="n">
-        <v>13.177</v>
+        <v>11.653</v>
       </c>
       <c r="U18" t="n">
-        <v>9.388999999999999</v>
+        <v>9.843</v>
       </c>
     </row>
     <row r="19">
@@ -1658,40 +1658,40 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0.872</v>
+        <v>1.35</v>
       </c>
       <c r="K19" t="n">
-        <v>1.291</v>
+        <v>1.387</v>
       </c>
       <c r="L19" t="n">
-        <v>1.29</v>
+        <v>1.069</v>
       </c>
       <c r="M19" t="n">
-        <v>4.413</v>
+        <v>0.8330000000000001</v>
       </c>
       <c r="N19" t="n">
-        <v>4.215</v>
+        <v>4.8</v>
       </c>
       <c r="O19" t="n">
-        <v>7.788</v>
+        <v>7.123</v>
       </c>
       <c r="P19" t="n">
-        <v>12.878</v>
+        <v>19.572</v>
       </c>
       <c r="Q19" t="n">
-        <v>18.149</v>
+        <v>12.519</v>
       </c>
       <c r="R19" t="n">
-        <v>1.223</v>
+        <v>1.942</v>
       </c>
       <c r="S19" t="n">
-        <v>18.203</v>
+        <v>18.701</v>
       </c>
       <c r="T19" t="n">
-        <v>16.454</v>
+        <v>16.59</v>
       </c>
       <c r="U19" t="n">
-        <v>13.224</v>
+        <v>14.114</v>
       </c>
     </row>
     <row r="20">
@@ -1723,40 +1723,40 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0.317</v>
+        <v>0.452</v>
       </c>
       <c r="K20" t="n">
-        <v>0.482</v>
+        <v>0.507</v>
       </c>
       <c r="L20" t="n">
-        <v>0.545</v>
+        <v>0.369</v>
       </c>
       <c r="M20" t="n">
-        <v>2.492</v>
+        <v>0.286</v>
       </c>
       <c r="N20" t="n">
-        <v>2.455</v>
+        <v>2.263</v>
       </c>
       <c r="O20" t="n">
-        <v>4.984</v>
+        <v>4.379</v>
       </c>
       <c r="P20" t="n">
-        <v>10.561</v>
+        <v>17.807</v>
       </c>
       <c r="Q20" t="n">
-        <v>17.576</v>
+        <v>9.331</v>
       </c>
       <c r="R20" t="n">
-        <v>0.64</v>
+        <v>1.02</v>
       </c>
       <c r="S20" t="n">
-        <v>20.826</v>
+        <v>20.207</v>
       </c>
       <c r="T20" t="n">
-        <v>19.585</v>
+        <v>23.152</v>
       </c>
       <c r="U20" t="n">
-        <v>19.537</v>
+        <v>20.227</v>
       </c>
     </row>
     <row r="21">
@@ -1788,40 +1788,40 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0.055</v>
+        <v>0.054</v>
       </c>
       <c r="K21" t="n">
-        <v>0.08099999999999999</v>
+        <v>0.116</v>
       </c>
       <c r="L21" t="n">
-        <v>0.122</v>
+        <v>0.041</v>
       </c>
       <c r="M21" t="n">
-        <v>0.629</v>
+        <v>0.041</v>
       </c>
       <c r="N21" t="n">
-        <v>1.007</v>
+        <v>0.472</v>
       </c>
       <c r="O21" t="n">
-        <v>1.892</v>
+        <v>1.69</v>
       </c>
       <c r="P21" t="n">
-        <v>5.249000000000001</v>
+        <v>8.256</v>
       </c>
       <c r="Q21" t="n">
-        <v>10.427</v>
+        <v>4.377000000000001</v>
       </c>
       <c r="R21" t="n">
-        <v>0.199</v>
+        <v>0.326</v>
       </c>
       <c r="S21" t="n">
-        <v>17.952</v>
+        <v>15.691</v>
       </c>
       <c r="T21" t="n">
-        <v>20.031</v>
+        <v>29.327</v>
       </c>
       <c r="U21" t="n">
-        <v>42.356</v>
+        <v>39.609</v>
       </c>
     </row>
   </sheetData>
@@ -1853,141 +1853,141 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Atlético Nacional</t>
+          <t>América de Cali</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99.96800000000002</v>
+        <v>99.997</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>América de Cali</t>
+          <t>Atlético Nacional</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.90699999999998</v>
+        <v>99.979</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Deportivo Cali</t>
+          <t>Atlético Bucaramanga</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>98.64699999999999</v>
+        <v>99.74100000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Atlético Bucaramanga</t>
+          <t>Deportivo Cali</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>98.191</v>
+        <v>99.06699999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Millonarios</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>90.221</v>
+        <v>98.18600000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>89.673</v>
+        <v>91.49000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Independiente Medellín</t>
+          <t>Deportes Tolima</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>86.03399999999999</v>
+        <v>83.91199999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Independiente Medellín</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>75.14099999999999</v>
+        <v>75.667</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>Águilas Doradas</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16.854</v>
+        <v>13.158</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Llaneros</t>
+          <t>Once Caldas</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>14.888</v>
+        <v>10.484</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Águilas Doradas</t>
+          <t>Junior</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>11.778</v>
+        <v>9.804</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Once Caldas</t>
+          <t>Llaneros</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>10.215</v>
+        <v>7.882</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Internacional de Bogotá</t>
+          <t>Cúcuta Deportivo</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3.231</v>
+        <v>6.241</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cúcuta Deportivo</t>
+          <t>Internacional de Bogotá</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3.07</v>
+        <v>1.974</v>
       </c>
     </row>
     <row r="16">
@@ -1997,7 +1997,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.568</v>
+        <v>1.803</v>
       </c>
     </row>
     <row r="17">
@@ -2007,27 +2007,27 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.366</v>
+        <v>0.517</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Deportivo Pereira</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.12</v>
+        <v>0.042</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Deportivo Pereira</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.098</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="20">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.02</v>
+        <v>0.019</v>
       </c>
     </row>
     <row r="21">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.01</v>
+        <v>0.013</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar resultados de Finalizacion 2026-II hasta el 11/10/2026
- Carga 7 partidos jugados entre el 9 y el 11 de octubre (Alianza
  Valledupar 2-2 Aguilas Doradas, Once Caldas 1-0 Llaneros,
  Deportivo Pereira 0-0 Deportivo Cali, Junior 2-2 Internacional de
  Bogota, Jaguares 3-2 Deportes Tolima, Boyaca Chico 0-1 Cucuta
  Deportivo, America de Cali 1-2 Independiente Medellin) con
  actualizar_resultados.py.
- Tabla.csv/Partidos.csv/Historial_partidos.csv actualizados;
  historial pasa de 775 a 782 partidos. Tabla verificada contra
  Dimayor en vivo. Independiente Medellin sube al 5 puesto tras
  ganarle al puntero.
- model_params.csv: DrawBias recalibrado exacto (233/782).
- Resultados.xlsx/Resultado.png regenerados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resultados.xlsx
+++ b/Resultados.xlsx
@@ -445,19 +445,19 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Independiente Medellín</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Millonarios</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Santa Fe</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Independiente Medellín</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
           <t>Deportes Tolima</t>
@@ -470,19 +470,19 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>Once Caldas</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Águilas Doradas</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>Llaneros</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Águilas Doradas</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Once Caldas</t>
-        </is>
-      </c>
       <c r="N1" t="inlineStr">
         <is>
           <t>Internacional de Bogotá</t>
@@ -495,14 +495,14 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>Alianza Valledupar</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>Fortaleza</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Alianza Valledupar</t>
-        </is>
-      </c>
       <c r="R1" t="inlineStr">
         <is>
           <t>Junior</t>
@@ -510,17 +510,17 @@
       </c>
       <c r="S1" t="inlineStr">
         <is>
+          <t>Jaguares</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>Deportivo Pasto</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Deportivo Pereira</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Jaguares</t>
         </is>
       </c>
     </row>
@@ -529,31 +529,31 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>46.212</v>
+        <v>26.386</v>
       </c>
       <c r="C2" t="n">
-        <v>4.383</v>
+        <v>3.867</v>
       </c>
       <c r="D2" t="n">
-        <v>33.591</v>
+        <v>45.645</v>
       </c>
       <c r="E2" t="n">
-        <v>13.462</v>
+        <v>19.653</v>
       </c>
       <c r="F2" t="n">
-        <v>0.039</v>
+        <v>0.642</v>
       </c>
       <c r="G2" t="n">
-        <v>2.196</v>
+        <v>0.12</v>
       </c>
       <c r="H2" t="n">
-        <v>0.08599999999999999</v>
+        <v>3.685999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>0.031</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -594,37 +594,37 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>29.85</v>
+        <v>31.269</v>
       </c>
       <c r="C3" t="n">
-        <v>10.167</v>
+        <v>10.024</v>
       </c>
       <c r="D3" t="n">
-        <v>32.823</v>
+        <v>26.064</v>
       </c>
       <c r="E3" t="n">
-        <v>19.351</v>
+        <v>21.375</v>
       </c>
       <c r="F3" t="n">
-        <v>0.42</v>
+        <v>2.417</v>
       </c>
       <c r="G3" t="n">
-        <v>6.58</v>
+        <v>0.8170000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>0.419</v>
+        <v>7.999000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>0.384</v>
+        <v>0.03</v>
       </c>
       <c r="J3" t="n">
         <v>0.003</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="L3" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -659,46 +659,46 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>14.012</v>
+        <v>20.935</v>
       </c>
       <c r="C4" t="n">
-        <v>20.556</v>
+        <v>17.701</v>
       </c>
       <c r="D4" t="n">
-        <v>17.959</v>
+        <v>14.281</v>
       </c>
       <c r="E4" t="n">
-        <v>26.339</v>
+        <v>22.589</v>
       </c>
       <c r="F4" t="n">
-        <v>2.536</v>
+        <v>5.989</v>
       </c>
       <c r="G4" t="n">
-        <v>14.799</v>
+        <v>3.208</v>
       </c>
       <c r="H4" t="n">
-        <v>1.491</v>
+        <v>14.874</v>
       </c>
       <c r="I4" t="n">
-        <v>2.263</v>
+        <v>0.362</v>
       </c>
       <c r="J4" t="n">
-        <v>0.003</v>
+        <v>0.034</v>
       </c>
       <c r="K4" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.012</v>
       </c>
       <c r="L4" t="n">
-        <v>0.025</v>
+        <v>0.015</v>
       </c>
       <c r="M4" t="n">
-        <v>0.006999999999999999</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
@@ -707,7 +707,7 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
@@ -724,46 +724,46 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>6.393</v>
+        <v>11.699</v>
       </c>
       <c r="C5" t="n">
-        <v>25.875</v>
+        <v>23.533</v>
       </c>
       <c r="D5" t="n">
-        <v>9.053000000000001</v>
+        <v>7.428</v>
       </c>
       <c r="E5" t="n">
-        <v>18.993</v>
+        <v>15.749</v>
       </c>
       <c r="F5" t="n">
-        <v>7.842000000000001</v>
+        <v>11.557</v>
       </c>
       <c r="G5" t="n">
-        <v>21.273</v>
+        <v>8.358000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>3.984</v>
+        <v>19.632</v>
       </c>
       <c r="I5" t="n">
-        <v>6.212</v>
+        <v>1.724</v>
       </c>
       <c r="J5" t="n">
-        <v>0.05</v>
+        <v>0.154</v>
       </c>
       <c r="K5" t="n">
-        <v>0.062</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="L5" t="n">
-        <v>0.157</v>
+        <v>0.078</v>
       </c>
       <c r="M5" t="n">
-        <v>0.043</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>0.006</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
@@ -772,7 +772,7 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>0.057</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -789,55 +789,55 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>2.45</v>
+        <v>5.915</v>
       </c>
       <c r="C6" t="n">
-        <v>18.412</v>
+        <v>19.757</v>
       </c>
       <c r="D6" t="n">
-        <v>4.251</v>
+        <v>3.902</v>
       </c>
       <c r="E6" t="n">
-        <v>12.012</v>
+        <v>10.686</v>
       </c>
       <c r="F6" t="n">
-        <v>16.671</v>
+        <v>17.914</v>
       </c>
       <c r="G6" t="n">
-        <v>24.153</v>
+        <v>15.329</v>
       </c>
       <c r="H6" t="n">
-        <v>8.466999999999999</v>
+        <v>20.77</v>
       </c>
       <c r="I6" t="n">
-        <v>12.084</v>
+        <v>4.475</v>
       </c>
       <c r="J6" t="n">
-        <v>0.132</v>
+        <v>0.49</v>
       </c>
       <c r="K6" t="n">
-        <v>0.221</v>
+        <v>0.386</v>
       </c>
       <c r="L6" t="n">
-        <v>0.5519999999999999</v>
+        <v>0.263</v>
       </c>
       <c r="M6" t="n">
-        <v>0.273</v>
+        <v>0.058</v>
       </c>
       <c r="N6" t="n">
-        <v>0.022</v>
+        <v>0.004</v>
       </c>
       <c r="O6" t="n">
-        <v>0.027</v>
+        <v>0.002</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>0.27</v>
+        <v>0.049</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -854,61 +854,61 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0.8080000000000001</v>
+        <v>2.659</v>
       </c>
       <c r="C7" t="n">
-        <v>11.088</v>
+        <v>13.543</v>
       </c>
       <c r="D7" t="n">
-        <v>1.599</v>
+        <v>1.787</v>
       </c>
       <c r="E7" t="n">
-        <v>6.02</v>
+        <v>5.917</v>
       </c>
       <c r="F7" t="n">
-        <v>25.113</v>
+        <v>23.232</v>
       </c>
       <c r="G7" t="n">
-        <v>16.152</v>
+        <v>22.921</v>
       </c>
       <c r="H7" t="n">
-        <v>15.351</v>
+        <v>16.307</v>
       </c>
       <c r="I7" t="n">
-        <v>19.183</v>
+        <v>9.454000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>0.475</v>
+        <v>1.35</v>
       </c>
       <c r="K7" t="n">
-        <v>0.6839999999999999</v>
+        <v>1.437</v>
       </c>
       <c r="L7" t="n">
-        <v>1.489</v>
+        <v>0.868</v>
       </c>
       <c r="M7" t="n">
-        <v>0.9079999999999999</v>
+        <v>0.217</v>
       </c>
       <c r="N7" t="n">
-        <v>0.096</v>
+        <v>0.053</v>
       </c>
       <c r="O7" t="n">
-        <v>0.107</v>
+        <v>0.016</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>0.8999999999999999</v>
+        <v>0.236</v>
       </c>
       <c r="S7" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="T7" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -919,64 +919,64 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>0.226</v>
+        <v>0.9259999999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>6.023</v>
+        <v>7.782999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>0.528</v>
+        <v>0.728</v>
       </c>
       <c r="E8" t="n">
-        <v>2.621</v>
+        <v>2.963</v>
       </c>
       <c r="F8" t="n">
-        <v>23.166</v>
+        <v>21.429</v>
       </c>
       <c r="G8" t="n">
-        <v>8.858000000000001</v>
+        <v>25.86</v>
       </c>
       <c r="H8" t="n">
-        <v>22.414</v>
+        <v>10.737</v>
       </c>
       <c r="I8" t="n">
-        <v>22.747</v>
+        <v>17.771</v>
       </c>
       <c r="J8" t="n">
-        <v>1.518</v>
+        <v>3.526</v>
       </c>
       <c r="K8" t="n">
-        <v>1.944</v>
+        <v>3.747</v>
       </c>
       <c r="L8" t="n">
-        <v>3.615</v>
+        <v>2.501</v>
       </c>
       <c r="M8" t="n">
-        <v>2.801</v>
+        <v>0.715</v>
       </c>
       <c r="N8" t="n">
-        <v>0.422</v>
+        <v>0.276</v>
       </c>
       <c r="O8" t="n">
-        <v>0.391</v>
+        <v>0.038</v>
       </c>
       <c r="P8" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.022</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.107</v>
+        <v>0.003</v>
       </c>
       <c r="R8" t="n">
-        <v>2.603</v>
+        <v>0.9560000000000001</v>
       </c>
       <c r="S8" t="n">
-        <v>0.004</v>
+        <v>0.017</v>
       </c>
       <c r="T8" t="n">
         <v>0.002</v>
       </c>
       <c r="U8" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -984,64 +984,64 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.046</v>
+        <v>0.196</v>
       </c>
       <c r="C9" t="n">
-        <v>2.563</v>
+        <v>2.965</v>
       </c>
       <c r="D9" t="n">
-        <v>0.175</v>
+        <v>0.132</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.826</v>
       </c>
       <c r="F9" t="n">
-        <v>15.703</v>
+        <v>10.396</v>
       </c>
       <c r="G9" t="n">
-        <v>4.175</v>
+        <v>14.772</v>
       </c>
       <c r="H9" t="n">
-        <v>23.455</v>
+        <v>4.109999999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>21.008</v>
+        <v>31.421</v>
       </c>
       <c r="J9" t="n">
-        <v>4.06</v>
+        <v>10.314</v>
       </c>
       <c r="K9" t="n">
-        <v>4.964</v>
+        <v>9.547000000000001</v>
       </c>
       <c r="L9" t="n">
-        <v>7.317</v>
+        <v>7.087000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>6.451999999999999</v>
+        <v>2.734</v>
       </c>
       <c r="N9" t="n">
-        <v>1.434</v>
+        <v>1.253</v>
       </c>
       <c r="O9" t="n">
-        <v>1.271</v>
+        <v>0.235</v>
       </c>
       <c r="P9" t="n">
-        <v>0.035</v>
+        <v>0.111</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.382</v>
+        <v>0.019</v>
       </c>
       <c r="R9" t="n">
-        <v>5.972</v>
+        <v>3.773</v>
       </c>
       <c r="S9" t="n">
-        <v>0.014</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="T9" t="n">
-        <v>0.021</v>
+        <v>0.026</v>
       </c>
       <c r="U9" t="n">
-        <v>0.01</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="10">
@@ -1049,64 +1049,64 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.003</v>
+        <v>0.012</v>
       </c>
       <c r="C10" t="n">
-        <v>0.729</v>
+        <v>0.664</v>
       </c>
       <c r="D10" t="n">
-        <v>0.017</v>
+        <v>0.027</v>
       </c>
       <c r="E10" t="n">
-        <v>0.197</v>
+        <v>0.188</v>
       </c>
       <c r="F10" t="n">
-        <v>5.712</v>
+        <v>4.098</v>
       </c>
       <c r="G10" t="n">
-        <v>1.301</v>
+        <v>5.706</v>
       </c>
       <c r="H10" t="n">
-        <v>12.443</v>
+        <v>1.289</v>
       </c>
       <c r="I10" t="n">
-        <v>9.275</v>
+        <v>17.672</v>
       </c>
       <c r="J10" t="n">
-        <v>10.222</v>
+        <v>19.065</v>
       </c>
       <c r="K10" t="n">
-        <v>11.427</v>
+        <v>18.23</v>
       </c>
       <c r="L10" t="n">
-        <v>13.268</v>
+        <v>12.101</v>
       </c>
       <c r="M10" t="n">
-        <v>13.045</v>
+        <v>6.691</v>
       </c>
       <c r="N10" t="n">
-        <v>3.986</v>
+        <v>3.916</v>
       </c>
       <c r="O10" t="n">
-        <v>3.704</v>
+        <v>0.8710000000000001</v>
       </c>
       <c r="P10" t="n">
-        <v>0.156</v>
+        <v>0.468</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.289</v>
+        <v>0.189</v>
       </c>
       <c r="R10" t="n">
-        <v>12.964</v>
+        <v>8.398999999999999</v>
       </c>
       <c r="S10" t="n">
-        <v>0.104</v>
+        <v>0.283</v>
       </c>
       <c r="T10" t="n">
-        <v>0.08800000000000001</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="U10" t="n">
-        <v>0.06999999999999999</v>
+        <v>0.045</v>
       </c>
     </row>
     <row r="11">
@@ -1114,64 +1114,64 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="C11" t="n">
-        <v>0.159</v>
+        <v>0.138</v>
       </c>
       <c r="D11" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="E11" t="n">
-        <v>0.054</v>
+        <v>0.043</v>
       </c>
       <c r="F11" t="n">
-        <v>1.934</v>
+        <v>1.582</v>
       </c>
       <c r="G11" t="n">
-        <v>0.374</v>
+        <v>2.068</v>
       </c>
       <c r="H11" t="n">
-        <v>6.347</v>
+        <v>0.4309999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>4.045</v>
+        <v>9.146000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>13.279</v>
+        <v>19.151</v>
       </c>
       <c r="K11" t="n">
-        <v>13.3</v>
+        <v>19.995</v>
       </c>
       <c r="L11" t="n">
-        <v>14.558</v>
+        <v>13.919</v>
       </c>
       <c r="M11" t="n">
-        <v>15.691</v>
+        <v>10.216</v>
       </c>
       <c r="N11" t="n">
-        <v>6.877</v>
+        <v>7.141999999999999</v>
       </c>
       <c r="O11" t="n">
-        <v>5.779999999999999</v>
+        <v>2.026</v>
       </c>
       <c r="P11" t="n">
-        <v>0.5309999999999999</v>
+        <v>1.25</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.521</v>
+        <v>0.457</v>
       </c>
       <c r="R11" t="n">
-        <v>13.86</v>
+        <v>11.288</v>
       </c>
       <c r="S11" t="n">
-        <v>0.322</v>
+        <v>0.659</v>
       </c>
       <c r="T11" t="n">
-        <v>0.191</v>
+        <v>0.318</v>
       </c>
       <c r="U11" t="n">
-        <v>0.173</v>
+        <v>0.163</v>
       </c>
     </row>
     <row r="12">
@@ -1182,61 +1182,61 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0.041</v>
+        <v>0.024</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.008</v>
       </c>
       <c r="F12" t="n">
-        <v>0.644</v>
+        <v>0.545</v>
       </c>
       <c r="G12" t="n">
-        <v>0.107</v>
+        <v>0.65</v>
       </c>
       <c r="H12" t="n">
-        <v>3.023</v>
+        <v>0.114</v>
       </c>
       <c r="I12" t="n">
-        <v>1.743</v>
+        <v>4.508999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>14.313</v>
+        <v>16.053</v>
       </c>
       <c r="K12" t="n">
-        <v>13.947</v>
+        <v>16.631</v>
       </c>
       <c r="L12" t="n">
-        <v>13.77</v>
+        <v>14.486</v>
       </c>
       <c r="M12" t="n">
-        <v>15.414</v>
+        <v>13.197</v>
       </c>
       <c r="N12" t="n">
-        <v>9.757</v>
+        <v>11.034</v>
       </c>
       <c r="O12" t="n">
-        <v>7.448</v>
+        <v>3.507</v>
       </c>
       <c r="P12" t="n">
-        <v>1.139</v>
+        <v>2.599</v>
       </c>
       <c r="Q12" t="n">
-        <v>3.885</v>
+        <v>1.073</v>
       </c>
       <c r="R12" t="n">
-        <v>13.115</v>
+        <v>13.07</v>
       </c>
       <c r="S12" t="n">
-        <v>0.711</v>
+        <v>1.377</v>
       </c>
       <c r="T12" t="n">
-        <v>0.479</v>
+        <v>0.698</v>
       </c>
       <c r="U12" t="n">
-        <v>0.457</v>
+        <v>0.424</v>
       </c>
     </row>
     <row r="13">
@@ -1247,61 +1247,61 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="F13" t="n">
-        <v>0.175</v>
+        <v>0.157</v>
       </c>
       <c r="G13" t="n">
-        <v>0.02</v>
+        <v>0.152</v>
       </c>
       <c r="H13" t="n">
-        <v>1.537</v>
+        <v>0.037</v>
       </c>
       <c r="I13" t="n">
-        <v>0.6839999999999999</v>
+        <v>2.126</v>
       </c>
       <c r="J13" t="n">
-        <v>14.244</v>
+        <v>12.394</v>
       </c>
       <c r="K13" t="n">
-        <v>13.429</v>
+        <v>12.153</v>
       </c>
       <c r="L13" t="n">
-        <v>12.501</v>
+        <v>14.041</v>
       </c>
       <c r="M13" t="n">
-        <v>13.643</v>
+        <v>14.56</v>
       </c>
       <c r="N13" t="n">
-        <v>11.745</v>
+        <v>14.416</v>
       </c>
       <c r="O13" t="n">
-        <v>9.100999999999999</v>
+        <v>5.476</v>
       </c>
       <c r="P13" t="n">
-        <v>2.093</v>
+        <v>4.295999999999999</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.513</v>
+        <v>2.095</v>
       </c>
       <c r="R13" t="n">
-        <v>12.075</v>
+        <v>13.29</v>
       </c>
       <c r="S13" t="n">
-        <v>1.396</v>
+        <v>2.415</v>
       </c>
       <c r="T13" t="n">
-        <v>0.992</v>
+        <v>1.551</v>
       </c>
       <c r="U13" t="n">
-        <v>0.847</v>
+        <v>0.8370000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -1321,52 +1321,52 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.041</v>
+        <v>0.032</v>
       </c>
       <c r="G14" t="n">
-        <v>0.01</v>
+        <v>0.032</v>
       </c>
       <c r="H14" t="n">
-        <v>0.639</v>
+        <v>0.012</v>
       </c>
       <c r="I14" t="n">
-        <v>0.235</v>
+        <v>0.909</v>
       </c>
       <c r="J14" t="n">
-        <v>13.166</v>
+        <v>8.468999999999999</v>
       </c>
       <c r="K14" t="n">
-        <v>12.042</v>
+        <v>8.378</v>
       </c>
       <c r="L14" t="n">
-        <v>10.616</v>
+        <v>12.598</v>
       </c>
       <c r="M14" t="n">
-        <v>10.978</v>
+        <v>14.556</v>
       </c>
       <c r="N14" t="n">
-        <v>13.566</v>
+        <v>15.857</v>
       </c>
       <c r="O14" t="n">
-        <v>10.947</v>
+        <v>7.582</v>
       </c>
       <c r="P14" t="n">
-        <v>3.566</v>
+        <v>6.642</v>
       </c>
       <c r="Q14" t="n">
-        <v>7.729</v>
+        <v>3.731</v>
       </c>
       <c r="R14" t="n">
-        <v>10.511</v>
+        <v>12.889</v>
       </c>
       <c r="S14" t="n">
-        <v>2.688</v>
+        <v>3.936</v>
       </c>
       <c r="T14" t="n">
-        <v>1.783</v>
+        <v>2.726</v>
       </c>
       <c r="U14" t="n">
-        <v>1.483</v>
+        <v>1.651</v>
       </c>
     </row>
     <row r="15">
@@ -1386,52 +1386,52 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.004</v>
+        <v>0.008</v>
       </c>
       <c r="G15" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="H15" t="n">
         <v>0.002</v>
       </c>
-      <c r="H15" t="n">
-        <v>0.241</v>
-      </c>
       <c r="I15" t="n">
-        <v>0.082</v>
+        <v>0.344</v>
       </c>
       <c r="J15" t="n">
-        <v>10.943</v>
+        <v>5.118</v>
       </c>
       <c r="K15" t="n">
-        <v>10.143</v>
+        <v>5.084000000000001</v>
       </c>
       <c r="L15" t="n">
-        <v>8.626000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>8.478</v>
+        <v>12.765</v>
       </c>
       <c r="N15" t="n">
-        <v>14.065</v>
+        <v>14.97</v>
       </c>
       <c r="O15" t="n">
-        <v>12.347</v>
+        <v>10.482</v>
       </c>
       <c r="P15" t="n">
-        <v>5.840999999999999</v>
+        <v>9.324999999999999</v>
       </c>
       <c r="Q15" t="n">
-        <v>10.025</v>
+        <v>6.015000000000001</v>
       </c>
       <c r="R15" t="n">
-        <v>8.972</v>
+        <v>11.671</v>
       </c>
       <c r="S15" t="n">
-        <v>4.764</v>
+        <v>6.307</v>
       </c>
       <c r="T15" t="n">
-        <v>2.963</v>
+        <v>5.019</v>
       </c>
       <c r="U15" t="n">
-        <v>2.504</v>
+        <v>3.083</v>
       </c>
     </row>
     <row r="16">
@@ -1451,52 +1451,52 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0.083</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="J16" t="n">
-        <v>7.927</v>
+        <v>2.448</v>
       </c>
       <c r="K16" t="n">
-        <v>7.609000000000001</v>
+        <v>2.488</v>
       </c>
       <c r="L16" t="n">
-        <v>5.999000000000001</v>
+        <v>5.879</v>
       </c>
       <c r="M16" t="n">
-        <v>5.806999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="N16" t="n">
-        <v>12.736</v>
+        <v>11.615</v>
       </c>
       <c r="O16" t="n">
-        <v>13.356</v>
+        <v>13.219</v>
       </c>
       <c r="P16" t="n">
-        <v>9.379</v>
+        <v>12.873</v>
       </c>
       <c r="Q16" t="n">
-        <v>13.095</v>
+        <v>9.422000000000001</v>
       </c>
       <c r="R16" t="n">
-        <v>7.002</v>
+        <v>8.706</v>
       </c>
       <c r="S16" t="n">
-        <v>7.907999999999999</v>
+        <v>9.733000000000001</v>
       </c>
       <c r="T16" t="n">
-        <v>4.979</v>
+        <v>8.373999999999999</v>
       </c>
       <c r="U16" t="n">
-        <v>4.100000000000001</v>
+        <v>5.691</v>
       </c>
     </row>
     <row r="17">
@@ -1522,46 +1522,46 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0.017</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
         <v>0.004</v>
       </c>
       <c r="J17" t="n">
-        <v>4.997999999999999</v>
+        <v>0.984</v>
       </c>
       <c r="K17" t="n">
-        <v>5.231</v>
+        <v>1.175</v>
       </c>
       <c r="L17" t="n">
-        <v>3.8</v>
+        <v>3.383</v>
       </c>
       <c r="M17" t="n">
-        <v>3.461</v>
+        <v>6.678000000000001</v>
       </c>
       <c r="N17" t="n">
-        <v>10.346</v>
+        <v>8.363</v>
       </c>
       <c r="O17" t="n">
-        <v>12.453</v>
+        <v>14.042</v>
       </c>
       <c r="P17" t="n">
-        <v>13.643</v>
+        <v>14.856</v>
       </c>
       <c r="Q17" t="n">
-        <v>14.773</v>
+        <v>12.815</v>
       </c>
       <c r="R17" t="n">
-        <v>5.115</v>
+        <v>6.242</v>
       </c>
       <c r="S17" t="n">
-        <v>11.82</v>
+        <v>12.38</v>
       </c>
       <c r="T17" t="n">
-        <v>7.779</v>
+        <v>10.841</v>
       </c>
       <c r="U17" t="n">
-        <v>6.56</v>
+        <v>8.237</v>
       </c>
     </row>
     <row r="18">
@@ -1587,46 +1587,46 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="J18" t="n">
-        <v>2.811</v>
+        <v>0.35</v>
       </c>
       <c r="K18" t="n">
-        <v>2.98</v>
+        <v>0.485</v>
       </c>
       <c r="L18" t="n">
-        <v>2.225</v>
+        <v>1.875</v>
       </c>
       <c r="M18" t="n">
-        <v>1.839</v>
+        <v>4.305</v>
       </c>
       <c r="N18" t="n">
-        <v>7.413</v>
+        <v>5.527</v>
       </c>
       <c r="O18" t="n">
-        <v>9.869</v>
+        <v>13.643</v>
       </c>
       <c r="P18" t="n">
-        <v>17.975</v>
+        <v>14.944</v>
       </c>
       <c r="Q18" t="n">
-        <v>14.426</v>
+        <v>15.625</v>
       </c>
       <c r="R18" t="n">
-        <v>3.294</v>
+        <v>4.157999999999999</v>
       </c>
       <c r="S18" t="n">
-        <v>15.669</v>
+        <v>14.02</v>
       </c>
       <c r="T18" t="n">
-        <v>11.653</v>
+        <v>13.701</v>
       </c>
       <c r="U18" t="n">
-        <v>9.843</v>
+        <v>11.365</v>
       </c>
     </row>
     <row r="19">
@@ -1655,43 +1655,43 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="J19" t="n">
-        <v>1.35</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>1.387</v>
+        <v>0.145</v>
       </c>
       <c r="L19" t="n">
-        <v>1.069</v>
+        <v>0.804</v>
       </c>
       <c r="M19" t="n">
-        <v>0.8330000000000001</v>
+        <v>2.446</v>
       </c>
       <c r="N19" t="n">
-        <v>4.8</v>
+        <v>3.489</v>
       </c>
       <c r="O19" t="n">
-        <v>7.123</v>
+        <v>12.295</v>
       </c>
       <c r="P19" t="n">
-        <v>19.572</v>
+        <v>14.022</v>
       </c>
       <c r="Q19" t="n">
-        <v>12.519</v>
+        <v>18.111</v>
       </c>
       <c r="R19" t="n">
-        <v>1.942</v>
+        <v>2.782</v>
       </c>
       <c r="S19" t="n">
-        <v>18.701</v>
+        <v>14.817</v>
       </c>
       <c r="T19" t="n">
-        <v>16.59</v>
+        <v>16.169</v>
       </c>
       <c r="U19" t="n">
-        <v>14.114</v>
+        <v>14.835</v>
       </c>
     </row>
     <row r="20">
@@ -1723,40 +1723,40 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0.452</v>
+        <v>0.012</v>
       </c>
       <c r="K20" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
       <c r="L20" t="n">
-        <v>0.369</v>
+        <v>0.254</v>
       </c>
       <c r="M20" t="n">
-        <v>0.286</v>
+        <v>1.108</v>
       </c>
       <c r="N20" t="n">
-        <v>2.263</v>
+        <v>1.684</v>
       </c>
       <c r="O20" t="n">
-        <v>4.379</v>
+        <v>9.994</v>
       </c>
       <c r="P20" t="n">
-        <v>17.807</v>
+        <v>11.654</v>
       </c>
       <c r="Q20" t="n">
-        <v>9.331</v>
+        <v>17.921</v>
       </c>
       <c r="R20" t="n">
-        <v>1.02</v>
+        <v>1.662</v>
       </c>
       <c r="S20" t="n">
-        <v>20.207</v>
+        <v>15.784</v>
       </c>
       <c r="T20" t="n">
-        <v>23.152</v>
+        <v>19.529</v>
       </c>
       <c r="U20" t="n">
-        <v>20.227</v>
+        <v>20.37</v>
       </c>
     </row>
     <row r="21">
@@ -1788,40 +1788,40 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0.054</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0.116</v>
+        <v>0.006</v>
       </c>
       <c r="L21" t="n">
-        <v>0.041</v>
+        <v>0.047</v>
       </c>
       <c r="M21" t="n">
-        <v>0.041</v>
+        <v>0.245</v>
       </c>
       <c r="N21" t="n">
-        <v>0.472</v>
+        <v>0.401</v>
       </c>
       <c r="O21" t="n">
-        <v>1.69</v>
+        <v>6.572</v>
       </c>
       <c r="P21" t="n">
-        <v>8.256</v>
+        <v>6.937</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.377000000000001</v>
+        <v>12.524</v>
       </c>
       <c r="R21" t="n">
-        <v>0.326</v>
+        <v>0.822</v>
       </c>
       <c r="S21" t="n">
-        <v>15.691</v>
+        <v>18.198</v>
       </c>
       <c r="T21" t="n">
-        <v>29.327</v>
+        <v>20.96</v>
       </c>
       <c r="U21" t="n">
-        <v>39.609</v>
+        <v>33.288</v>
       </c>
     </row>
   </sheetData>
@@ -1857,7 +1857,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99.997</v>
+        <v>99.985</v>
       </c>
     </row>
     <row r="3">
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.979</v>
+        <v>99.96700000000001</v>
       </c>
     </row>
     <row r="4">
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>99.74100000000001</v>
+        <v>99.75800000000001</v>
       </c>
     </row>
     <row r="5">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>99.06699999999999</v>
+        <v>99.173</v>
       </c>
     </row>
     <row r="6">
@@ -1897,47 +1897,47 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>98.18600000000001</v>
+        <v>98.11500000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Millonarios</t>
+          <t>Independiente Medellín</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>91.49000000000001</v>
+        <v>93.57600000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>83.91199999999999</v>
+        <v>91.38500000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Independiente Medellín</t>
+          <t>Deportes Tolima</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>75.667</v>
+        <v>65.23699999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Águilas Doradas</t>
+          <t>Cúcuta Deportivo</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>13.158</v>
+        <v>15.872</v>
       </c>
     </row>
     <row r="11">
@@ -1947,37 +1947,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10.484</v>
+        <v>15.202</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>Águilas Doradas</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9.804</v>
+        <v>10.813</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Llaneros</t>
+          <t>Junior</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7.882</v>
+        <v>5.021</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cúcuta Deportivo</t>
+          <t>Llaneros</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6.241</v>
+        <v>3.733</v>
       </c>
     </row>
     <row r="15">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.974</v>
+        <v>1.586</v>
       </c>
     </row>
     <row r="16">
@@ -1997,7 +1997,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.803</v>
+        <v>0.291</v>
       </c>
     </row>
     <row r="17">
@@ -2007,47 +2007,47 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.517</v>
+        <v>0.134</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Jaguares</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.042</v>
+        <v>0.09100000000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Deportivo Pereira</t>
+          <t>Deportivo Pasto</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.024</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Deportivo Pasto</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.019</v>
+        <v>0.022</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Jaguares</t>
+          <t>Deportivo Pereira</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.013</v>
+        <v>0.011</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar resultados de Finalizacion 2026-II hasta el 17/10/2026
- Carga 5 partidos jugados entre el 13 y el 17 de octubre (Atletico
  Bucaramanga 1-1 Aguilas Doradas, Junior 1-1 Deportivo Pereira,
  Boyaca Chico 1-4 Atletico Nacional -el ultimo aplazado de fecha 1,
  pendiente desde julio-, Millonarios 4-1 Jaguares, Independiente
  Medellin 0-2 Once Caldas) con actualizar_resultados.py.
- Tabla.csv/Partidos.csv/Historial_partidos.csv actualizados;
  historial pasa de 782 a 787 partidos. Tabla verificada contra
  Dimayor en vivo. Atletico Nacional sube al 2 puesto (26 pts, +14).
- model_params.csv: DrawBias recalibrado exacto (235/787).
- Resultados.xlsx/Resultado.png regenerados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resultados.xlsx
+++ b/Resultados.xlsx
@@ -430,29 +430,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Atlético Nacional</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Deportivo Cali</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Atlético Nacional</t>
-        </is>
-      </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Millonarios</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Atlético Bucaramanga</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Independiente Medellín</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Millonarios</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>Santa Fe</t>
@@ -465,14 +465,14 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>Once Caldas</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>Cúcuta Deportivo</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Once Caldas</t>
-        </is>
-      </c>
       <c r="L1" t="inlineStr">
         <is>
           <t>Águilas Doradas</t>
@@ -490,37 +490,37 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>Alianza Valledupar</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>Boyacá Chicó</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Alianza Valledupar</t>
-        </is>
-      </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>Fortaleza</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
       <c r="S1" t="inlineStr">
         <is>
+          <t>Deportivo Pereira</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>Jaguares</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Deportivo Pasto</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Deportivo Pereira</t>
         </is>
       </c>
     </row>
@@ -529,31 +529,31 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>26.386</v>
+        <v>22.468</v>
       </c>
       <c r="C2" t="n">
-        <v>3.867</v>
+        <v>61.035</v>
       </c>
       <c r="D2" t="n">
-        <v>45.645</v>
+        <v>3.097</v>
       </c>
       <c r="E2" t="n">
-        <v>19.653</v>
+        <v>0.114</v>
       </c>
       <c r="F2" t="n">
-        <v>0.642</v>
+        <v>10.119</v>
       </c>
       <c r="G2" t="n">
-        <v>0.12</v>
+        <v>0.036</v>
       </c>
       <c r="H2" t="n">
-        <v>3.685999999999999</v>
+        <v>3.13</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="J2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -594,37 +594,37 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>31.269</v>
+        <v>36.838</v>
       </c>
       <c r="C3" t="n">
-        <v>10.024</v>
+        <v>23.479</v>
       </c>
       <c r="D3" t="n">
-        <v>26.064</v>
+        <v>10.823</v>
       </c>
       <c r="E3" t="n">
-        <v>21.375</v>
+        <v>1.526</v>
       </c>
       <c r="F3" t="n">
-        <v>2.417</v>
+        <v>18.597</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8170000000000001</v>
+        <v>0.299</v>
       </c>
       <c r="H3" t="n">
-        <v>7.999000000000001</v>
+        <v>8.365</v>
       </c>
       <c r="I3" t="n">
-        <v>0.03</v>
+        <v>0.062</v>
       </c>
       <c r="J3" t="n">
         <v>0.003</v>
       </c>
       <c r="K3" t="n">
-        <v>0.001</v>
+        <v>0.008</v>
       </c>
       <c r="L3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -659,40 +659,40 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>20.935</v>
+        <v>20.723</v>
       </c>
       <c r="C4" t="n">
-        <v>17.701</v>
+        <v>9.4</v>
       </c>
       <c r="D4" t="n">
-        <v>14.281</v>
+        <v>20.115</v>
       </c>
       <c r="E4" t="n">
-        <v>22.589</v>
+        <v>6.321000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>5.989</v>
+        <v>24.665</v>
       </c>
       <c r="G4" t="n">
-        <v>3.208</v>
+        <v>1.34</v>
       </c>
       <c r="H4" t="n">
-        <v>14.874</v>
+        <v>16.834</v>
       </c>
       <c r="I4" t="n">
-        <v>0.362</v>
+        <v>0.509</v>
       </c>
       <c r="J4" t="n">
-        <v>0.034</v>
+        <v>0.053</v>
       </c>
       <c r="K4" t="n">
-        <v>0.012</v>
+        <v>0.03</v>
       </c>
       <c r="L4" t="n">
-        <v>0.015</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -724,40 +724,40 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>11.699</v>
+        <v>11.056</v>
       </c>
       <c r="C5" t="n">
-        <v>23.533</v>
+        <v>3.885</v>
       </c>
       <c r="D5" t="n">
-        <v>7.428</v>
+        <v>24.257</v>
       </c>
       <c r="E5" t="n">
-        <v>15.749</v>
+        <v>14.263</v>
       </c>
       <c r="F5" t="n">
-        <v>11.557</v>
+        <v>19.432</v>
       </c>
       <c r="G5" t="n">
-        <v>8.358000000000001</v>
+        <v>4.041</v>
       </c>
       <c r="H5" t="n">
-        <v>19.632</v>
+        <v>20.436</v>
       </c>
       <c r="I5" t="n">
-        <v>1.724</v>
+        <v>2.005</v>
       </c>
       <c r="J5" t="n">
-        <v>0.154</v>
+        <v>0.398</v>
       </c>
       <c r="K5" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="L5" t="n">
-        <v>0.078</v>
+        <v>0.05599999999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -769,10 +769,10 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="R5" t="n">
-        <v>0.006999999999999999</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -789,55 +789,55 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>5.915</v>
+        <v>5.627</v>
       </c>
       <c r="C6" t="n">
-        <v>19.757</v>
+        <v>1.489</v>
       </c>
       <c r="D6" t="n">
-        <v>3.902</v>
+        <v>19.424</v>
       </c>
       <c r="E6" t="n">
-        <v>10.686</v>
+        <v>22.683</v>
       </c>
       <c r="F6" t="n">
-        <v>17.914</v>
+        <v>13.754</v>
       </c>
       <c r="G6" t="n">
-        <v>15.329</v>
+        <v>8.863999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>20.77</v>
+        <v>20.676</v>
       </c>
       <c r="I6" t="n">
-        <v>4.475</v>
+        <v>4.858</v>
       </c>
       <c r="J6" t="n">
-        <v>0.49</v>
+        <v>1.694</v>
       </c>
       <c r="K6" t="n">
-        <v>0.386</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="L6" t="n">
-        <v>0.263</v>
+        <v>0.298</v>
       </c>
       <c r="M6" t="n">
-        <v>0.058</v>
+        <v>0.062</v>
       </c>
       <c r="N6" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
         <v>0.004</v>
       </c>
-      <c r="O6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
       <c r="R6" t="n">
-        <v>0.049</v>
+        <v>0</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -854,58 +854,58 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>2.659</v>
+        <v>2.451</v>
       </c>
       <c r="C7" t="n">
-        <v>13.543</v>
+        <v>0.526</v>
       </c>
       <c r="D7" t="n">
-        <v>1.787</v>
+        <v>12.738</v>
       </c>
       <c r="E7" t="n">
-        <v>5.917</v>
+        <v>26.097</v>
       </c>
       <c r="F7" t="n">
-        <v>23.232</v>
+        <v>8.423999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>22.921</v>
+        <v>16.486</v>
       </c>
       <c r="H7" t="n">
-        <v>16.307</v>
+        <v>16.044</v>
       </c>
       <c r="I7" t="n">
-        <v>9.454000000000001</v>
+        <v>9.66</v>
       </c>
       <c r="J7" t="n">
-        <v>1.35</v>
+        <v>4.725</v>
       </c>
       <c r="K7" t="n">
-        <v>1.437</v>
+        <v>1.451</v>
       </c>
       <c r="L7" t="n">
-        <v>0.868</v>
+        <v>1.045</v>
       </c>
       <c r="M7" t="n">
-        <v>0.217</v>
+        <v>0.247</v>
       </c>
       <c r="N7" t="n">
-        <v>0.053</v>
+        <v>0.058</v>
       </c>
       <c r="O7" t="n">
-        <v>0.016</v>
+        <v>0.005</v>
       </c>
       <c r="P7" t="n">
         <v>0.001</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="R7" t="n">
-        <v>0.236</v>
+        <v>0.002</v>
       </c>
       <c r="S7" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="T7" t="n">
         <v>0</v>
@@ -919,64 +919,64 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>0.9259999999999999</v>
+        <v>0.681</v>
       </c>
       <c r="C8" t="n">
-        <v>7.782999999999999</v>
+        <v>0.149</v>
       </c>
       <c r="D8" t="n">
-        <v>0.728</v>
+        <v>6.188</v>
       </c>
       <c r="E8" t="n">
-        <v>2.963</v>
+        <v>16.195</v>
       </c>
       <c r="F8" t="n">
-        <v>21.429</v>
+        <v>3.473</v>
       </c>
       <c r="G8" t="n">
-        <v>25.86</v>
+        <v>26.814</v>
       </c>
       <c r="H8" t="n">
-        <v>10.737</v>
+        <v>8.452999999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>17.771</v>
+        <v>18.155</v>
       </c>
       <c r="J8" t="n">
-        <v>3.526</v>
+        <v>11.074</v>
       </c>
       <c r="K8" t="n">
-        <v>3.747</v>
+        <v>3.7</v>
       </c>
       <c r="L8" t="n">
-        <v>2.501</v>
+        <v>3.611</v>
       </c>
       <c r="M8" t="n">
-        <v>0.715</v>
+        <v>0.799</v>
       </c>
       <c r="N8" t="n">
-        <v>0.276</v>
+        <v>0.393</v>
       </c>
       <c r="O8" t="n">
-        <v>0.038</v>
+        <v>0.033</v>
       </c>
       <c r="P8" t="n">
-        <v>0.022</v>
+        <v>0.012</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.003</v>
+        <v>0.261</v>
       </c>
       <c r="R8" t="n">
-        <v>0.9560000000000001</v>
+        <v>0.004</v>
       </c>
       <c r="S8" t="n">
-        <v>0.017</v>
+        <v>0.002</v>
       </c>
       <c r="T8" t="n">
         <v>0.002</v>
       </c>
       <c r="U8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="9">
@@ -984,64 +984,64 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.196</v>
+        <v>0.132</v>
       </c>
       <c r="C9" t="n">
-        <v>2.965</v>
+        <v>0.032</v>
       </c>
       <c r="D9" t="n">
-        <v>0.132</v>
+        <v>2.444</v>
       </c>
       <c r="E9" t="n">
-        <v>0.826</v>
+        <v>8.173</v>
       </c>
       <c r="F9" t="n">
-        <v>10.396</v>
+        <v>1.123</v>
       </c>
       <c r="G9" t="n">
-        <v>14.772</v>
+        <v>20.485</v>
       </c>
       <c r="H9" t="n">
-        <v>4.109999999999999</v>
+        <v>3.662</v>
       </c>
       <c r="I9" t="n">
-        <v>31.421</v>
+        <v>23.835</v>
       </c>
       <c r="J9" t="n">
-        <v>10.314</v>
+        <v>20.328</v>
       </c>
       <c r="K9" t="n">
-        <v>9.547000000000001</v>
+        <v>8.218</v>
       </c>
       <c r="L9" t="n">
-        <v>7.087000000000001</v>
+        <v>6.988</v>
       </c>
       <c r="M9" t="n">
-        <v>2.734</v>
+        <v>2.166</v>
       </c>
       <c r="N9" t="n">
-        <v>1.253</v>
+        <v>1.152</v>
       </c>
       <c r="O9" t="n">
-        <v>0.235</v>
+        <v>0.097</v>
       </c>
       <c r="P9" t="n">
-        <v>0.111</v>
+        <v>0.054</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.019</v>
+        <v>1.07</v>
       </c>
       <c r="R9" t="n">
-        <v>3.773</v>
+        <v>0.018</v>
       </c>
       <c r="S9" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.008</v>
       </c>
       <c r="T9" t="n">
-        <v>0.026</v>
+        <v>0.006</v>
       </c>
       <c r="U9" t="n">
-        <v>0.011</v>
+        <v>0.009000000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -1049,64 +1049,64 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.012</v>
+        <v>0.022</v>
       </c>
       <c r="C10" t="n">
-        <v>0.664</v>
+        <v>0.005</v>
       </c>
       <c r="D10" t="n">
-        <v>0.027</v>
+        <v>0.7230000000000001</v>
       </c>
       <c r="E10" t="n">
-        <v>0.188</v>
+        <v>3.526</v>
       </c>
       <c r="F10" t="n">
-        <v>4.098</v>
+        <v>0.336</v>
       </c>
       <c r="G10" t="n">
-        <v>5.706</v>
+        <v>12.526</v>
       </c>
       <c r="H10" t="n">
-        <v>1.289</v>
+        <v>1.584</v>
       </c>
       <c r="I10" t="n">
-        <v>17.672</v>
+        <v>19.18</v>
       </c>
       <c r="J10" t="n">
-        <v>19.065</v>
+        <v>25.127</v>
       </c>
       <c r="K10" t="n">
-        <v>18.23</v>
+        <v>14.435</v>
       </c>
       <c r="L10" t="n">
-        <v>12.101</v>
+        <v>10.796</v>
       </c>
       <c r="M10" t="n">
-        <v>6.691</v>
+        <v>5.042</v>
       </c>
       <c r="N10" t="n">
-        <v>3.916</v>
+        <v>2.918</v>
       </c>
       <c r="O10" t="n">
-        <v>0.8710000000000001</v>
+        <v>0.365</v>
       </c>
       <c r="P10" t="n">
-        <v>0.468</v>
+        <v>0.202</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.189</v>
+        <v>2.953</v>
       </c>
       <c r="R10" t="n">
-        <v>8.398999999999999</v>
+        <v>0.109</v>
       </c>
       <c r="S10" t="n">
-        <v>0.283</v>
+        <v>0.039</v>
       </c>
       <c r="T10" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.053</v>
       </c>
       <c r="U10" t="n">
-        <v>0.045</v>
+        <v>0.059</v>
       </c>
     </row>
     <row r="11">
@@ -1114,64 +1114,64 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="C11" t="n">
-        <v>0.138</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>0.005</v>
+        <v>0.156</v>
       </c>
       <c r="E11" t="n">
-        <v>0.043</v>
+        <v>0.972</v>
       </c>
       <c r="F11" t="n">
-        <v>1.582</v>
+        <v>0.063</v>
       </c>
       <c r="G11" t="n">
-        <v>2.068</v>
+        <v>5.893000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4309999999999999</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>9.146000000000001</v>
+        <v>11.811</v>
       </c>
       <c r="J11" t="n">
-        <v>19.151</v>
+        <v>18.222</v>
       </c>
       <c r="K11" t="n">
-        <v>19.995</v>
+        <v>21.295</v>
       </c>
       <c r="L11" t="n">
-        <v>13.919</v>
+        <v>15.625</v>
       </c>
       <c r="M11" t="n">
-        <v>10.216</v>
+        <v>9.533999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>7.141999999999999</v>
+        <v>6.532</v>
       </c>
       <c r="O11" t="n">
-        <v>2.026</v>
+        <v>0.9730000000000001</v>
       </c>
       <c r="P11" t="n">
-        <v>1.25</v>
+        <v>0.754</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.457</v>
+        <v>6.641</v>
       </c>
       <c r="R11" t="n">
-        <v>11.288</v>
+        <v>0.415</v>
       </c>
       <c r="S11" t="n">
-        <v>0.659</v>
+        <v>0.118</v>
       </c>
       <c r="T11" t="n">
-        <v>0.318</v>
+        <v>0.214</v>
       </c>
       <c r="U11" t="n">
-        <v>0.163</v>
+        <v>0.223</v>
       </c>
     </row>
     <row r="12">
@@ -1182,61 +1182,61 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0.024</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>0.001</v>
+        <v>0.03</v>
       </c>
       <c r="E12" t="n">
-        <v>0.008</v>
+        <v>0.122</v>
       </c>
       <c r="F12" t="n">
-        <v>0.545</v>
+        <v>0.012</v>
       </c>
       <c r="G12" t="n">
-        <v>0.65</v>
+        <v>2.235</v>
       </c>
       <c r="H12" t="n">
-        <v>0.114</v>
+        <v>0.196</v>
       </c>
       <c r="I12" t="n">
-        <v>4.508999999999999</v>
+        <v>5.911</v>
       </c>
       <c r="J12" t="n">
-        <v>16.053</v>
+        <v>10.196</v>
       </c>
       <c r="K12" t="n">
-        <v>16.631</v>
+        <v>18.776</v>
       </c>
       <c r="L12" t="n">
-        <v>14.486</v>
+        <v>17.966</v>
       </c>
       <c r="M12" t="n">
-        <v>13.197</v>
+        <v>14.794</v>
       </c>
       <c r="N12" t="n">
-        <v>11.034</v>
+        <v>11.822</v>
       </c>
       <c r="O12" t="n">
-        <v>3.507</v>
+        <v>2.424</v>
       </c>
       <c r="P12" t="n">
-        <v>2.599</v>
+        <v>2.096</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.073</v>
+        <v>10.647</v>
       </c>
       <c r="R12" t="n">
-        <v>13.07</v>
+        <v>1.085</v>
       </c>
       <c r="S12" t="n">
-        <v>1.377</v>
+        <v>0.381</v>
       </c>
       <c r="T12" t="n">
-        <v>0.698</v>
+        <v>0.627</v>
       </c>
       <c r="U12" t="n">
-        <v>0.424</v>
+        <v>0.6799999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -1247,61 +1247,61 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="E13" t="n">
-        <v>0.003</v>
+        <v>0.006</v>
       </c>
       <c r="F13" t="n">
-        <v>0.157</v>
+        <v>0.002</v>
       </c>
       <c r="G13" t="n">
-        <v>0.152</v>
+        <v>0.783</v>
       </c>
       <c r="H13" t="n">
-        <v>0.037</v>
+        <v>0.055</v>
       </c>
       <c r="I13" t="n">
-        <v>2.126</v>
+        <v>2.621</v>
       </c>
       <c r="J13" t="n">
-        <v>12.394</v>
+        <v>5.000999999999999</v>
       </c>
       <c r="K13" t="n">
-        <v>12.153</v>
+        <v>14.222</v>
       </c>
       <c r="L13" t="n">
-        <v>14.041</v>
+        <v>16.219</v>
       </c>
       <c r="M13" t="n">
-        <v>14.56</v>
+        <v>16.912</v>
       </c>
       <c r="N13" t="n">
-        <v>14.416</v>
+        <v>16.177</v>
       </c>
       <c r="O13" t="n">
-        <v>5.476</v>
+        <v>4.689</v>
       </c>
       <c r="P13" t="n">
-        <v>4.295999999999999</v>
+        <v>3.866</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.095</v>
+        <v>13.001</v>
       </c>
       <c r="R13" t="n">
-        <v>13.29</v>
+        <v>2.304</v>
       </c>
       <c r="S13" t="n">
-        <v>2.415</v>
+        <v>1.041</v>
       </c>
       <c r="T13" t="n">
-        <v>1.551</v>
+        <v>1.466</v>
       </c>
       <c r="U13" t="n">
-        <v>0.8370000000000001</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="14">
@@ -1318,55 +1318,55 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="F14" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0.032</v>
+        <v>0.18</v>
       </c>
       <c r="H14" t="n">
-        <v>0.012</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>0.909</v>
+        <v>1.001</v>
       </c>
       <c r="J14" t="n">
-        <v>8.468999999999999</v>
+        <v>2.193</v>
       </c>
       <c r="K14" t="n">
-        <v>8.378</v>
+        <v>9.157999999999999</v>
       </c>
       <c r="L14" t="n">
-        <v>12.598</v>
+        <v>12.193</v>
       </c>
       <c r="M14" t="n">
-        <v>14.556</v>
+        <v>15.687</v>
       </c>
       <c r="N14" t="n">
-        <v>15.857</v>
+        <v>17.97</v>
       </c>
       <c r="O14" t="n">
-        <v>7.582</v>
+        <v>7.598000000000001</v>
       </c>
       <c r="P14" t="n">
-        <v>6.642</v>
+        <v>6.419999999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.731</v>
+        <v>14.84</v>
       </c>
       <c r="R14" t="n">
-        <v>12.889</v>
+        <v>4.294</v>
       </c>
       <c r="S14" t="n">
-        <v>3.936</v>
+        <v>2.277</v>
       </c>
       <c r="T14" t="n">
-        <v>2.726</v>
+        <v>2.834</v>
       </c>
       <c r="U14" t="n">
-        <v>1.651</v>
+        <v>3.346</v>
       </c>
     </row>
     <row r="15">
@@ -1386,52 +1386,52 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.008</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.016</v>
       </c>
       <c r="H15" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="I15" t="n">
-        <v>0.344</v>
+        <v>0.328</v>
       </c>
       <c r="J15" t="n">
-        <v>5.118</v>
+        <v>0.736</v>
       </c>
       <c r="K15" t="n">
-        <v>5.084000000000001</v>
+        <v>4.875999999999999</v>
       </c>
       <c r="L15" t="n">
-        <v>9.800000000000001</v>
+        <v>7.82</v>
       </c>
       <c r="M15" t="n">
-        <v>12.765</v>
+        <v>12.919</v>
       </c>
       <c r="N15" t="n">
-        <v>14.97</v>
+        <v>15.097</v>
       </c>
       <c r="O15" t="n">
-        <v>10.482</v>
+        <v>10.885</v>
       </c>
       <c r="P15" t="n">
-        <v>9.324999999999999</v>
+        <v>9.243</v>
       </c>
       <c r="Q15" t="n">
-        <v>6.015000000000001</v>
+        <v>15.078</v>
       </c>
       <c r="R15" t="n">
-        <v>11.671</v>
+        <v>6.887</v>
       </c>
       <c r="S15" t="n">
-        <v>6.307</v>
+        <v>4.782999999999999</v>
       </c>
       <c r="T15" t="n">
-        <v>5.019</v>
+        <v>5.081</v>
       </c>
       <c r="U15" t="n">
-        <v>3.083</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="16">
@@ -1451,10 +1451,10 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
         <v>0.002</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1463,40 +1463,40 @@
         <v>0.05</v>
       </c>
       <c r="J16" t="n">
-        <v>2.448</v>
+        <v>0.191</v>
       </c>
       <c r="K16" t="n">
-        <v>2.488</v>
+        <v>2.013</v>
       </c>
       <c r="L16" t="n">
-        <v>5.879</v>
+        <v>4.041</v>
       </c>
       <c r="M16" t="n">
-        <v>9.5</v>
+        <v>9.077</v>
       </c>
       <c r="N16" t="n">
-        <v>11.615</v>
+        <v>10.735</v>
       </c>
       <c r="O16" t="n">
-        <v>13.219</v>
+        <v>14.055</v>
       </c>
       <c r="P16" t="n">
-        <v>12.873</v>
+        <v>11.873</v>
       </c>
       <c r="Q16" t="n">
-        <v>9.422000000000001</v>
+        <v>12.008</v>
       </c>
       <c r="R16" t="n">
-        <v>8.706</v>
+        <v>10.328</v>
       </c>
       <c r="S16" t="n">
-        <v>9.733000000000001</v>
+        <v>8.371</v>
       </c>
       <c r="T16" t="n">
-        <v>8.373999999999999</v>
+        <v>8.004</v>
       </c>
       <c r="U16" t="n">
-        <v>5.691</v>
+        <v>9.252000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -1525,43 +1525,43 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>0.004</v>
+        <v>0.011</v>
       </c>
       <c r="J17" t="n">
-        <v>0.984</v>
+        <v>0.051</v>
       </c>
       <c r="K17" t="n">
-        <v>1.175</v>
+        <v>0.804</v>
       </c>
       <c r="L17" t="n">
-        <v>3.383</v>
+        <v>2.013</v>
       </c>
       <c r="M17" t="n">
-        <v>6.678000000000001</v>
+        <v>5.93</v>
       </c>
       <c r="N17" t="n">
-        <v>8.363</v>
+        <v>7.331</v>
       </c>
       <c r="O17" t="n">
-        <v>14.042</v>
+        <v>14.618</v>
       </c>
       <c r="P17" t="n">
-        <v>14.856</v>
+        <v>13.688</v>
       </c>
       <c r="Q17" t="n">
-        <v>12.815</v>
+        <v>8.747</v>
       </c>
       <c r="R17" t="n">
-        <v>6.242</v>
+        <v>13.597</v>
       </c>
       <c r="S17" t="n">
-        <v>12.38</v>
+        <v>11.33</v>
       </c>
       <c r="T17" t="n">
-        <v>10.841</v>
+        <v>10.409</v>
       </c>
       <c r="U17" t="n">
-        <v>8.237</v>
+        <v>11.471</v>
       </c>
     </row>
     <row r="18">
@@ -1590,43 +1590,43 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="J18" t="n">
-        <v>0.35</v>
+        <v>0.008</v>
       </c>
       <c r="K18" t="n">
-        <v>0.485</v>
+        <v>0.242</v>
       </c>
       <c r="L18" t="n">
-        <v>1.875</v>
+        <v>0.947</v>
       </c>
       <c r="M18" t="n">
-        <v>4.305</v>
+        <v>3.505</v>
       </c>
       <c r="N18" t="n">
-        <v>5.527</v>
+        <v>5.041</v>
       </c>
       <c r="O18" t="n">
-        <v>13.643</v>
+        <v>13.918</v>
       </c>
       <c r="P18" t="n">
-        <v>14.944</v>
+        <v>14.323</v>
       </c>
       <c r="Q18" t="n">
-        <v>15.625</v>
+        <v>6.244000000000001</v>
       </c>
       <c r="R18" t="n">
-        <v>4.157999999999999</v>
+        <v>15.499</v>
       </c>
       <c r="S18" t="n">
-        <v>14.02</v>
+        <v>13.757</v>
       </c>
       <c r="T18" t="n">
-        <v>13.701</v>
+        <v>12.899</v>
       </c>
       <c r="U18" t="n">
-        <v>11.365</v>
+        <v>13.616</v>
       </c>
     </row>
     <row r="19">
@@ -1658,40 +1658,40 @@
         <v>0.001</v>
       </c>
       <c r="J19" t="n">
-        <v>0.08400000000000001</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>0.145</v>
+        <v>0.046</v>
       </c>
       <c r="L19" t="n">
-        <v>0.804</v>
+        <v>0.28</v>
       </c>
       <c r="M19" t="n">
-        <v>2.446</v>
+        <v>2.143</v>
       </c>
       <c r="N19" t="n">
-        <v>3.489</v>
+        <v>2.984</v>
       </c>
       <c r="O19" t="n">
-        <v>12.295</v>
+        <v>12.858</v>
       </c>
       <c r="P19" t="n">
-        <v>14.022</v>
+        <v>14.256</v>
       </c>
       <c r="Q19" t="n">
-        <v>18.111</v>
+        <v>4.297</v>
       </c>
       <c r="R19" t="n">
-        <v>2.782</v>
+        <v>16.994</v>
       </c>
       <c r="S19" t="n">
-        <v>14.817</v>
+        <v>15.965</v>
       </c>
       <c r="T19" t="n">
-        <v>16.169</v>
+        <v>15.024</v>
       </c>
       <c r="U19" t="n">
-        <v>14.835</v>
+        <v>15.152</v>
       </c>
     </row>
     <row r="20">
@@ -1723,40 +1723,40 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0.012</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>0.028</v>
+        <v>0.003</v>
       </c>
       <c r="L20" t="n">
-        <v>0.254</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="M20" t="n">
-        <v>1.108</v>
+        <v>0.927</v>
       </c>
       <c r="N20" t="n">
-        <v>1.684</v>
+        <v>1.399</v>
       </c>
       <c r="O20" t="n">
-        <v>9.994</v>
+        <v>10.72</v>
       </c>
       <c r="P20" t="n">
-        <v>11.654</v>
+        <v>13.44</v>
       </c>
       <c r="Q20" t="n">
-        <v>17.921</v>
+        <v>2.863</v>
       </c>
       <c r="R20" t="n">
-        <v>1.662</v>
+        <v>16.673</v>
       </c>
       <c r="S20" t="n">
-        <v>15.784</v>
+        <v>18.7</v>
       </c>
       <c r="T20" t="n">
-        <v>19.529</v>
+        <v>17.605</v>
       </c>
       <c r="U20" t="n">
-        <v>20.37</v>
+        <v>17.586</v>
       </c>
     </row>
     <row r="21">
@@ -1791,37 +1791,37 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0.006</v>
+        <v>0.001</v>
       </c>
       <c r="L21" t="n">
-        <v>0.047</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="M21" t="n">
         <v>0.245</v>
       </c>
       <c r="N21" t="n">
-        <v>0.401</v>
+        <v>0.386</v>
       </c>
       <c r="O21" t="n">
-        <v>6.572</v>
+        <v>6.762</v>
       </c>
       <c r="P21" t="n">
-        <v>6.937</v>
+        <v>9.772</v>
       </c>
       <c r="Q21" t="n">
-        <v>12.524</v>
+        <v>1.305</v>
       </c>
       <c r="R21" t="n">
-        <v>0.822</v>
+        <v>11.791</v>
       </c>
       <c r="S21" t="n">
-        <v>18.198</v>
+        <v>23.228</v>
       </c>
       <c r="T21" t="n">
-        <v>20.96</v>
+        <v>25.776</v>
       </c>
       <c r="U21" t="n">
-        <v>33.288</v>
+        <v>20.725</v>
       </c>
     </row>
   </sheetData>
@@ -1853,21 +1853,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>América de Cali</t>
+          <t>Atlético Nacional</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99.985</v>
+        <v>99.99499999999999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Atlético Nacional</t>
+          <t>América de Cali</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.96700000000001</v>
+        <v>99.976</v>
       </c>
     </row>
     <row r="4">
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>99.75800000000001</v>
+        <v>99.58699999999999</v>
       </c>
     </row>
     <row r="5">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>99.173</v>
+        <v>99.086</v>
       </c>
     </row>
     <row r="6">
@@ -1897,27 +1897,27 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>98.11500000000001</v>
+        <v>97.59999999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Independiente Medellín</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>93.57600000000001</v>
+        <v>95.372</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Millonarios</t>
+          <t>Independiente Medellín</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>91.38500000000001</v>
+        <v>78.36499999999999</v>
       </c>
     </row>
     <row r="9">
@@ -1927,27 +1927,27 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>65.23699999999999</v>
+        <v>59.08499999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cúcuta Deportivo</t>
+          <t>Once Caldas</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15.872</v>
+        <v>38.275</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Once Caldas</t>
+          <t>Cúcuta Deportivo</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15.202</v>
+        <v>14.129</v>
       </c>
     </row>
     <row r="12">
@@ -1957,67 +1957,67 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>10.813</v>
+        <v>12.007</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>Llaneros</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5.021</v>
+        <v>3.285</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Llaneros</t>
+          <t>Internacional de Bogotá</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3.733</v>
+        <v>1.608</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Internacional de Bogotá</t>
+          <t>Junior</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.586</v>
+        <v>1.376</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Boyacá Chicó</t>
+          <t>Alianza Valledupar</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.291</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Alianza Valledupar</t>
+          <t>Boyacá Chicó</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.134</v>
+        <v>0.067</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Jaguares</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.09100000000000001</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="19">
@@ -2027,27 +2027,27 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.028</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Deportivo Pereira</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.022</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Deportivo Pereira</t>
+          <t>Jaguares</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.011</v>
+        <v>0.008</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar resultados de Finalizacion 2026-II hasta el 21/10/2026
- Carga 11 partidos jugados entre el 18 y el 21 de octubre (Aguilas
  Doradas 2-1 Deportes Tolima, Atletico Bucaramanga 1-1 America de
  Cali, Llaneros 1-0 Santa Fe, Deportivo Cali 0-0 Junior, Deportivo
  Pasto 0-1 Alianza Valledupar, Millonarios 1-1 Once Caldas,
  Deportivo Pereira 2-0 Boyaca Chico, Internacional de Bogota 2-1
  Fortaleza, Cucuta Deportivo 1-0 Atletico Nacional, Santa Fe 2-1
  Jaguares, Llaneros 0-3 Deportivo Cali) con actualizar_resultados.py.
- Tabla.csv/Partidos.csv/Historial_partidos.csv actualizados;
  historial pasa de 787 a 798 partidos. Tabla verificada contra
  Dimayor en vivo. Deportivo Cali toma la punta (29 pts) tras su
  goleada a Llaneros.
- model_params.csv: DrawBias recalibrado exacto (238/798).
- Resultados.xlsx/Resultado.png regenerados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resultados.xlsx
+++ b/Resultados.xlsx
@@ -425,19 +425,19 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Deportivo Cali</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>América de Cali</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Atlético Nacional</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Deportivo Cali</t>
-        </is>
-      </c>
       <c r="E1" t="inlineStr">
         <is>
           <t>Millonarios</t>
@@ -450,29 +450,29 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Independiente Medellín</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Cúcuta Deportivo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Once Caldas</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>Deportes Tolima</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Once Caldas</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Cúcuta Deportivo</t>
-        </is>
-      </c>
       <c r="L1" t="inlineStr">
         <is>
           <t>Águilas Doradas</t>
@@ -480,14 +480,14 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>Internacional de Bogotá</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>Llaneros</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Internacional de Bogotá</t>
-        </is>
-      </c>
       <c r="O1" t="inlineStr">
         <is>
           <t>Alianza Valledupar</t>
@@ -495,22 +495,22 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>Deportivo Pereira</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>Boyacá Chicó</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Fortaleza</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Deportivo Pereira</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
@@ -529,28 +529,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>22.468</v>
+        <v>9.411999999999999</v>
       </c>
       <c r="C2" t="n">
-        <v>61.035</v>
+        <v>33.861</v>
       </c>
       <c r="D2" t="n">
-        <v>3.097</v>
+        <v>43.972</v>
       </c>
       <c r="E2" t="n">
-        <v>0.114</v>
+        <v>0.03</v>
       </c>
       <c r="F2" t="n">
-        <v>10.119</v>
+        <v>10.821</v>
       </c>
       <c r="G2" t="n">
-        <v>0.036</v>
+        <v>1.804</v>
       </c>
       <c r="H2" t="n">
-        <v>3.13</v>
+        <v>0.096</v>
       </c>
       <c r="I2" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -594,34 +594,34 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>36.838</v>
+        <v>18.824</v>
       </c>
       <c r="C3" t="n">
-        <v>23.479</v>
+        <v>31.92</v>
       </c>
       <c r="D3" t="n">
-        <v>10.823</v>
+        <v>27.454</v>
       </c>
       <c r="E3" t="n">
-        <v>1.526</v>
+        <v>0.493</v>
       </c>
       <c r="F3" t="n">
-        <v>18.597</v>
+        <v>15.998</v>
       </c>
       <c r="G3" t="n">
-        <v>0.299</v>
+        <v>4.826</v>
       </c>
       <c r="H3" t="n">
-        <v>8.365</v>
+        <v>0.436</v>
       </c>
       <c r="I3" t="n">
-        <v>0.062</v>
+        <v>0.049</v>
       </c>
       <c r="J3" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0.008</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -659,40 +659,40 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>20.723</v>
+        <v>28.843</v>
       </c>
       <c r="C4" t="n">
-        <v>9.4</v>
+        <v>17.832</v>
       </c>
       <c r="D4" t="n">
-        <v>20.115</v>
+        <v>14.869</v>
       </c>
       <c r="E4" t="n">
-        <v>6.321000000000001</v>
+        <v>2.746</v>
       </c>
       <c r="F4" t="n">
-        <v>24.665</v>
+        <v>23.268</v>
       </c>
       <c r="G4" t="n">
-        <v>1.34</v>
+        <v>10.723</v>
       </c>
       <c r="H4" t="n">
-        <v>16.834</v>
+        <v>1.459</v>
       </c>
       <c r="I4" t="n">
-        <v>0.509</v>
+        <v>0.21</v>
       </c>
       <c r="J4" t="n">
-        <v>0.053</v>
+        <v>0.005</v>
       </c>
       <c r="K4" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="L4" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.025</v>
       </c>
       <c r="M4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -724,40 +724,40 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>11.056</v>
+        <v>26.013</v>
       </c>
       <c r="C5" t="n">
-        <v>3.885</v>
+        <v>10.501</v>
       </c>
       <c r="D5" t="n">
-        <v>24.257</v>
+        <v>8.302</v>
       </c>
       <c r="E5" t="n">
-        <v>14.263</v>
+        <v>8.669</v>
       </c>
       <c r="F5" t="n">
-        <v>19.432</v>
+        <v>23.094</v>
       </c>
       <c r="G5" t="n">
-        <v>4.041</v>
+        <v>17.945</v>
       </c>
       <c r="H5" t="n">
-        <v>20.436</v>
+        <v>4.082</v>
       </c>
       <c r="I5" t="n">
-        <v>2.005</v>
+        <v>0.869</v>
       </c>
       <c r="J5" t="n">
-        <v>0.398</v>
+        <v>0.149</v>
       </c>
       <c r="K5" t="n">
-        <v>0.16</v>
+        <v>0.232</v>
       </c>
       <c r="L5" t="n">
-        <v>0.05599999999999999</v>
+        <v>0.144</v>
       </c>
       <c r="M5" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -769,7 +769,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -789,40 +789,40 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>5.627</v>
+        <v>11.463</v>
       </c>
       <c r="C6" t="n">
-        <v>1.489</v>
+        <v>3.899</v>
       </c>
       <c r="D6" t="n">
-        <v>19.424</v>
+        <v>3.606</v>
       </c>
       <c r="E6" t="n">
-        <v>22.683</v>
+        <v>22.001</v>
       </c>
       <c r="F6" t="n">
-        <v>13.754</v>
+        <v>14.685</v>
       </c>
       <c r="G6" t="n">
-        <v>8.863999999999999</v>
+        <v>27.529</v>
       </c>
       <c r="H6" t="n">
-        <v>20.676</v>
+        <v>10.372</v>
       </c>
       <c r="I6" t="n">
-        <v>4.858</v>
+        <v>2.9</v>
       </c>
       <c r="J6" t="n">
-        <v>1.694</v>
+        <v>1.122</v>
       </c>
       <c r="K6" t="n">
-        <v>0.5620000000000001</v>
+        <v>1.499</v>
       </c>
       <c r="L6" t="n">
-        <v>0.298</v>
+        <v>0.905</v>
       </c>
       <c r="M6" t="n">
-        <v>0.062</v>
+        <v>0.014</v>
       </c>
       <c r="N6" t="n">
         <v>0.005</v>
@@ -834,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -854,55 +854,55 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>2.451</v>
+        <v>4.122</v>
       </c>
       <c r="C7" t="n">
-        <v>0.526</v>
+        <v>1.443</v>
       </c>
       <c r="D7" t="n">
-        <v>12.738</v>
+        <v>1.249</v>
       </c>
       <c r="E7" t="n">
-        <v>26.097</v>
+        <v>30.589</v>
       </c>
       <c r="F7" t="n">
-        <v>8.423999999999999</v>
+        <v>7.663</v>
       </c>
       <c r="G7" t="n">
-        <v>16.486</v>
+        <v>19.338</v>
       </c>
       <c r="H7" t="n">
-        <v>16.044</v>
+        <v>17.904</v>
       </c>
       <c r="I7" t="n">
-        <v>9.66</v>
+        <v>6.074</v>
       </c>
       <c r="J7" t="n">
-        <v>4.725</v>
+        <v>4.16</v>
       </c>
       <c r="K7" t="n">
-        <v>1.451</v>
+        <v>4.566</v>
       </c>
       <c r="L7" t="n">
-        <v>1.045</v>
+        <v>2.655</v>
       </c>
       <c r="M7" t="n">
-        <v>0.247</v>
+        <v>0.148</v>
       </c>
       <c r="N7" t="n">
-        <v>0.058</v>
+        <v>0.052</v>
       </c>
       <c r="O7" t="n">
-        <v>0.005</v>
+        <v>0.033</v>
       </c>
       <c r="P7" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.04</v>
+        <v>0.004</v>
       </c>
       <c r="R7" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
         <v>0</v>
@@ -919,64 +919,64 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>0.681</v>
+        <v>1.108</v>
       </c>
       <c r="C8" t="n">
-        <v>0.149</v>
+        <v>0.427</v>
       </c>
       <c r="D8" t="n">
-        <v>6.188</v>
+        <v>0.426</v>
       </c>
       <c r="E8" t="n">
-        <v>16.195</v>
+        <v>20.197</v>
       </c>
       <c r="F8" t="n">
-        <v>3.473</v>
+        <v>3.179</v>
       </c>
       <c r="G8" t="n">
-        <v>26.814</v>
+        <v>10.15</v>
       </c>
       <c r="H8" t="n">
-        <v>8.452999999999999</v>
+        <v>23.887</v>
       </c>
       <c r="I8" t="n">
-        <v>18.155</v>
+        <v>10.969</v>
       </c>
       <c r="J8" t="n">
-        <v>11.074</v>
+        <v>11.823</v>
       </c>
       <c r="K8" t="n">
-        <v>3.7</v>
+        <v>9.908999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>3.611</v>
+        <v>6.754</v>
       </c>
       <c r="M8" t="n">
-        <v>0.799</v>
+        <v>0.637</v>
       </c>
       <c r="N8" t="n">
-        <v>0.393</v>
+        <v>0.334</v>
       </c>
       <c r="O8" t="n">
-        <v>0.033</v>
+        <v>0.105</v>
       </c>
       <c r="P8" t="n">
-        <v>0.012</v>
+        <v>0.001</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.261</v>
+        <v>0.094</v>
       </c>
       <c r="R8" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -984,64 +984,64 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.132</v>
+        <v>0.188</v>
       </c>
       <c r="C9" t="n">
-        <v>0.032</v>
+        <v>0.098</v>
       </c>
       <c r="D9" t="n">
-        <v>2.444</v>
+        <v>0.094</v>
       </c>
       <c r="E9" t="n">
-        <v>8.173</v>
+        <v>9.610000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>1.123</v>
+        <v>0.9329999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>20.485</v>
+        <v>4.567</v>
       </c>
       <c r="H9" t="n">
-        <v>3.662</v>
+        <v>16.968</v>
       </c>
       <c r="I9" t="n">
-        <v>23.835</v>
+        <v>17.278</v>
       </c>
       <c r="J9" t="n">
-        <v>20.328</v>
+        <v>19.9</v>
       </c>
       <c r="K9" t="n">
-        <v>8.218</v>
+        <v>16.182</v>
       </c>
       <c r="L9" t="n">
-        <v>6.988</v>
+        <v>10.258</v>
       </c>
       <c r="M9" t="n">
-        <v>2.166</v>
+        <v>1.711</v>
       </c>
       <c r="N9" t="n">
-        <v>1.152</v>
+        <v>1.235</v>
       </c>
       <c r="O9" t="n">
-        <v>0.097</v>
+        <v>0.352</v>
       </c>
       <c r="P9" t="n">
-        <v>0.054</v>
+        <v>0.014</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.07</v>
+        <v>0.611</v>
       </c>
       <c r="R9" t="n">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0.008</v>
+        <v>0.001</v>
       </c>
       <c r="T9" t="n">
-        <v>0.006</v>
+        <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>0.009000000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1049,64 +1049,64 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.022</v>
+        <v>0.027</v>
       </c>
       <c r="C10" t="n">
-        <v>0.005</v>
+        <v>0.016</v>
       </c>
       <c r="D10" t="n">
-        <v>0.7230000000000001</v>
+        <v>0.026</v>
       </c>
       <c r="E10" t="n">
-        <v>3.526</v>
+        <v>4.175</v>
       </c>
       <c r="F10" t="n">
-        <v>0.336</v>
+        <v>0.291</v>
       </c>
       <c r="G10" t="n">
-        <v>12.526</v>
+        <v>2.066</v>
       </c>
       <c r="H10" t="n">
-        <v>1.584</v>
+        <v>11.464</v>
       </c>
       <c r="I10" t="n">
-        <v>19.18</v>
+        <v>17.913</v>
       </c>
       <c r="J10" t="n">
-        <v>25.127</v>
+        <v>21.456</v>
       </c>
       <c r="K10" t="n">
-        <v>14.435</v>
+        <v>20.153</v>
       </c>
       <c r="L10" t="n">
-        <v>10.796</v>
+        <v>13.113</v>
       </c>
       <c r="M10" t="n">
-        <v>5.042</v>
+        <v>3.693</v>
       </c>
       <c r="N10" t="n">
-        <v>2.918</v>
+        <v>3.104</v>
       </c>
       <c r="O10" t="n">
-        <v>0.365</v>
+        <v>0.786</v>
       </c>
       <c r="P10" t="n">
-        <v>0.202</v>
+        <v>0.061</v>
       </c>
       <c r="Q10" t="n">
-        <v>2.953</v>
+        <v>1.626</v>
       </c>
       <c r="R10" t="n">
-        <v>0.109</v>
+        <v>0.016</v>
       </c>
       <c r="S10" t="n">
-        <v>0.039</v>
+        <v>0.012</v>
       </c>
       <c r="T10" t="n">
-        <v>0.053</v>
+        <v>0.002</v>
       </c>
       <c r="U10" t="n">
-        <v>0.059</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1114,64 +1114,64 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D11" t="n">
         <v>0.002</v>
       </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.156</v>
-      </c>
       <c r="E11" t="n">
-        <v>0.972</v>
+        <v>1.286</v>
       </c>
       <c r="F11" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
       <c r="G11" t="n">
-        <v>5.893000000000001</v>
+        <v>0.8049999999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>0.5570000000000001</v>
+        <v>7.113</v>
       </c>
       <c r="I11" t="n">
-        <v>11.811</v>
+        <v>16.926</v>
       </c>
       <c r="J11" t="n">
-        <v>18.222</v>
+        <v>18.174</v>
       </c>
       <c r="K11" t="n">
-        <v>21.295</v>
+        <v>20.626</v>
       </c>
       <c r="L11" t="n">
-        <v>15.625</v>
+        <v>16.124</v>
       </c>
       <c r="M11" t="n">
-        <v>9.533999999999999</v>
+        <v>6.941</v>
       </c>
       <c r="N11" t="n">
-        <v>6.532</v>
+        <v>6.31</v>
       </c>
       <c r="O11" t="n">
-        <v>0.9730000000000001</v>
+        <v>1.862</v>
       </c>
       <c r="P11" t="n">
-        <v>0.754</v>
+        <v>0.15</v>
       </c>
       <c r="Q11" t="n">
-        <v>6.641</v>
+        <v>3.494</v>
       </c>
       <c r="R11" t="n">
-        <v>0.415</v>
+        <v>0.059</v>
       </c>
       <c r="S11" t="n">
-        <v>0.118</v>
+        <v>0.025</v>
       </c>
       <c r="T11" t="n">
-        <v>0.214</v>
+        <v>0.03</v>
       </c>
       <c r="U11" t="n">
-        <v>0.223</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="12">
@@ -1185,58 +1185,58 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>0.122</v>
+        <v>0.192</v>
       </c>
       <c r="F12" t="n">
-        <v>0.012</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>2.235</v>
+        <v>0.201</v>
       </c>
       <c r="H12" t="n">
-        <v>0.196</v>
+        <v>3.844</v>
       </c>
       <c r="I12" t="n">
-        <v>5.911</v>
+        <v>13.388</v>
       </c>
       <c r="J12" t="n">
-        <v>10.196</v>
+        <v>12.248</v>
       </c>
       <c r="K12" t="n">
-        <v>18.776</v>
+        <v>14.075</v>
       </c>
       <c r="L12" t="n">
-        <v>17.966</v>
+        <v>19.151</v>
       </c>
       <c r="M12" t="n">
-        <v>14.794</v>
+        <v>12.527</v>
       </c>
       <c r="N12" t="n">
-        <v>11.822</v>
+        <v>12.139</v>
       </c>
       <c r="O12" t="n">
-        <v>2.424</v>
+        <v>4.233</v>
       </c>
       <c r="P12" t="n">
-        <v>2.096</v>
+        <v>0.428</v>
       </c>
       <c r="Q12" t="n">
-        <v>10.647</v>
+        <v>7.045999999999999</v>
       </c>
       <c r="R12" t="n">
-        <v>1.085</v>
+        <v>0.251</v>
       </c>
       <c r="S12" t="n">
-        <v>0.381</v>
+        <v>0.132</v>
       </c>
       <c r="T12" t="n">
-        <v>0.627</v>
+        <v>0.107</v>
       </c>
       <c r="U12" t="n">
-        <v>0.6799999999999999</v>
+        <v>0.031</v>
       </c>
     </row>
     <row r="13">
@@ -1250,58 +1250,58 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0.006</v>
+        <v>0.012</v>
       </c>
       <c r="F13" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G13" t="n">
-        <v>0.783</v>
+        <v>0.041</v>
       </c>
       <c r="H13" t="n">
-        <v>0.055</v>
+        <v>1.715</v>
       </c>
       <c r="I13" t="n">
-        <v>2.621</v>
+        <v>8.054</v>
       </c>
       <c r="J13" t="n">
-        <v>5.000999999999999</v>
+        <v>6.63</v>
       </c>
       <c r="K13" t="n">
-        <v>14.222</v>
+        <v>7.834000000000001</v>
       </c>
       <c r="L13" t="n">
-        <v>16.219</v>
+        <v>15.219</v>
       </c>
       <c r="M13" t="n">
-        <v>16.912</v>
+        <v>19.333</v>
       </c>
       <c r="N13" t="n">
-        <v>16.177</v>
+        <v>19.069</v>
       </c>
       <c r="O13" t="n">
-        <v>4.689</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="P13" t="n">
-        <v>3.866</v>
+        <v>1.119</v>
       </c>
       <c r="Q13" t="n">
-        <v>13.001</v>
+        <v>11.021</v>
       </c>
       <c r="R13" t="n">
-        <v>2.304</v>
+        <v>0.931</v>
       </c>
       <c r="S13" t="n">
-        <v>1.041</v>
+        <v>0.415</v>
       </c>
       <c r="T13" t="n">
-        <v>1.466</v>
+        <v>0.368</v>
       </c>
       <c r="U13" t="n">
-        <v>1.63</v>
+        <v>0.118</v>
       </c>
     </row>
     <row r="14">
@@ -1318,55 +1318,55 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0.18</v>
+        <v>0.005</v>
       </c>
       <c r="H14" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.573</v>
       </c>
       <c r="I14" t="n">
-        <v>1.001</v>
+        <v>3.892</v>
       </c>
       <c r="J14" t="n">
-        <v>2.193</v>
+        <v>3.031</v>
       </c>
       <c r="K14" t="n">
-        <v>9.157999999999999</v>
+        <v>3.445</v>
       </c>
       <c r="L14" t="n">
-        <v>12.193</v>
+        <v>9.463000000000001</v>
       </c>
       <c r="M14" t="n">
-        <v>15.687</v>
+        <v>21.656</v>
       </c>
       <c r="N14" t="n">
-        <v>17.97</v>
+        <v>21.459</v>
       </c>
       <c r="O14" t="n">
-        <v>7.598000000000001</v>
+        <v>13.625</v>
       </c>
       <c r="P14" t="n">
-        <v>6.419999999999999</v>
+        <v>2.794</v>
       </c>
       <c r="Q14" t="n">
-        <v>14.84</v>
+        <v>15.646</v>
       </c>
       <c r="R14" t="n">
-        <v>4.294</v>
+        <v>2.131</v>
       </c>
       <c r="S14" t="n">
-        <v>2.277</v>
+        <v>0.9480000000000001</v>
       </c>
       <c r="T14" t="n">
-        <v>2.834</v>
+        <v>0.9490000000000001</v>
       </c>
       <c r="U14" t="n">
-        <v>3.346</v>
+        <v>0.383</v>
       </c>
     </row>
     <row r="15">
@@ -1389,49 +1389,49 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0.016</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>0.001</v>
+        <v>0.08</v>
       </c>
       <c r="I15" t="n">
-        <v>0.328</v>
+        <v>1.23</v>
       </c>
       <c r="J15" t="n">
-        <v>0.736</v>
+        <v>0.991</v>
       </c>
       <c r="K15" t="n">
-        <v>4.875999999999999</v>
+        <v>1.143</v>
       </c>
       <c r="L15" t="n">
-        <v>7.82</v>
+        <v>4.383</v>
       </c>
       <c r="M15" t="n">
-        <v>12.919</v>
+        <v>16.415</v>
       </c>
       <c r="N15" t="n">
-        <v>15.097</v>
+        <v>17.475</v>
       </c>
       <c r="O15" t="n">
-        <v>10.885</v>
+        <v>19.388</v>
       </c>
       <c r="P15" t="n">
-        <v>9.243</v>
+        <v>7.628</v>
       </c>
       <c r="Q15" t="n">
-        <v>15.078</v>
+        <v>20.003</v>
       </c>
       <c r="R15" t="n">
-        <v>6.887</v>
+        <v>4.434</v>
       </c>
       <c r="S15" t="n">
-        <v>4.782999999999999</v>
+        <v>2.715</v>
       </c>
       <c r="T15" t="n">
-        <v>5.081</v>
+        <v>2.785</v>
       </c>
       <c r="U15" t="n">
-        <v>6.25</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="16">
@@ -1454,49 +1454,49 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>0.05</v>
+        <v>0.223</v>
       </c>
       <c r="J16" t="n">
-        <v>0.191</v>
+        <v>0.27</v>
       </c>
       <c r="K16" t="n">
-        <v>2.013</v>
+        <v>0.266</v>
       </c>
       <c r="L16" t="n">
-        <v>4.041</v>
+        <v>1.415</v>
       </c>
       <c r="M16" t="n">
-        <v>9.077</v>
+        <v>10.054</v>
       </c>
       <c r="N16" t="n">
-        <v>10.735</v>
+        <v>11.1</v>
       </c>
       <c r="O16" t="n">
-        <v>14.055</v>
+        <v>21.83</v>
       </c>
       <c r="P16" t="n">
-        <v>11.873</v>
+        <v>14.961</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.008</v>
+        <v>17.108</v>
       </c>
       <c r="R16" t="n">
-        <v>10.328</v>
+        <v>7.631</v>
       </c>
       <c r="S16" t="n">
-        <v>8.371</v>
+        <v>5.972</v>
       </c>
       <c r="T16" t="n">
-        <v>8.004</v>
+        <v>6.065</v>
       </c>
       <c r="U16" t="n">
-        <v>9.252000000000001</v>
+        <v>3.098</v>
       </c>
     </row>
     <row r="17">
@@ -1525,43 +1525,43 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>0.011</v>
+        <v>0.02</v>
       </c>
       <c r="J17" t="n">
-        <v>0.051</v>
+        <v>0.039</v>
       </c>
       <c r="K17" t="n">
-        <v>0.804</v>
+        <v>0.047</v>
       </c>
       <c r="L17" t="n">
-        <v>2.013</v>
+        <v>0.342</v>
       </c>
       <c r="M17" t="n">
-        <v>5.93</v>
+        <v>4.693</v>
       </c>
       <c r="N17" t="n">
-        <v>7.331</v>
+        <v>5.067</v>
       </c>
       <c r="O17" t="n">
-        <v>14.618</v>
+        <v>15.544</v>
       </c>
       <c r="P17" t="n">
-        <v>13.688</v>
+        <v>22.359</v>
       </c>
       <c r="Q17" t="n">
-        <v>8.747</v>
+        <v>10.768</v>
       </c>
       <c r="R17" t="n">
-        <v>13.597</v>
+        <v>12.115</v>
       </c>
       <c r="S17" t="n">
-        <v>11.33</v>
+        <v>11.848</v>
       </c>
       <c r="T17" t="n">
-        <v>10.409</v>
+        <v>10.573</v>
       </c>
       <c r="U17" t="n">
-        <v>11.471</v>
+        <v>6.585000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -1593,40 +1593,40 @@
         <v>0.001</v>
       </c>
       <c r="J18" t="n">
-        <v>0.008</v>
+        <v>0.002</v>
       </c>
       <c r="K18" t="n">
-        <v>0.242</v>
+        <v>0.003</v>
       </c>
       <c r="L18" t="n">
-        <v>0.947</v>
+        <v>0.044</v>
       </c>
       <c r="M18" t="n">
-        <v>3.505</v>
+        <v>1.709</v>
       </c>
       <c r="N18" t="n">
-        <v>5.041</v>
+        <v>1.974</v>
       </c>
       <c r="O18" t="n">
-        <v>13.918</v>
+        <v>8.477</v>
       </c>
       <c r="P18" t="n">
-        <v>14.323</v>
+        <v>19.69</v>
       </c>
       <c r="Q18" t="n">
-        <v>6.244000000000001</v>
+        <v>6.463000000000001</v>
       </c>
       <c r="R18" t="n">
-        <v>15.499</v>
+        <v>18.455</v>
       </c>
       <c r="S18" t="n">
-        <v>13.757</v>
+        <v>17.894</v>
       </c>
       <c r="T18" t="n">
-        <v>12.899</v>
+        <v>14.18</v>
       </c>
       <c r="U18" t="n">
-        <v>13.616</v>
+        <v>11.108</v>
       </c>
     </row>
     <row r="19">
@@ -1655,43 +1655,43 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>0.046</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>0.28</v>
+        <v>0.005</v>
       </c>
       <c r="M19" t="n">
-        <v>2.143</v>
+        <v>0.404</v>
       </c>
       <c r="N19" t="n">
-        <v>2.984</v>
+        <v>0.5950000000000001</v>
       </c>
       <c r="O19" t="n">
-        <v>12.858</v>
+        <v>4.048999999999999</v>
       </c>
       <c r="P19" t="n">
-        <v>14.256</v>
+        <v>15.442</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.297</v>
+        <v>3.566</v>
       </c>
       <c r="R19" t="n">
-        <v>16.994</v>
+        <v>20.874</v>
       </c>
       <c r="S19" t="n">
-        <v>15.965</v>
+        <v>21.647</v>
       </c>
       <c r="T19" t="n">
-        <v>15.024</v>
+        <v>17.305</v>
       </c>
       <c r="U19" t="n">
-        <v>15.152</v>
+        <v>16.113</v>
       </c>
     </row>
     <row r="20">
@@ -1726,37 +1726,37 @@
         <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>0.08400000000000001</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>0.927</v>
+        <v>0.065</v>
       </c>
       <c r="N20" t="n">
-        <v>1.399</v>
+        <v>0.075</v>
       </c>
       <c r="O20" t="n">
-        <v>10.72</v>
+        <v>1.386</v>
       </c>
       <c r="P20" t="n">
-        <v>13.44</v>
+        <v>10.804</v>
       </c>
       <c r="Q20" t="n">
-        <v>2.863</v>
+        <v>1.878</v>
       </c>
       <c r="R20" t="n">
-        <v>16.673</v>
+        <v>20.437</v>
       </c>
       <c r="S20" t="n">
-        <v>18.7</v>
+        <v>22.968</v>
       </c>
       <c r="T20" t="n">
-        <v>17.605</v>
+        <v>20.525</v>
       </c>
       <c r="U20" t="n">
-        <v>17.586</v>
+        <v>21.862</v>
       </c>
     </row>
     <row r="21">
@@ -1791,37 +1791,37 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>0.009000000000000001</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>0.245</v>
+        <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>0.386</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="O21" t="n">
-        <v>6.762</v>
+        <v>0.21</v>
       </c>
       <c r="P21" t="n">
-        <v>9.772</v>
+        <v>4.549</v>
       </c>
       <c r="Q21" t="n">
-        <v>1.305</v>
+        <v>0.672</v>
       </c>
       <c r="R21" t="n">
-        <v>11.791</v>
+        <v>12.666</v>
       </c>
       <c r="S21" t="n">
-        <v>23.228</v>
+        <v>15.423</v>
       </c>
       <c r="T21" t="n">
-        <v>25.776</v>
+        <v>27.111</v>
       </c>
       <c r="U21" t="n">
-        <v>20.725</v>
+        <v>39.362</v>
       </c>
     </row>
   </sheetData>
@@ -1853,41 +1853,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Atlético Nacional</t>
+          <t>América de Cali</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99.99499999999999</v>
+        <v>99.98100000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>América de Cali</t>
+          <t>Deportivo Cali</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.976</v>
+        <v>99.973</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Atlético Bucaramanga</t>
+          <t>Atlético Nacional</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>99.58699999999999</v>
+        <v>99.97200000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Deportivo Cali</t>
+          <t>Atlético Bucaramanga</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>99.086</v>
+        <v>99.64100000000002</v>
       </c>
     </row>
     <row r="6">
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>97.59999999999999</v>
+        <v>96.88200000000001</v>
       </c>
     </row>
     <row r="7">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>95.372</v>
+        <v>94.33500000000001</v>
       </c>
     </row>
     <row r="8">
@@ -1917,17 +1917,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>78.36499999999999</v>
+        <v>75.20400000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Cúcuta Deportivo</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>59.08499999999999</v>
+        <v>38.353</v>
       </c>
     </row>
     <row r="10">
@@ -1937,17 +1937,17 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>38.275</v>
+        <v>37.15900000000001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Cúcuta Deportivo</t>
+          <t>Deportes Tolima</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>14.129</v>
+        <v>32.408</v>
       </c>
     </row>
     <row r="12">
@@ -1957,27 +1957,27 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12.007</v>
+        <v>20.741</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Llaneros</t>
+          <t>Internacional de Bogotá</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3.285</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Internacional de Bogotá</t>
+          <t>Llaneros</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.608</v>
+        <v>1.626</v>
       </c>
     </row>
     <row r="15">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.376</v>
+        <v>0.709</v>
       </c>
     </row>
     <row r="16">
@@ -1997,17 +1997,17 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.135</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Boyacá Chicó</t>
+          <t>Deportivo Pereira</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.067</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="18">
@@ -2017,37 +2017,37 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.024</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Deportivo Pasto</t>
+          <t>Boyacá Chicó</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Deportivo Pereira</t>
+          <t>Jaguares</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Jaguares</t>
+          <t>Deportivo Pasto</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.008</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar resultados de Finalizacion 2026-II hasta el 27/10/2026
- Carga 13 partidos jugados entre el 22 y el 27 de octubre (Atletico
  Nacional 3-0 Deportivo Pasto, Boyaca Chico 1-0 Atletico
  Bucaramanga, Junior 1-0 Aguilas Doradas, America de Cali 3-1
  Cucuta Deportivo, Once Caldas 1-1 Deportivo Pereira, Fortaleza 1-1
  Deportivo Cali, Alianza Valledupar 1-0 Internacional de Bogota,
  Atletico Nacional 2-1 Independiente Medellin, Deportes Tolima 0-1
  Deportivo Pasto, Santa Fe 2-1 Atletico Bucaramanga, Jaguares 1-0
  Llaneros, Cucuta Deportivo 0-2 Aguilas Doradas, Boyaca Chico 1-1
  Junior) con actualizar_resultados.py.
- Tabla.csv/Partidos.csv/Historial_partidos.csv actualizados;
  historial pasa de 798 a 811 partidos. Tabla verificada contra
  Dimayor en vivo. Atletico Nacional toma la punta (32 pts, +17).
- model_params.csv: DrawBias recalibrado exacto (241/811).
- Resultados.xlsx/Resultado.png regenerados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resultados.xlsx
+++ b/Resultados.xlsx
@@ -425,34 +425,34 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Atlético Nacional</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>América de Cali</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Deportivo Cali</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>América de Cali</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Atlético Nacional</t>
-        </is>
-      </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Millonarios</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Atlético Bucaramanga</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>Independiente Medellín</t>
@@ -460,62 +460,62 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Águilas Doradas</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Once Caldas</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>Cúcuta Deportivo</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Once Caldas</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Deportes Tolima</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Águilas Doradas</t>
-        </is>
-      </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>Alianza Valledupar</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>Internacional de Bogotá</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Llaneros</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Alianza Valledupar</t>
-        </is>
-      </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Boyacá Chicó</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>Deportivo Pereira</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Boyacá Chicó</t>
-        </is>
-      </c>
       <c r="S1" t="inlineStr">
         <is>
+          <t>Jaguares</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>Fortaleza</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Jaguares</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
@@ -529,28 +529,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>9.411999999999999</v>
+        <v>64.944</v>
       </c>
       <c r="C2" t="n">
-        <v>33.861</v>
+        <v>30.808</v>
       </c>
       <c r="D2" t="n">
-        <v>43.972</v>
+        <v>2.118</v>
       </c>
       <c r="E2" t="n">
-        <v>0.03</v>
+        <v>1.984</v>
       </c>
       <c r="F2" t="n">
-        <v>10.821</v>
+        <v>0.002</v>
       </c>
       <c r="G2" t="n">
-        <v>1.804</v>
+        <v>0.144</v>
       </c>
       <c r="H2" t="n">
-        <v>0.096</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -594,28 +594,28 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>18.824</v>
+        <v>28.219</v>
       </c>
       <c r="C3" t="n">
-        <v>31.92</v>
+        <v>50.53100000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>27.454</v>
+        <v>13.03</v>
       </c>
       <c r="E3" t="n">
-        <v>0.493</v>
+        <v>6.5</v>
       </c>
       <c r="F3" t="n">
-        <v>15.998</v>
+        <v>0.263</v>
       </c>
       <c r="G3" t="n">
-        <v>4.826</v>
+        <v>1.437</v>
       </c>
       <c r="H3" t="n">
-        <v>0.436</v>
+        <v>0.02</v>
       </c>
       <c r="I3" t="n">
-        <v>0.049</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -659,37 +659,37 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>28.843</v>
+        <v>4.909</v>
       </c>
       <c r="C4" t="n">
-        <v>17.832</v>
+        <v>12.714</v>
       </c>
       <c r="D4" t="n">
-        <v>14.869</v>
+        <v>42.701</v>
       </c>
       <c r="E4" t="n">
-        <v>2.746</v>
+        <v>25.453</v>
       </c>
       <c r="F4" t="n">
-        <v>23.268</v>
+        <v>3.745</v>
       </c>
       <c r="G4" t="n">
-        <v>10.723</v>
+        <v>9.782</v>
       </c>
       <c r="H4" t="n">
-        <v>1.459</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>0.21</v>
+        <v>0.004</v>
       </c>
       <c r="J4" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
@@ -724,40 +724,40 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>26.013</v>
+        <v>1.54</v>
       </c>
       <c r="C5" t="n">
-        <v>10.501</v>
+        <v>4.534</v>
       </c>
       <c r="D5" t="n">
-        <v>8.302</v>
+        <v>27.997</v>
       </c>
       <c r="E5" t="n">
-        <v>8.669</v>
+        <v>31.75</v>
       </c>
       <c r="F5" t="n">
-        <v>23.094</v>
+        <v>11.497</v>
       </c>
       <c r="G5" t="n">
-        <v>17.945</v>
+        <v>19.766</v>
       </c>
       <c r="H5" t="n">
-        <v>4.082</v>
+        <v>2.781</v>
       </c>
       <c r="I5" t="n">
-        <v>0.869</v>
+        <v>0.119</v>
       </c>
       <c r="J5" t="n">
-        <v>0.149</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>0.232</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="L5" t="n">
-        <v>0.144</v>
+        <v>0.001</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -789,43 +789,43 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>11.463</v>
+        <v>0.356</v>
       </c>
       <c r="C6" t="n">
-        <v>3.899</v>
+        <v>1.202</v>
       </c>
       <c r="D6" t="n">
-        <v>3.606</v>
+        <v>10.838</v>
       </c>
       <c r="E6" t="n">
-        <v>22.001</v>
+        <v>21.158</v>
       </c>
       <c r="F6" t="n">
-        <v>14.685</v>
+        <v>26.232</v>
       </c>
       <c r="G6" t="n">
-        <v>27.529</v>
+        <v>30.347</v>
       </c>
       <c r="H6" t="n">
-        <v>10.372</v>
+        <v>8.285</v>
       </c>
       <c r="I6" t="n">
-        <v>2.9</v>
+        <v>1.182</v>
       </c>
       <c r="J6" t="n">
-        <v>1.122</v>
+        <v>0.215</v>
       </c>
       <c r="K6" t="n">
-        <v>1.499</v>
+        <v>0.108</v>
       </c>
       <c r="L6" t="n">
-        <v>0.905</v>
+        <v>0.05</v>
       </c>
       <c r="M6" t="n">
-        <v>0.014</v>
+        <v>0.027</v>
       </c>
       <c r="N6" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -854,52 +854,52 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>4.122</v>
+        <v>0.032</v>
       </c>
       <c r="C7" t="n">
-        <v>1.443</v>
+        <v>0.197</v>
       </c>
       <c r="D7" t="n">
-        <v>1.249</v>
+        <v>2.959</v>
       </c>
       <c r="E7" t="n">
-        <v>30.589</v>
+        <v>10.189</v>
       </c>
       <c r="F7" t="n">
-        <v>7.663</v>
+        <v>34.69900000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>19.338</v>
+        <v>24.892</v>
       </c>
       <c r="H7" t="n">
-        <v>17.904</v>
+        <v>18.259</v>
       </c>
       <c r="I7" t="n">
-        <v>6.074</v>
+        <v>5.482</v>
       </c>
       <c r="J7" t="n">
-        <v>4.16</v>
+        <v>1.707</v>
       </c>
       <c r="K7" t="n">
-        <v>4.566</v>
+        <v>0.6629999999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>2.655</v>
+        <v>0.721</v>
       </c>
       <c r="M7" t="n">
-        <v>0.148</v>
+        <v>0.2</v>
       </c>
       <c r="N7" t="n">
-        <v>0.052</v>
+        <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>0.033</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -919,55 +919,55 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>1.108</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0.427</v>
+        <v>0.014</v>
       </c>
       <c r="D8" t="n">
-        <v>0.426</v>
+        <v>0.357</v>
       </c>
       <c r="E8" t="n">
-        <v>20.197</v>
+        <v>2.645</v>
       </c>
       <c r="F8" t="n">
-        <v>3.179</v>
+        <v>18.052</v>
       </c>
       <c r="G8" t="n">
-        <v>10.15</v>
+        <v>10.744</v>
       </c>
       <c r="H8" t="n">
-        <v>23.887</v>
+        <v>32.26</v>
       </c>
       <c r="I8" t="n">
-        <v>10.969</v>
+        <v>19.486</v>
       </c>
       <c r="J8" t="n">
-        <v>11.823</v>
+        <v>9.647</v>
       </c>
       <c r="K8" t="n">
-        <v>9.908999999999999</v>
+        <v>2.812</v>
       </c>
       <c r="L8" t="n">
-        <v>6.754</v>
+        <v>3.215</v>
       </c>
       <c r="M8" t="n">
-        <v>0.637</v>
+        <v>0.672</v>
       </c>
       <c r="N8" t="n">
-        <v>0.334</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>0.105</v>
+        <v>0.012</v>
       </c>
       <c r="P8" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
         <v>0.001</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.094</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
@@ -984,64 +984,64 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.188</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>0.098</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0.094</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>9.610000000000001</v>
+        <v>0.306</v>
       </c>
       <c r="F9" t="n">
-        <v>0.9329999999999999</v>
+        <v>4.278</v>
       </c>
       <c r="G9" t="n">
-        <v>4.567</v>
+        <v>2.23</v>
       </c>
       <c r="H9" t="n">
-        <v>16.968</v>
+        <v>19.237</v>
       </c>
       <c r="I9" t="n">
-        <v>17.278</v>
+        <v>26.104</v>
       </c>
       <c r="J9" t="n">
-        <v>19.9</v>
+        <v>24.012</v>
       </c>
       <c r="K9" t="n">
-        <v>16.182</v>
+        <v>9.827</v>
       </c>
       <c r="L9" t="n">
-        <v>10.258</v>
+        <v>10.048</v>
       </c>
       <c r="M9" t="n">
-        <v>1.711</v>
+        <v>2.035</v>
       </c>
       <c r="N9" t="n">
-        <v>1.235</v>
+        <v>0.8330000000000001</v>
       </c>
       <c r="O9" t="n">
-        <v>0.352</v>
+        <v>0.474</v>
       </c>
       <c r="P9" t="n">
+        <v>0.5890000000000001</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="R9" t="n">
         <v>0.014</v>
       </c>
-      <c r="Q9" t="n">
-        <v>0.611</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0</v>
-      </c>
       <c r="S9" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="T9" t="n">
         <v>0.001</v>
       </c>
-      <c r="T9" t="n">
-        <v>0</v>
-      </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="10">
@@ -1049,64 +1049,64 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.027</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0.016</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.026</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>4.175</v>
+        <v>0.015</v>
       </c>
       <c r="F10" t="n">
-        <v>0.291</v>
+        <v>1.027</v>
       </c>
       <c r="G10" t="n">
-        <v>2.066</v>
+        <v>0.545</v>
       </c>
       <c r="H10" t="n">
-        <v>11.464</v>
+        <v>9.825000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>17.913</v>
+        <v>20.053</v>
       </c>
       <c r="J10" t="n">
-        <v>21.456</v>
+        <v>21.996</v>
       </c>
       <c r="K10" t="n">
-        <v>20.153</v>
+        <v>17.546</v>
       </c>
       <c r="L10" t="n">
-        <v>13.113</v>
+        <v>17.342</v>
       </c>
       <c r="M10" t="n">
-        <v>3.693</v>
+        <v>3.889</v>
       </c>
       <c r="N10" t="n">
-        <v>3.104</v>
+        <v>2.409</v>
       </c>
       <c r="O10" t="n">
-        <v>0.786</v>
+        <v>1.964</v>
       </c>
       <c r="P10" t="n">
-        <v>0.061</v>
+        <v>3.141</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.626</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="R10" t="n">
-        <v>0.016</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="S10" t="n">
-        <v>0.012</v>
+        <v>0.067</v>
       </c>
       <c r="T10" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="U10" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="11">
@@ -1117,61 +1117,61 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>1.286</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0.06</v>
+        <v>0.195</v>
       </c>
       <c r="G11" t="n">
-        <v>0.8049999999999999</v>
+        <v>0.094</v>
       </c>
       <c r="H11" t="n">
-        <v>7.113</v>
+        <v>4.918</v>
       </c>
       <c r="I11" t="n">
-        <v>16.926</v>
+        <v>14.024</v>
       </c>
       <c r="J11" t="n">
-        <v>18.174</v>
+        <v>18.307</v>
       </c>
       <c r="K11" t="n">
-        <v>20.626</v>
+        <v>21.293</v>
       </c>
       <c r="L11" t="n">
-        <v>16.124</v>
+        <v>19.652</v>
       </c>
       <c r="M11" t="n">
-        <v>6.941</v>
+        <v>6.379</v>
       </c>
       <c r="N11" t="n">
-        <v>6.31</v>
+        <v>4.448</v>
       </c>
       <c r="O11" t="n">
-        <v>1.862</v>
+        <v>4.18</v>
       </c>
       <c r="P11" t="n">
-        <v>0.15</v>
+        <v>5.666</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.494</v>
+        <v>0.275</v>
       </c>
       <c r="R11" t="n">
-        <v>0.059</v>
+        <v>0.316</v>
       </c>
       <c r="S11" t="n">
-        <v>0.025</v>
+        <v>0.204</v>
       </c>
       <c r="T11" t="n">
-        <v>0.03</v>
+        <v>0.018</v>
       </c>
       <c r="U11" t="n">
-        <v>0.01</v>
+        <v>0.031</v>
       </c>
     </row>
     <row r="12">
@@ -1188,55 +1188,55 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>0.192</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="G12" t="n">
-        <v>0.201</v>
+        <v>0.019</v>
       </c>
       <c r="H12" t="n">
-        <v>3.844</v>
+        <v>2.326</v>
       </c>
       <c r="I12" t="n">
-        <v>13.388</v>
+        <v>8.061999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>12.248</v>
+        <v>11.793</v>
       </c>
       <c r="K12" t="n">
-        <v>14.075</v>
+        <v>19.79</v>
       </c>
       <c r="L12" t="n">
-        <v>19.151</v>
+        <v>19.8</v>
       </c>
       <c r="M12" t="n">
-        <v>12.527</v>
+        <v>9.747</v>
       </c>
       <c r="N12" t="n">
-        <v>12.139</v>
+        <v>8.444000000000001</v>
       </c>
       <c r="O12" t="n">
-        <v>4.233</v>
+        <v>8.305</v>
       </c>
       <c r="P12" t="n">
-        <v>0.428</v>
+        <v>9.173999999999999</v>
       </c>
       <c r="Q12" t="n">
-        <v>7.045999999999999</v>
+        <v>0.9039999999999999</v>
       </c>
       <c r="R12" t="n">
-        <v>0.251</v>
+        <v>0.8840000000000001</v>
       </c>
       <c r="S12" t="n">
-        <v>0.132</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="T12" t="n">
-        <v>0.107</v>
+        <v>0.036</v>
       </c>
       <c r="U12" t="n">
-        <v>0.031</v>
+        <v>0.141</v>
       </c>
     </row>
     <row r="13">
@@ -1253,55 +1253,55 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0.012</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>0.041</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>1.715</v>
+        <v>0.996</v>
       </c>
       <c r="I13" t="n">
-        <v>8.054</v>
+        <v>3.888</v>
       </c>
       <c r="J13" t="n">
-        <v>6.63</v>
+        <v>6.815</v>
       </c>
       <c r="K13" t="n">
-        <v>7.834000000000001</v>
+        <v>13.545</v>
       </c>
       <c r="L13" t="n">
-        <v>15.219</v>
+        <v>13.384</v>
       </c>
       <c r="M13" t="n">
-        <v>19.333</v>
+        <v>14.887</v>
       </c>
       <c r="N13" t="n">
-        <v>19.069</v>
+        <v>13.002</v>
       </c>
       <c r="O13" t="n">
-        <v>8.119999999999999</v>
+        <v>12.905</v>
       </c>
       <c r="P13" t="n">
-        <v>1.119</v>
+        <v>14.11</v>
       </c>
       <c r="Q13" t="n">
-        <v>11.021</v>
+        <v>2.984</v>
       </c>
       <c r="R13" t="n">
-        <v>0.931</v>
+        <v>1.739</v>
       </c>
       <c r="S13" t="n">
-        <v>0.415</v>
+        <v>1.146</v>
       </c>
       <c r="T13" t="n">
-        <v>0.368</v>
+        <v>0.154</v>
       </c>
       <c r="U13" t="n">
-        <v>0.118</v>
+        <v>0.445</v>
       </c>
     </row>
     <row r="14">
@@ -1324,49 +1324,49 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0.573</v>
+        <v>0.316</v>
       </c>
       <c r="I14" t="n">
-        <v>3.892</v>
+        <v>1.312</v>
       </c>
       <c r="J14" t="n">
-        <v>3.031</v>
+        <v>3.843</v>
       </c>
       <c r="K14" t="n">
-        <v>3.445</v>
+        <v>8.305999999999999</v>
       </c>
       <c r="L14" t="n">
-        <v>9.463000000000001</v>
+        <v>8.504000000000001</v>
       </c>
       <c r="M14" t="n">
-        <v>21.656</v>
+        <v>17.89</v>
       </c>
       <c r="N14" t="n">
-        <v>21.459</v>
+        <v>16.732</v>
       </c>
       <c r="O14" t="n">
-        <v>13.625</v>
+        <v>14.882</v>
       </c>
       <c r="P14" t="n">
-        <v>2.794</v>
+        <v>16.101</v>
       </c>
       <c r="Q14" t="n">
-        <v>15.646</v>
+        <v>5.31</v>
       </c>
       <c r="R14" t="n">
-        <v>2.131</v>
+        <v>3.273</v>
       </c>
       <c r="S14" t="n">
-        <v>0.9480000000000001</v>
+        <v>2.011</v>
       </c>
       <c r="T14" t="n">
-        <v>0.9490000000000001</v>
+        <v>0.464</v>
       </c>
       <c r="U14" t="n">
-        <v>0.383</v>
+        <v>1.056</v>
       </c>
     </row>
     <row r="15">
@@ -1392,46 +1392,46 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>0.08</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>1.23</v>
+        <v>0.265</v>
       </c>
       <c r="J15" t="n">
-        <v>0.991</v>
+        <v>1.405</v>
       </c>
       <c r="K15" t="n">
-        <v>1.143</v>
+        <v>4.324</v>
       </c>
       <c r="L15" t="n">
-        <v>4.383</v>
+        <v>4.867</v>
       </c>
       <c r="M15" t="n">
-        <v>16.415</v>
+        <v>16.34</v>
       </c>
       <c r="N15" t="n">
-        <v>17.475</v>
+        <v>18.688</v>
       </c>
       <c r="O15" t="n">
-        <v>19.388</v>
+        <v>16.724</v>
       </c>
       <c r="P15" t="n">
-        <v>7.628</v>
+        <v>16.563</v>
       </c>
       <c r="Q15" t="n">
-        <v>20.003</v>
+        <v>7.829</v>
       </c>
       <c r="R15" t="n">
-        <v>4.434</v>
+        <v>6.167</v>
       </c>
       <c r="S15" t="n">
-        <v>2.715</v>
+        <v>3.591</v>
       </c>
       <c r="T15" t="n">
-        <v>2.785</v>
+        <v>0.9530000000000001</v>
       </c>
       <c r="U15" t="n">
-        <v>1.33</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="16">
@@ -1457,46 +1457,46 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.001</v>
       </c>
       <c r="I16" t="n">
-        <v>0.223</v>
+        <v>0.017</v>
       </c>
       <c r="J16" t="n">
-        <v>0.27</v>
+        <v>0.233</v>
       </c>
       <c r="K16" t="n">
-        <v>0.266</v>
+        <v>1.479</v>
       </c>
       <c r="L16" t="n">
-        <v>1.415</v>
+        <v>1.875</v>
       </c>
       <c r="M16" t="n">
-        <v>10.054</v>
+        <v>12.939</v>
       </c>
       <c r="N16" t="n">
-        <v>11.1</v>
+        <v>14.289</v>
       </c>
       <c r="O16" t="n">
-        <v>21.83</v>
+        <v>17.599</v>
       </c>
       <c r="P16" t="n">
-        <v>14.961</v>
+        <v>14.902</v>
       </c>
       <c r="Q16" t="n">
-        <v>17.108</v>
+        <v>12.498</v>
       </c>
       <c r="R16" t="n">
-        <v>7.631</v>
+        <v>10.589</v>
       </c>
       <c r="S16" t="n">
-        <v>5.972</v>
+        <v>6.978</v>
       </c>
       <c r="T16" t="n">
-        <v>6.065</v>
+        <v>2.311</v>
       </c>
       <c r="U16" t="n">
-        <v>3.098</v>
+        <v>4.29</v>
       </c>
     </row>
     <row r="17">
@@ -1525,43 +1525,43 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>0.02</v>
+        <v>0.001</v>
       </c>
       <c r="J17" t="n">
-        <v>0.039</v>
+        <v>0.019</v>
       </c>
       <c r="K17" t="n">
-        <v>0.047</v>
+        <v>0.287</v>
       </c>
       <c r="L17" t="n">
-        <v>0.342</v>
+        <v>0.483</v>
       </c>
       <c r="M17" t="n">
-        <v>4.693</v>
+        <v>8.85</v>
       </c>
       <c r="N17" t="n">
-        <v>5.067</v>
+        <v>10.08</v>
       </c>
       <c r="O17" t="n">
-        <v>15.544</v>
+        <v>11.529</v>
       </c>
       <c r="P17" t="n">
-        <v>22.359</v>
+        <v>9.558</v>
       </c>
       <c r="Q17" t="n">
-        <v>10.768</v>
+        <v>17.144</v>
       </c>
       <c r="R17" t="n">
-        <v>12.115</v>
+        <v>17.105</v>
       </c>
       <c r="S17" t="n">
-        <v>11.848</v>
+        <v>11.654</v>
       </c>
       <c r="T17" t="n">
-        <v>10.573</v>
+        <v>5.06</v>
       </c>
       <c r="U17" t="n">
-        <v>6.585000000000001</v>
+        <v>8.23</v>
       </c>
     </row>
     <row r="18">
@@ -1593,40 +1593,40 @@
         <v>0.001</v>
       </c>
       <c r="J18" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="K18" t="n">
-        <v>0.003</v>
+        <v>0.013</v>
       </c>
       <c r="L18" t="n">
-        <v>0.044</v>
+        <v>0.057</v>
       </c>
       <c r="M18" t="n">
-        <v>1.709</v>
+        <v>4.516</v>
       </c>
       <c r="N18" t="n">
-        <v>1.974</v>
+        <v>7.177</v>
       </c>
       <c r="O18" t="n">
-        <v>8.477</v>
+        <v>7.556</v>
       </c>
       <c r="P18" t="n">
-        <v>19.69</v>
+        <v>5.861000000000001</v>
       </c>
       <c r="Q18" t="n">
-        <v>6.463000000000001</v>
+        <v>21.054</v>
       </c>
       <c r="R18" t="n">
-        <v>18.455</v>
+        <v>18.988</v>
       </c>
       <c r="S18" t="n">
-        <v>17.894</v>
+        <v>13.971</v>
       </c>
       <c r="T18" t="n">
-        <v>14.18</v>
+        <v>8.620999999999999</v>
       </c>
       <c r="U18" t="n">
-        <v>11.108</v>
+        <v>12.184</v>
       </c>
     </row>
     <row r="19">
@@ -1664,34 +1664,34 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>0.005</v>
+        <v>0.001</v>
       </c>
       <c r="M19" t="n">
-        <v>0.404</v>
+        <v>1.426</v>
       </c>
       <c r="N19" t="n">
-        <v>0.5950000000000001</v>
+        <v>3.141999999999999</v>
       </c>
       <c r="O19" t="n">
-        <v>4.048999999999999</v>
+        <v>3.213</v>
       </c>
       <c r="P19" t="n">
-        <v>15.442</v>
+        <v>3.165</v>
       </c>
       <c r="Q19" t="n">
-        <v>3.566</v>
+        <v>19.463</v>
       </c>
       <c r="R19" t="n">
-        <v>20.874</v>
+        <v>18.053</v>
       </c>
       <c r="S19" t="n">
-        <v>21.647</v>
+        <v>17.949</v>
       </c>
       <c r="T19" t="n">
-        <v>17.305</v>
+        <v>15.137</v>
       </c>
       <c r="U19" t="n">
-        <v>16.113</v>
+        <v>18.451</v>
       </c>
     </row>
     <row r="20">
@@ -1732,31 +1732,31 @@
         <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>0.065</v>
+        <v>0.19</v>
       </c>
       <c r="N20" t="n">
-        <v>0.075</v>
+        <v>0.641</v>
       </c>
       <c r="O20" t="n">
-        <v>1.386</v>
+        <v>0.617</v>
       </c>
       <c r="P20" t="n">
-        <v>10.804</v>
+        <v>1.02</v>
       </c>
       <c r="Q20" t="n">
-        <v>1.878</v>
+        <v>10.162</v>
       </c>
       <c r="R20" t="n">
-        <v>20.437</v>
+        <v>14.443</v>
       </c>
       <c r="S20" t="n">
-        <v>22.968</v>
+        <v>20.606</v>
       </c>
       <c r="T20" t="n">
-        <v>20.525</v>
+        <v>28.578</v>
       </c>
       <c r="U20" t="n">
-        <v>21.862</v>
+        <v>23.743</v>
       </c>
     </row>
     <row r="21">
@@ -1797,31 +1797,31 @@
         <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>0.012</v>
       </c>
       <c r="N21" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.043</v>
       </c>
       <c r="O21" t="n">
-        <v>0.21</v>
+        <v>0.04</v>
       </c>
       <c r="P21" t="n">
-        <v>4.549</v>
+        <v>0.139</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.672</v>
+        <v>2.286</v>
       </c>
       <c r="R21" t="n">
-        <v>12.666</v>
+        <v>8.340999999999999</v>
       </c>
       <c r="S21" t="n">
-        <v>15.423</v>
+        <v>21.254</v>
       </c>
       <c r="T21" t="n">
-        <v>27.111</v>
+        <v>38.662</v>
       </c>
       <c r="U21" t="n">
-        <v>39.362</v>
+        <v>29.223</v>
       </c>
     </row>
   </sheetData>
@@ -1853,51 +1853,51 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>América de Cali</t>
+          <t>Atlético Nacional</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99.98100000000001</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Deportivo Cali</t>
+          <t>América de Cali</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.973</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Atlético Nacional</t>
+          <t>Deportivo Cali</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>99.97200000000001</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Atlético Bucaramanga</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>99.64100000000002</v>
+        <v>99.98499999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Atlético Bucaramanga</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>96.88200000000001</v>
+        <v>99.34200000000001</v>
       </c>
     </row>
     <row r="7">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>94.33500000000001</v>
+        <v>98.768</v>
       </c>
     </row>
     <row r="8">
@@ -1917,17 +1917,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>75.20400000000001</v>
+        <v>81.53399999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cúcuta Deportivo</t>
+          <t>Águilas Doradas</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>38.353</v>
+        <v>52.377</v>
       </c>
     </row>
     <row r="10">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>37.15900000000001</v>
+        <v>35.58799999999999</v>
       </c>
     </row>
     <row r="11">
@@ -1947,37 +1947,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>32.408</v>
+        <v>14.035</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Águilas Doradas</t>
+          <t>Cúcuta Deportivo</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>20.741</v>
+        <v>13.417</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Internacional de Bogotá</t>
+          <t>Alianza Valledupar</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2.51</v>
+        <v>2.935</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Llaneros</t>
+          <t>Internacional de Bogotá</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.626</v>
+        <v>0.905</v>
       </c>
     </row>
     <row r="15">
@@ -1987,17 +1987,17 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.709</v>
+        <v>0.6000000000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Alianza Valledupar</t>
+          <t>Llaneros</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.49</v>
+        <v>0.486</v>
       </c>
     </row>
     <row r="17">
@@ -2013,31 +2013,31 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Boyacá Chicó</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.001</v>
+        <v>0.006999999999999999</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Boyacá Chicó</t>
+          <t>Jaguares</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Jaguares</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="21">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>